<commit_message>
Just forgot to save!
</commit_message>
<xml_diff>
--- a/Tables.xlsx
+++ b/Tables.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nchaku/Documents/GitHub/pubertybrain/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA6F57F1-411C-594C-8E26-89B79748C104}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A063C0BF-9634-0944-BC9A-5DF77A458D5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2040" yWindow="500" windowWidth="26380" windowHeight="16460" activeTab="1" xr2:uid="{E0F15479-AA73-0644-8B08-3949D67CD8FE}"/>
+    <workbookView xWindow="2040" yWindow="500" windowWidth="26380" windowHeight="16460" activeTab="4" xr2:uid="{E0F15479-AA73-0644-8B08-3949D67CD8FE}"/>
   </bookViews>
   <sheets>
     <sheet name="Descriptive table" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="97">
   <si>
     <t>16.10 (2.98)</t>
   </si>
@@ -376,6 +376,21 @@
       </rPr>
       <t>)</t>
     </r>
+  </si>
+  <si>
+    <t>Model 1</t>
+  </si>
+  <si>
+    <t>Model 2</t>
+  </si>
+  <si>
+    <t>Model 3</t>
+  </si>
+  <si>
+    <t>Model 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Table 2. </t>
   </si>
 </sst>
 </file>
@@ -1695,9 +1710,29 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BBA86F85-A8D4-F648-84C3-730F1A42C846}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="C2" t="s">
+        <v>92</v>
+      </c>
+      <c r="E2" t="s">
+        <v>93</v>
+      </c>
+      <c r="G2" t="s">
+        <v>94</v>
+      </c>
+      <c r="I2" t="s">
+        <v>95</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Ran female cort models again
</commit_message>
<xml_diff>
--- a/Tables.xlsx
+++ b/Tables.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10125"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nchaku/Documents/GitHub/pubertybrain/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nchaku\Documents\GitHub\pubertybrain\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A063C0BF-9634-0944-BC9A-5DF77A458D5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9548B466-316A-40C6-8CA5-F307D8B9796E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2040" yWindow="500" windowWidth="26380" windowHeight="16460" activeTab="4" xr2:uid="{E0F15479-AA73-0644-8B08-3949D67CD8FE}"/>
+    <workbookView xWindow="1725" yWindow="15" windowWidth="28860" windowHeight="15135" activeTab="4" xr2:uid="{E0F15479-AA73-0644-8B08-3949D67CD8FE}"/>
   </bookViews>
   <sheets>
     <sheet name="Descriptive table" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="127">
   <si>
     <t>16.10 (2.98)</t>
   </si>
@@ -387,17 +387,303 @@
     <t>Model 3</t>
   </si>
   <si>
-    <t>Model 4</t>
-  </si>
-  <si>
     <t xml:space="preserve">Table 2. </t>
+  </si>
+  <si>
+    <t>Means</t>
+  </si>
+  <si>
+    <t>Variances</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Timing</t>
+  </si>
+  <si>
+    <t>Latent variables</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Covariances </t>
+  </si>
+  <si>
+    <t>Path coefficients</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Timing      with Tempo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Tempo</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>SE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">p </t>
+  </si>
+  <si>
+    <t xml:space="preserve">   ELA</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>95%</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>CI</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">   Intercept</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="subscript"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>b</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">   Slope</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="subscript"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>b</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">   Intercept</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="subscript"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>b</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> with Slope</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="subscript"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>b</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">   Intercept</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="subscript"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>b</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> with Timing</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">   Intercept</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="subscript"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>b</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> with Tempo</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">   Slope</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="subscript"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>b</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">      with Tempo</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">   Timing on Slope</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="subscript"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>b</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">   ELA    on Intercept</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="subscript"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>b</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">   ELA    on Slope</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="subscript"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>b</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">   WM    on Intercept</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="subscript"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>b</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">   WM    on Slope</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="subscript"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>b</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">   ELA    on Timing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   ELA    on Tempo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   WM    on Tempo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   WM    on Timing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   WM    on ELA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   WM</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -453,13 +739,45 @@
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <vertAlign val="subscript"/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF333333"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="3">
@@ -492,7 +810,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -513,6 +831,34 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -1094,20 +1440,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39987BE7-3659-524A-81AE-D479F97EF698}">
   <dimension ref="A1:F34"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="28.83203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="4" width="20.1640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.83203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28.875" bestFit="1" customWidth="1"/>
+    <col min="2" max="4" width="20.125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="9"/>
       <c r="B2" s="10" t="s">
         <v>75</v>
@@ -1125,7 +1471,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="6"/>
       <c r="B3" s="11" t="s">
         <v>81</v>
@@ -1139,7 +1485,7 @@
       <c r="E3" s="11"/>
       <c r="F3" s="6"/>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>72</v>
       </c>
@@ -1149,7 +1495,7 @@
       <c r="E4" s="2"/>
       <c r="F4" s="1"/>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>73</v>
       </c>
@@ -1169,7 +1515,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>74</v>
       </c>
@@ -1189,7 +1535,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>70</v>
       </c>
@@ -1209,7 +1555,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
         <v>71</v>
       </c>
@@ -1219,7 +1565,7 @@
       <c r="E8" s="12"/>
       <c r="F8" s="1"/>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>73</v>
       </c>
@@ -1239,7 +1585,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>78</v>
       </c>
@@ -1259,7 +1605,7 @@
         <v>0.06</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>79</v>
       </c>
@@ -1279,7 +1625,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>74</v>
       </c>
@@ -1299,7 +1645,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
         <v>80</v>
       </c>
@@ -1309,7 +1655,7 @@
       <c r="E13" s="12"/>
       <c r="F13" s="1"/>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>86</v>
       </c>
@@ -1329,7 +1675,7 @@
         <v>1.74</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>87</v>
       </c>
@@ -1349,7 +1695,7 @@
         <v>1.93</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>88</v>
       </c>
@@ -1369,7 +1715,7 @@
         <v>1.69</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>89</v>
       </c>
@@ -1387,7 +1733,7 @@
       </c>
       <c r="F17" s="1"/>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
         <v>83</v>
       </c>
@@ -1397,7 +1743,7 @@
       <c r="E18" s="12"/>
       <c r="F18" s="1"/>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>73</v>
       </c>
@@ -1417,7 +1763,7 @@
         <v>0.89</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
         <v>78</v>
       </c>
@@ -1437,7 +1783,7 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
         <v>79</v>
       </c>
@@ -1457,7 +1803,7 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
         <v>74</v>
       </c>
@@ -1477,7 +1823,7 @@
         <v>1.27</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="8" t="s">
         <v>84</v>
       </c>
@@ -1487,7 +1833,7 @@
       <c r="E23" s="12"/>
       <c r="F23" s="1"/>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
         <v>73</v>
       </c>
@@ -1507,7 +1853,7 @@
         <v>0.87</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
         <v>78</v>
       </c>
@@ -1527,7 +1873,7 @@
         <v>0.93</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
         <v>79</v>
       </c>
@@ -1547,7 +1893,7 @@
         <v>1.18</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
         <v>74</v>
       </c>
@@ -1567,7 +1913,7 @@
         <v>1.24</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="8" t="s">
         <v>85</v>
       </c>
@@ -1577,7 +1923,7 @@
       <c r="E28" s="12"/>
       <c r="F28" s="1"/>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
         <v>73</v>
       </c>
@@ -1597,7 +1943,7 @@
         <v>0.88</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
         <v>78</v>
       </c>
@@ -1617,7 +1963,7 @@
         <v>0.88</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
         <v>79</v>
       </c>
@@ -1637,7 +1983,7 @@
         <v>1.1299999999999999</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="7" t="s">
         <v>74</v>
       </c>
@@ -1657,7 +2003,7 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="33" spans="1:6" ht="18" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:6" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A33" s="4"/>
       <c r="B33" s="1"/>
       <c r="C33" s="1"/>
@@ -1665,7 +2011,7 @@
       <c r="E33" s="1"/>
       <c r="F33" s="1"/>
     </row>
-    <row r="34" spans="1:6" ht="18" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:6" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A34" s="4"/>
       <c r="B34" s="1"/>
       <c r="C34" s="1"/>
@@ -1681,7 +2027,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A749072B-F938-0F49-BE23-243603B2B3D0}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1691,7 +2037,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45875D41-9C56-AA4E-A18A-2D3A4CE169B3}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1701,7 +2047,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A2A5153E-6E5C-054A-8ACA-5118463B96C5}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1710,29 +2056,1192 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BBA86F85-A8D4-F648-84C3-730F1A42C846}">
-  <dimension ref="A1:I2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:R36"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="19.625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="5.875" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="4.625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="5.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="5.875" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="6.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="4.625" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="5.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="5.875" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="16384" width="11" style="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1" s="14" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
+      <c r="I1" s="14"/>
+      <c r="J1" s="14"/>
+      <c r="K1" s="14"/>
+      <c r="L1" s="14"/>
+      <c r="M1" s="14"/>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A2" s="15"/>
+      <c r="B2" s="16" t="s">
+        <v>84</v>
+      </c>
+      <c r="C2" s="16"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="16"/>
+      <c r="G2" s="16"/>
+      <c r="H2" s="16"/>
+      <c r="I2" s="16"/>
+      <c r="J2" s="16"/>
+      <c r="K2" s="16"/>
+      <c r="L2" s="16"/>
+      <c r="M2" s="16"/>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A3" s="17"/>
+      <c r="B3" s="18" t="s">
+        <v>92</v>
+      </c>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18" t="s">
+        <v>93</v>
+      </c>
+      <c r="G3" s="18"/>
+      <c r="H3" s="18"/>
+      <c r="I3" s="18"/>
+      <c r="J3" s="18" t="s">
+        <v>94</v>
+      </c>
+      <c r="K3" s="18"/>
+      <c r="L3" s="18"/>
+      <c r="M3" s="18"/>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A4" s="19"/>
+      <c r="B4" s="20" t="s">
+        <v>104</v>
+      </c>
+      <c r="C4" s="20" t="s">
+        <v>105</v>
+      </c>
+      <c r="D4" s="20" t="s">
+        <v>106</v>
+      </c>
+      <c r="E4" s="20" t="s">
+        <v>109</v>
+      </c>
+      <c r="F4" s="20" t="s">
+        <v>104</v>
+      </c>
+      <c r="G4" s="20" t="s">
+        <v>105</v>
+      </c>
+      <c r="H4" s="20" t="s">
+        <v>106</v>
+      </c>
+      <c r="I4" s="20" t="s">
+        <v>109</v>
+      </c>
+      <c r="J4" s="20" t="s">
+        <v>104</v>
+      </c>
+      <c r="K4" s="20" t="s">
+        <v>105</v>
+      </c>
+      <c r="L4" s="20" t="s">
+        <v>106</v>
+      </c>
+      <c r="M4" s="20" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A5" s="20" t="s">
+        <v>99</v>
+      </c>
+      <c r="B5" s="19"/>
+      <c r="C5" s="19"/>
+      <c r="D5" s="19"/>
+      <c r="E5" s="19"/>
+      <c r="F5" s="19"/>
+      <c r="G5" s="19"/>
+      <c r="H5" s="19"/>
+      <c r="I5" s="19"/>
+      <c r="J5" s="19"/>
+      <c r="K5" s="19"/>
+      <c r="L5" s="19"/>
+      <c r="M5" s="19"/>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A6" s="19" t="s">
+        <v>110</v>
+      </c>
+      <c r="B6" s="19">
+        <v>576.59</v>
+      </c>
+      <c r="C6" s="19">
+        <v>1.07</v>
+      </c>
+      <c r="D6" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="E6" s="19"/>
+      <c r="F6" s="19">
+        <v>583.54999999999995</v>
+      </c>
+      <c r="G6" s="19">
+        <v>1.51</v>
+      </c>
+      <c r="H6" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="I6" s="19"/>
+      <c r="J6" s="19"/>
+      <c r="K6" s="19"/>
+      <c r="L6" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="M6" s="19"/>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A7" s="19" t="s">
+        <v>111</v>
+      </c>
+      <c r="B7" s="19">
+        <v>-93.95</v>
+      </c>
+      <c r="C7" s="19">
+        <v>4.51</v>
+      </c>
+      <c r="D7" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="E7" s="19"/>
+      <c r="F7" s="19">
+        <v>-94.05</v>
+      </c>
+      <c r="G7" s="19">
+        <v>4.62</v>
+      </c>
+      <c r="H7" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="I7" s="19"/>
+      <c r="J7" s="19"/>
+      <c r="K7" s="19"/>
+      <c r="L7" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="M7" s="19"/>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A8" s="20" t="s">
+        <v>100</v>
+      </c>
+      <c r="B8" s="19"/>
+      <c r="C8" s="19"/>
+      <c r="D8" s="19"/>
+      <c r="E8" s="19"/>
+      <c r="F8" s="19"/>
+      <c r="G8" s="19"/>
+      <c r="H8" s="19"/>
+      <c r="I8" s="19"/>
+      <c r="J8" s="19"/>
+      <c r="K8" s="19"/>
+      <c r="L8" s="19"/>
+      <c r="M8" s="19"/>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A9" s="19" t="s">
+        <v>112</v>
+      </c>
+      <c r="B9" s="19">
+        <v>-143.01</v>
+      </c>
+      <c r="C9" s="19">
+        <v>19.41</v>
+      </c>
+      <c r="D9" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="E9" s="19"/>
+      <c r="F9" s="19">
+        <v>-143.01</v>
+      </c>
+      <c r="G9" s="19">
+        <v>19.260000000000002</v>
+      </c>
+      <c r="H9" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="I9" s="19"/>
+      <c r="J9" s="19">
+        <v>-143.02000000000001</v>
+      </c>
+      <c r="K9" s="19">
+        <v>19.260000000000002</v>
+      </c>
+      <c r="L9" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="M9" s="19"/>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A10" s="19" t="s">
+        <v>113</v>
+      </c>
+      <c r="B10" s="19">
+        <v>6.87</v>
+      </c>
+      <c r="C10" s="19">
+        <v>1.0900000000000001</v>
+      </c>
+      <c r="D10" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="E10" s="19"/>
+      <c r="F10" s="19">
+        <v>5.48</v>
+      </c>
+      <c r="G10" s="19">
+        <v>1.05</v>
+      </c>
+      <c r="H10" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="I10" s="19"/>
+      <c r="J10" s="19">
+        <v>5.48</v>
+      </c>
+      <c r="K10" s="19">
+        <v>1.05</v>
+      </c>
+      <c r="L10" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="M10" s="19"/>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A11" s="22" t="s">
+        <v>114</v>
+      </c>
+      <c r="B11" s="22">
+        <v>1.1499999999999999</v>
+      </c>
+      <c r="C11" s="22">
+        <v>0.16</v>
+      </c>
+      <c r="D11" s="26" t="s">
+        <v>24</v>
+      </c>
+      <c r="E11" s="22"/>
+      <c r="F11" s="22">
+        <v>0.93</v>
+      </c>
+      <c r="G11" s="22">
+        <v>0.15</v>
+      </c>
+      <c r="H11" s="26" t="s">
+        <v>24</v>
+      </c>
+      <c r="I11" s="22"/>
+      <c r="J11" s="22">
+        <v>0.93</v>
+      </c>
+      <c r="K11" s="22">
+        <v>0.15</v>
+      </c>
+      <c r="L11" s="26" t="s">
+        <v>24</v>
+      </c>
+      <c r="M11" s="22"/>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A12" s="19" t="s">
+        <v>115</v>
+      </c>
+      <c r="B12" s="19">
+        <v>-0.08</v>
+      </c>
+      <c r="C12" s="19">
+        <v>0.05</v>
+      </c>
+      <c r="D12" s="21">
+        <v>0.15</v>
+      </c>
+      <c r="E12" s="19"/>
+      <c r="F12" s="19">
+        <v>-0.08</v>
+      </c>
+      <c r="G12" s="19">
+        <v>0.05</v>
+      </c>
+      <c r="H12" s="21">
+        <v>0.15</v>
+      </c>
+      <c r="I12" s="19"/>
+      <c r="J12" s="19">
+        <v>-0.08</v>
+      </c>
+      <c r="K12" s="19">
+        <v>0.05</v>
+      </c>
+      <c r="L12" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="M12" s="19"/>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A13" s="19" t="s">
+        <v>102</v>
+      </c>
+      <c r="B13" s="19">
+        <v>0.05</v>
+      </c>
+      <c r="C13" s="19">
+        <v>4.0000000000000001E-3</v>
+      </c>
+      <c r="D13" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="E13" s="19"/>
+      <c r="F13" s="19">
+        <v>0.05</v>
+      </c>
+      <c r="G13" s="19">
+        <v>3.0000000000000001E-3</v>
+      </c>
+      <c r="H13" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="I13" s="19"/>
+      <c r="J13" s="19">
+        <v>0.05</v>
+      </c>
+      <c r="K13" s="19">
+        <v>3.0000000000000001E-3</v>
+      </c>
+      <c r="L13" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="M13" s="19"/>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A14" s="20" t="s">
+        <v>101</v>
+      </c>
+      <c r="B14" s="19"/>
+      <c r="C14" s="19"/>
+      <c r="D14" s="19"/>
+      <c r="E14" s="19"/>
+      <c r="F14" s="19"/>
+      <c r="G14" s="19"/>
+      <c r="H14" s="19"/>
+      <c r="I14" s="19"/>
+      <c r="J14" s="19"/>
+      <c r="K14" s="19"/>
+      <c r="L14" s="19"/>
+      <c r="M14" s="19"/>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A15" s="19" t="s">
+        <v>116</v>
+      </c>
+      <c r="B15" s="19">
+        <v>3.2</v>
+      </c>
+      <c r="C15" s="19">
+        <v>0.37</v>
+      </c>
+      <c r="D15" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="E15" s="21"/>
+      <c r="F15" s="19">
+        <v>3.21</v>
+      </c>
+      <c r="G15" s="19">
+        <v>0.38</v>
+      </c>
+      <c r="H15" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="I15" s="19"/>
+      <c r="J15" s="19">
+        <v>3.2</v>
+      </c>
+      <c r="K15" s="19">
+        <v>0.38</v>
+      </c>
+      <c r="L15" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="M15" s="19"/>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A16" s="19" t="s">
+        <v>117</v>
+      </c>
+      <c r="B16" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="C16" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="D16" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="E16" s="24" t="s">
+        <v>108</v>
+      </c>
+      <c r="F16" s="19">
+        <v>-3.81</v>
+      </c>
+      <c r="G16" s="19">
+        <v>0.56999999999999995</v>
+      </c>
+      <c r="H16" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="I16" s="19"/>
+      <c r="J16" s="19">
+        <v>-3.82</v>
+      </c>
+      <c r="K16" s="19">
+        <v>0.56999999999999995</v>
+      </c>
+      <c r="L16" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="M16" s="19"/>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A17" s="19" t="s">
+        <v>118</v>
+      </c>
+      <c r="B17" s="23" t="s">
+        <v>108</v>
+      </c>
+      <c r="C17" s="23" t="s">
+        <v>108</v>
+      </c>
+      <c r="D17" s="23" t="s">
+        <v>108</v>
+      </c>
+      <c r="E17" s="24" t="s">
+        <v>108</v>
+      </c>
+      <c r="F17" s="19">
+        <v>0.02</v>
+      </c>
+      <c r="G17" s="19">
+        <v>0.22</v>
+      </c>
+      <c r="H17" s="19">
+        <v>0.94</v>
+      </c>
+      <c r="I17" s="19"/>
+      <c r="J17" s="19">
+        <v>0.01</v>
+      </c>
+      <c r="K17" s="19">
+        <v>0.22</v>
+      </c>
+      <c r="L17" s="21">
+        <v>0.65</v>
+      </c>
+      <c r="M17" s="19"/>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A18" s="19" t="s">
+        <v>121</v>
+      </c>
+      <c r="B18" s="23" t="s">
+        <v>108</v>
+      </c>
+      <c r="C18" s="23" t="s">
+        <v>108</v>
+      </c>
+      <c r="D18" s="23" t="s">
+        <v>108</v>
+      </c>
+      <c r="E18" s="24" t="s">
+        <v>108</v>
+      </c>
+      <c r="F18" s="19">
+        <v>-0.11</v>
+      </c>
+      <c r="G18" s="19">
+        <v>0.01</v>
+      </c>
+      <c r="H18" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="I18" s="19"/>
+      <c r="J18" s="23">
+        <v>-0.11</v>
+      </c>
+      <c r="K18" s="23">
+        <v>0.01</v>
+      </c>
+      <c r="L18" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="M18" s="19"/>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A19" s="19" t="s">
+        <v>122</v>
+      </c>
+      <c r="B19" s="23" t="s">
+        <v>108</v>
+      </c>
+      <c r="C19" s="23" t="s">
+        <v>108</v>
+      </c>
+      <c r="D19" s="23" t="s">
+        <v>108</v>
+      </c>
+      <c r="E19" s="24" t="s">
+        <v>108</v>
+      </c>
+      <c r="F19" s="19">
+        <v>-0.02</v>
+      </c>
+      <c r="G19" s="19">
+        <v>2E-3</v>
+      </c>
+      <c r="H19" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="I19" s="19"/>
+      <c r="J19" s="19">
+        <v>-0.02</v>
+      </c>
+      <c r="K19" s="19">
+        <v>2E-3</v>
+      </c>
+      <c r="L19" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="M19" s="19"/>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A20" s="19" t="s">
+        <v>119</v>
+      </c>
+      <c r="B20" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="C20" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="D20" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="E20" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="F20" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="G20" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="H20" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="I20" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="J20" s="19">
+        <v>0.01</v>
+      </c>
+      <c r="K20" s="19">
+        <v>2E-3</v>
+      </c>
+      <c r="L20" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="M20" s="19"/>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A21" s="19" t="s">
+        <v>120</v>
+      </c>
+      <c r="B21" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="C21" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="D21" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="E21" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="F21" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="G21" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="H21" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="I21" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="J21" s="19">
+        <v>-2E-3</v>
+      </c>
+      <c r="K21" s="19">
+        <v>0.01</v>
+      </c>
+      <c r="L21" s="21">
+        <v>0.84</v>
+      </c>
+      <c r="M21" s="19"/>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A22" s="19" t="s">
+        <v>124</v>
+      </c>
+      <c r="B22" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="C22" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="D22" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="E22" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="F22" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="G22" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="H22" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="I22" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="J22" s="19">
+        <v>0.11</v>
+      </c>
+      <c r="K22" s="19">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="L22" s="21">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="M22" s="19"/>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A23" s="19" t="s">
+        <v>123</v>
+      </c>
+      <c r="B23" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="C23" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="D23" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="E23" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="F23" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="G23" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="H23" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="I23" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="J23" s="19">
+        <v>1.84</v>
+      </c>
+      <c r="K23" s="19">
+        <v>0.41</v>
+      </c>
+      <c r="L23" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="M23" s="19"/>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A24" s="19" t="s">
+        <v>125</v>
+      </c>
+      <c r="B24" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="C24" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="D24" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="E24" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="F24" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="G24" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="H24" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="I24" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="J24" s="19">
+        <v>-0.17</v>
+      </c>
+      <c r="K24" s="19">
+        <v>0.04</v>
+      </c>
+      <c r="L24" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="M24" s="19"/>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A25" s="20" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="C2" t="s">
-        <v>92</v>
-      </c>
-      <c r="E2" t="s">
-        <v>93</v>
-      </c>
-      <c r="G2" t="s">
-        <v>94</v>
-      </c>
-      <c r="I2" t="s">
-        <v>95</v>
-      </c>
+      <c r="B25" s="19"/>
+      <c r="C25" s="19"/>
+      <c r="D25" s="19"/>
+      <c r="E25" s="19"/>
+      <c r="F25" s="19"/>
+      <c r="G25" s="19"/>
+      <c r="H25" s="19"/>
+      <c r="I25" s="19"/>
+      <c r="J25" s="19"/>
+      <c r="K25" s="19"/>
+      <c r="L25" s="19"/>
+      <c r="M25" s="19"/>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A26" s="19" t="s">
+        <v>98</v>
+      </c>
+      <c r="B26" s="23">
+        <v>12.02</v>
+      </c>
+      <c r="C26" s="23">
+        <v>0.02</v>
+      </c>
+      <c r="D26" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="E26" s="19"/>
+      <c r="F26" s="19">
+        <v>12.23</v>
+      </c>
+      <c r="G26" s="19">
+        <v>0.04</v>
+      </c>
+      <c r="H26" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="I26" s="19"/>
+      <c r="J26" s="19">
+        <v>12.23</v>
+      </c>
+      <c r="K26" s="19">
+        <v>0.04</v>
+      </c>
+      <c r="L26" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="M26" s="19"/>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A27" s="19" t="s">
+        <v>103</v>
+      </c>
+      <c r="B27" s="19">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="C27" s="19">
+        <v>3.0000000000000001E-3</v>
+      </c>
+      <c r="D27" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="E27" s="19"/>
+      <c r="F27" s="19">
+        <v>0.59</v>
+      </c>
+      <c r="G27" s="19">
+        <v>0.01</v>
+      </c>
+      <c r="H27" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="I27" s="19"/>
+      <c r="J27" s="19">
+        <v>0.59</v>
+      </c>
+      <c r="K27" s="19">
+        <v>0.01</v>
+      </c>
+      <c r="L27" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="M27" s="19"/>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A28" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="B28" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="C28" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="D28" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="E28" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="F28" s="24">
+        <v>1.83</v>
+      </c>
+      <c r="G28" s="24">
+        <v>0.04</v>
+      </c>
+      <c r="H28" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="I28" s="19"/>
+      <c r="J28" s="19">
+        <v>1.83</v>
+      </c>
+      <c r="K28" s="19">
+        <v>0.04</v>
+      </c>
+      <c r="L28" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="M28" s="19"/>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A29" s="19" t="s">
+        <v>126</v>
+      </c>
+      <c r="B29" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="C29" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="D29" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="E29" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="F29" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="G29" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="H29" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="I29" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="J29" s="19">
+        <v>10.97</v>
+      </c>
+      <c r="K29" s="19">
+        <v>1.21</v>
+      </c>
+      <c r="L29" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="M29" s="19"/>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A30" s="20" t="s">
+        <v>97</v>
+      </c>
+      <c r="B30" s="19"/>
+      <c r="C30" s="19"/>
+      <c r="D30" s="19"/>
+      <c r="E30" s="19"/>
+      <c r="F30" s="19"/>
+      <c r="G30" s="19"/>
+      <c r="H30" s="19"/>
+      <c r="I30" s="23"/>
+      <c r="J30" s="23"/>
+      <c r="K30" s="23"/>
+      <c r="L30" s="23"/>
+      <c r="M30" s="23"/>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A31" s="19" t="s">
+        <v>110</v>
+      </c>
+      <c r="B31" s="19">
+        <v>2247.4699999999998</v>
+      </c>
+      <c r="C31" s="19">
+        <v>76.02</v>
+      </c>
+      <c r="D31" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="E31" s="23"/>
+      <c r="F31" s="23">
+        <v>2200.12</v>
+      </c>
+      <c r="G31" s="23">
+        <v>14.08</v>
+      </c>
+      <c r="H31" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="I31" s="23"/>
+      <c r="J31" s="23">
+        <v>2199.7800000000002</v>
+      </c>
+      <c r="K31" s="23">
+        <v>74.569999999999993</v>
+      </c>
+      <c r="L31" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="M31" s="23"/>
+    </row>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A32" s="19" t="s">
+        <v>111</v>
+      </c>
+      <c r="B32" s="27">
+        <v>93.62</v>
+      </c>
+      <c r="C32" s="27">
+        <v>14.08</v>
+      </c>
+      <c r="D32" s="28" t="s">
+        <v>24</v>
+      </c>
+      <c r="E32" s="23"/>
+      <c r="F32" s="23">
+        <v>93.66</v>
+      </c>
+      <c r="G32" s="23">
+        <v>14.08</v>
+      </c>
+      <c r="H32" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="I32" s="23"/>
+      <c r="J32" s="23">
+        <v>93.71</v>
+      </c>
+      <c r="K32" s="23">
+        <v>14.08</v>
+      </c>
+      <c r="L32" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="M32" s="23"/>
+    </row>
+    <row r="33" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A33" s="19" t="s">
+        <v>98</v>
+      </c>
+      <c r="B33" s="19">
+        <v>1.2</v>
+      </c>
+      <c r="C33" s="19">
+        <v>0.04</v>
+      </c>
+      <c r="D33" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="E33" s="23"/>
+      <c r="F33" s="23">
+        <v>1.1599999999999999</v>
+      </c>
+      <c r="G33" s="23">
+        <v>0.03</v>
+      </c>
+      <c r="H33" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="I33" s="23"/>
+      <c r="J33" s="23">
+        <v>1.1599999999999999</v>
+      </c>
+      <c r="K33" s="23">
+        <v>0.03</v>
+      </c>
+      <c r="L33" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="M33" s="23"/>
+    </row>
+    <row r="34" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A34" s="19" t="s">
+        <v>103</v>
+      </c>
+      <c r="B34" s="19">
+        <v>0.02</v>
+      </c>
+      <c r="C34" s="19">
+        <v>1E-3</v>
+      </c>
+      <c r="D34" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="E34" s="23"/>
+      <c r="F34" s="23">
+        <v>0.02</v>
+      </c>
+      <c r="G34" s="23">
+        <v>1E-3</v>
+      </c>
+      <c r="H34" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="I34" s="24"/>
+      <c r="J34" s="24">
+        <v>0.02</v>
+      </c>
+      <c r="K34" s="24">
+        <v>1E-3</v>
+      </c>
+      <c r="L34" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="M34" s="24"/>
+    </row>
+    <row r="35" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A35" s="24" t="s">
+        <v>107</v>
+      </c>
+      <c r="B35" s="24" t="s">
+        <v>108</v>
+      </c>
+      <c r="C35" s="24" t="s">
+        <v>108</v>
+      </c>
+      <c r="D35" s="24" t="s">
+        <v>108</v>
+      </c>
+      <c r="E35" s="24" t="s">
+        <v>108</v>
+      </c>
+      <c r="F35" s="23">
+        <v>3.26</v>
+      </c>
+      <c r="G35" s="23">
+        <v>0.13</v>
+      </c>
+      <c r="H35" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="I35" s="24"/>
+      <c r="J35" s="23">
+        <v>3.26</v>
+      </c>
+      <c r="K35" s="23">
+        <v>0.13</v>
+      </c>
+      <c r="L35" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="M35" s="24"/>
+    </row>
+    <row r="36" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A36" s="17" t="s">
+        <v>126</v>
+      </c>
+      <c r="B36" s="25" t="s">
+        <v>108</v>
+      </c>
+      <c r="C36" s="25" t="s">
+        <v>108</v>
+      </c>
+      <c r="D36" s="25" t="s">
+        <v>108</v>
+      </c>
+      <c r="E36" s="25" t="s">
+        <v>108</v>
+      </c>
+      <c r="F36" s="25" t="s">
+        <v>108</v>
+      </c>
+      <c r="G36" s="25" t="s">
+        <v>108</v>
+      </c>
+      <c r="H36" s="25" t="s">
+        <v>108</v>
+      </c>
+      <c r="I36" s="25" t="s">
+        <v>108</v>
+      </c>
+      <c r="J36" s="25">
+        <v>7.64</v>
+      </c>
+      <c r="K36" s="25">
+        <v>0.3</v>
+      </c>
+      <c r="L36" s="29" t="s">
+        <v>24</v>
+      </c>
+      <c r="M36" s="6"/>
+      <c r="N36" s="6"/>
+      <c r="O36" s="6"/>
+      <c r="P36" s="6"/>
+      <c r="Q36" s="6"/>
+      <c r="R36" s="6"/>
     </row>
   </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="B2:M2"/>
+    <mergeCell ref="F3:I3"/>
+    <mergeCell ref="J3:M3"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Updated more of the tabl
</commit_message>
<xml_diff>
--- a/Tables.xlsx
+++ b/Tables.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10208"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nchaku\Documents\GitHub\pubertybrain\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nchaku/Documents/GitHub/pubertybrain/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3049B952-14D7-4B8A-9371-24029F884A01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DF775CB-4F28-1742-9002-F940C250CB44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{E0F15479-AA73-0644-8B08-3949D67CD8FE}"/>
+    <workbookView xWindow="13360" yWindow="500" windowWidth="15440" windowHeight="16400" firstSheet="1" activeTab="5" xr2:uid="{E0F15479-AA73-0644-8B08-3949D67CD8FE}"/>
   </bookViews>
   <sheets>
     <sheet name="Descriptive table" sheetId="1" r:id="rId1"/>
@@ -18,8 +18,9 @@
     <sheet name="Fig1 (Pub)" sheetId="3" r:id="rId3"/>
     <sheet name="Fig2 (Brain)" sheetId="4" r:id="rId4"/>
     <sheet name="CortModels" sheetId="6" r:id="rId5"/>
-    <sheet name="Youth report PDS" sheetId="9" r:id="rId6"/>
-    <sheet name="Indirect effects" sheetId="7" r:id="rId7"/>
+    <sheet name="SubCortModel" sheetId="10" r:id="rId6"/>
+    <sheet name="Youth report PDS" sheetId="9" r:id="rId7"/>
+    <sheet name="Indirect effects" sheetId="7" r:id="rId8"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="487" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="723" uniqueCount="137">
   <si>
     <t>16.10 (2.98)</t>
   </si>
@@ -884,7 +885,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -925,34 +926,31 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="11" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1533,20 +1531,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39987BE7-3659-524A-81AE-D479F97EF698}">
   <dimension ref="A1:F29"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="28.875" bestFit="1" customWidth="1"/>
-    <col min="2" max="4" width="20.125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28.83203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="4" width="20.1640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="9"/>
       <c r="B2" s="10" t="s">
         <v>63</v>
@@ -1564,7 +1562,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="6"/>
       <c r="B3" s="11" t="s">
         <v>69</v>
@@ -1578,7 +1576,7 @@
       <c r="E3" s="11"/>
       <c r="F3" s="6"/>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
         <v>60</v>
       </c>
@@ -1588,7 +1586,7 @@
       <c r="E4" s="2"/>
       <c r="F4" s="1"/>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
         <v>61</v>
       </c>
@@ -1608,7 +1606,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
         <v>62</v>
       </c>
@@ -1628,7 +1626,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
         <v>58</v>
       </c>
@@ -1648,7 +1646,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="8" t="s">
         <v>59</v>
       </c>
@@ -1658,7 +1656,7 @@
       <c r="E8" s="12"/>
       <c r="F8" s="1"/>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="3" t="s">
         <v>61</v>
       </c>
@@ -1678,7 +1676,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="3" t="s">
         <v>66</v>
       </c>
@@ -1698,7 +1696,7 @@
         <v>0.06</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="3" t="s">
         <v>67</v>
       </c>
@@ -1718,7 +1716,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="3" t="s">
         <v>62</v>
       </c>
@@ -1738,7 +1736,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" s="8" t="s">
         <v>68</v>
       </c>
@@ -1748,7 +1746,7 @@
       <c r="E13" s="12"/>
       <c r="F13" s="1"/>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" s="3" t="s">
         <v>73</v>
       </c>
@@ -1768,7 +1766,7 @@
         <v>1.74</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
         <v>74</v>
       </c>
@@ -1788,7 +1786,7 @@
         <v>1.93</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" s="3" t="s">
         <v>75</v>
       </c>
@@ -1808,7 +1806,7 @@
         <v>1.69</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" s="3" t="s">
         <v>76</v>
       </c>
@@ -1826,7 +1824,7 @@
       </c>
       <c r="F17" s="19"/>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" s="8" t="s">
         <v>71</v>
       </c>
@@ -1836,7 +1834,7 @@
       <c r="E18" s="12"/>
       <c r="F18" s="1"/>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" s="3" t="s">
         <v>61</v>
       </c>
@@ -1856,7 +1854,7 @@
         <v>0.87</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" s="3" t="s">
         <v>66</v>
       </c>
@@ -1876,7 +1874,7 @@
         <v>0.93</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" s="3" t="s">
         <v>67</v>
       </c>
@@ -1896,7 +1894,7 @@
         <v>1.18</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" s="3" t="s">
         <v>62</v>
       </c>
@@ -1916,7 +1914,7 @@
         <v>1.24</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23" s="8" t="s">
         <v>72</v>
       </c>
@@ -1926,7 +1924,7 @@
       <c r="E23" s="12"/>
       <c r="F23" s="1"/>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" s="3" t="s">
         <v>61</v>
       </c>
@@ -1946,7 +1944,7 @@
         <v>0.88</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" s="3" t="s">
         <v>66</v>
       </c>
@@ -1966,7 +1964,7 @@
         <v>0.88</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" s="3" t="s">
         <v>67</v>
       </c>
@@ -1986,7 +1984,7 @@
         <v>1.1299999999999999</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27" s="7" t="s">
         <v>62</v>
       </c>
@@ -2006,7 +2004,7 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="28" spans="1:6" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" ht="18" x14ac:dyDescent="0.2">
       <c r="A28" s="4"/>
       <c r="B28" s="1"/>
       <c r="C28" s="1"/>
@@ -2014,7 +2012,7 @@
       <c r="E28" s="1"/>
       <c r="F28" s="1"/>
     </row>
-    <row r="29" spans="1:6" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" ht="18" x14ac:dyDescent="0.2">
       <c r="A29" s="4"/>
       <c r="B29" s="1"/>
       <c r="C29" s="1"/>
@@ -2030,9 +2028,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A749072B-F938-0F49-BE23-243603B2B3D0}">
   <dimension ref="M2"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="2" spans="13:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="13:13" x14ac:dyDescent="0.2">
       <c r="M2" t="s">
         <v>113</v>
       </c>
@@ -2046,7 +2044,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45875D41-9C56-AA4E-A18A-2D3A4CE169B3}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2056,7 +2054,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A2A5153E-6E5C-054A-8ACA-5118463B96C5}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2066,241 +2064,240 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BBA86F85-A8D4-F648-84C3-730F1A42C846}">
   <dimension ref="A1:AM34"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.125" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="6.5" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="1.125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="1.1640625" style="1" customWidth="1"/>
     <col min="8" max="8" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="5.125" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="5.625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="5.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="5.6640625" style="1" customWidth="1"/>
     <col min="11" max="11" width="6.5" style="1" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="1.125" style="1" customWidth="1"/>
+    <col min="13" max="13" width="1.1640625" style="1" customWidth="1"/>
     <col min="14" max="14" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="5.125" style="1" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="5.625" style="1" customWidth="1"/>
+    <col min="15" max="15" width="5.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="5.6640625" style="1" customWidth="1"/>
     <col min="17" max="17" width="6.5" style="1" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="0.875" style="1" customWidth="1"/>
+    <col min="19" max="19" width="0.83203125" style="1" customWidth="1"/>
     <col min="20" max="20" width="8.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="5.125" style="1" bestFit="1" customWidth="1"/>
-    <col min="22" max="23" width="5.625" style="1" customWidth="1"/>
-    <col min="24" max="24" width="6.25" style="1" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="1" style="33" customWidth="1"/>
+    <col min="21" max="21" width="5.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="22" max="23" width="5.6640625" style="1" customWidth="1"/>
+    <col min="24" max="24" width="6.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="1" style="1" customWidth="1"/>
     <col min="26" max="26" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="5.125" style="1" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="5.625" style="1" customWidth="1"/>
+    <col min="27" max="27" width="5.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="5.6640625" style="1" customWidth="1"/>
     <col min="29" max="30" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="1.125" style="33" customWidth="1"/>
+    <col min="31" max="31" width="1.1640625" style="1" customWidth="1"/>
     <col min="32" max="32" width="7" style="1" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="5.125" style="1" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="5.625" style="1" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="5.625" style="1" customWidth="1"/>
-    <col min="36" max="36" width="6.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="5.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="5.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="5.6640625" style="1" customWidth="1"/>
+    <col min="36" max="36" width="6.1640625" style="1" bestFit="1" customWidth="1"/>
     <col min="37" max="16384" width="11" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A2" s="14"/>
-      <c r="B2" s="35" t="s">
+      <c r="B2" s="32" t="s">
         <v>114</v>
       </c>
-      <c r="C2" s="35"/>
-      <c r="D2" s="35"/>
-      <c r="E2" s="35"/>
-      <c r="F2" s="35"/>
-      <c r="G2" s="35"/>
-      <c r="H2" s="35"/>
-      <c r="I2" s="35"/>
-      <c r="J2" s="35"/>
-      <c r="K2" s="35"/>
-      <c r="L2" s="35"/>
-      <c r="M2" s="35"/>
-      <c r="N2" s="35"/>
-      <c r="O2" s="35"/>
-      <c r="P2" s="35"/>
-      <c r="Q2" s="35"/>
-      <c r="R2" s="35"/>
+      <c r="C2" s="32"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
+      <c r="F2" s="32"/>
+      <c r="G2" s="32"/>
+      <c r="H2" s="32"/>
+      <c r="I2" s="32"/>
+      <c r="J2" s="32"/>
+      <c r="K2" s="32"/>
+      <c r="L2" s="32"/>
+      <c r="M2" s="32"/>
+      <c r="N2" s="32"/>
+      <c r="O2" s="32"/>
+      <c r="P2" s="32"/>
+      <c r="Q2" s="32"/>
+      <c r="R2" s="32"/>
       <c r="S2" s="9"/>
-      <c r="T2" s="35" t="s">
+      <c r="T2" s="32" t="s">
         <v>115</v>
       </c>
-      <c r="U2" s="35"/>
-      <c r="V2" s="35"/>
-      <c r="W2" s="35"/>
-      <c r="X2" s="35"/>
-      <c r="Y2" s="35"/>
-      <c r="Z2" s="35"/>
-      <c r="AA2" s="35"/>
-      <c r="AB2" s="35"/>
-      <c r="AC2" s="35"/>
-      <c r="AD2" s="35"/>
-      <c r="AE2" s="35"/>
-      <c r="AF2" s="35"/>
-      <c r="AG2" s="35"/>
-      <c r="AH2" s="35"/>
-      <c r="AI2" s="35"/>
-      <c r="AJ2" s="35"/>
-    </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A3" s="31"/>
-      <c r="B3" s="35" t="s">
+      <c r="U2" s="32"/>
+      <c r="V2" s="32"/>
+      <c r="W2" s="32"/>
+      <c r="X2" s="32"/>
+      <c r="Y2" s="32"/>
+      <c r="Z2" s="32"/>
+      <c r="AA2" s="32"/>
+      <c r="AB2" s="32"/>
+      <c r="AC2" s="32"/>
+      <c r="AD2" s="32"/>
+      <c r="AE2" s="32"/>
+      <c r="AF2" s="32"/>
+      <c r="AG2" s="32"/>
+      <c r="AH2" s="32"/>
+      <c r="AI2" s="32"/>
+      <c r="AJ2" s="32"/>
+    </row>
+    <row r="3" spans="1:36" x14ac:dyDescent="0.2">
+      <c r="A3" s="16"/>
+      <c r="B3" s="32" t="s">
         <v>79</v>
       </c>
-      <c r="C3" s="35"/>
-      <c r="D3" s="35"/>
-      <c r="E3" s="35"/>
-      <c r="F3" s="35"/>
-      <c r="G3" s="37"/>
-      <c r="H3" s="35" t="s">
+      <c r="C3" s="32"/>
+      <c r="D3" s="32"/>
+      <c r="E3" s="32"/>
+      <c r="F3" s="32"/>
+      <c r="G3" s="28"/>
+      <c r="H3" s="32" t="s">
         <v>80</v>
       </c>
-      <c r="I3" s="35"/>
-      <c r="J3" s="35"/>
-      <c r="K3" s="35"/>
-      <c r="L3" s="35"/>
-      <c r="M3" s="37"/>
-      <c r="N3" s="35" t="s">
+      <c r="I3" s="32"/>
+      <c r="J3" s="32"/>
+      <c r="K3" s="32"/>
+      <c r="L3" s="32"/>
+      <c r="M3" s="28"/>
+      <c r="N3" s="32" t="s">
         <v>81</v>
       </c>
-      <c r="O3" s="35"/>
-      <c r="P3" s="35"/>
-      <c r="Q3" s="35"/>
-      <c r="R3" s="35"/>
-      <c r="S3" s="33"/>
-      <c r="T3" s="32" t="s">
+      <c r="O3" s="32"/>
+      <c r="P3" s="32"/>
+      <c r="Q3" s="32"/>
+      <c r="R3" s="32"/>
+      <c r="T3" s="33" t="s">
         <v>79</v>
       </c>
-      <c r="U3" s="32"/>
-      <c r="V3" s="32"/>
-      <c r="W3" s="32"/>
-      <c r="X3" s="32"/>
-      <c r="Y3" s="37"/>
-      <c r="Z3" s="35" t="s">
+      <c r="U3" s="33"/>
+      <c r="V3" s="33"/>
+      <c r="W3" s="33"/>
+      <c r="X3" s="33"/>
+      <c r="Y3" s="28"/>
+      <c r="Z3" s="32" t="s">
         <v>80</v>
       </c>
-      <c r="AA3" s="35"/>
-      <c r="AB3" s="35"/>
-      <c r="AC3" s="35"/>
-      <c r="AD3" s="35"/>
-      <c r="AE3" s="37"/>
-      <c r="AF3" s="35" t="s">
+      <c r="AA3" s="32"/>
+      <c r="AB3" s="32"/>
+      <c r="AC3" s="32"/>
+      <c r="AD3" s="32"/>
+      <c r="AE3" s="28"/>
+      <c r="AF3" s="32" t="s">
         <v>81</v>
       </c>
-      <c r="AG3" s="35"/>
-      <c r="AH3" s="35"/>
-      <c r="AI3" s="35"/>
-      <c r="AJ3" s="35"/>
-    </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AG3" s="32"/>
+      <c r="AH3" s="32"/>
+      <c r="AI3" s="32"/>
+      <c r="AJ3" s="32"/>
+    </row>
+    <row r="4" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A4" s="15"/>
-      <c r="B4" s="36" t="s">
+      <c r="B4" s="29" t="s">
         <v>90</v>
       </c>
-      <c r="C4" s="36" t="s">
+      <c r="C4" s="29" t="s">
         <v>91</v>
       </c>
-      <c r="D4" s="36" t="s">
+      <c r="D4" s="29" t="s">
         <v>92</v>
       </c>
-      <c r="E4" s="36" t="s">
+      <c r="E4" s="29" t="s">
         <v>135</v>
       </c>
-      <c r="F4" s="36" t="s">
+      <c r="F4" s="29" t="s">
         <v>136</v>
       </c>
-      <c r="G4" s="36"/>
-      <c r="H4" s="36" t="s">
+      <c r="G4" s="29"/>
+      <c r="H4" s="29" t="s">
         <v>90</v>
       </c>
-      <c r="I4" s="36" t="s">
+      <c r="I4" s="29" t="s">
         <v>91</v>
       </c>
-      <c r="J4" s="36" t="s">
+      <c r="J4" s="29" t="s">
         <v>92</v>
       </c>
-      <c r="K4" s="36" t="s">
+      <c r="K4" s="29" t="s">
         <v>135</v>
       </c>
-      <c r="L4" s="36" t="s">
+      <c r="L4" s="29" t="s">
         <v>136</v>
       </c>
-      <c r="M4" s="36"/>
-      <c r="N4" s="36" t="s">
+      <c r="M4" s="29"/>
+      <c r="N4" s="29" t="s">
         <v>90</v>
       </c>
-      <c r="O4" s="36" t="s">
+      <c r="O4" s="29" t="s">
         <v>91</v>
       </c>
-      <c r="P4" s="36" t="s">
+      <c r="P4" s="29" t="s">
         <v>92</v>
       </c>
-      <c r="Q4" s="36" t="s">
+      <c r="Q4" s="29" t="s">
         <v>135</v>
       </c>
-      <c r="R4" s="36" t="s">
+      <c r="R4" s="29" t="s">
         <v>136</v>
       </c>
       <c r="S4" s="6"/>
-      <c r="T4" s="36" t="s">
+      <c r="T4" s="29" t="s">
         <v>90</v>
       </c>
-      <c r="U4" s="36" t="s">
+      <c r="U4" s="29" t="s">
         <v>91</v>
       </c>
-      <c r="V4" s="36" t="s">
+      <c r="V4" s="29" t="s">
         <v>92</v>
       </c>
-      <c r="W4" s="36" t="s">
+      <c r="W4" s="29" t="s">
         <v>135</v>
       </c>
-      <c r="X4" s="36" t="s">
+      <c r="X4" s="29" t="s">
         <v>136</v>
       </c>
-      <c r="Y4" s="34"/>
-      <c r="Z4" s="36" t="s">
+      <c r="Y4" s="17"/>
+      <c r="Z4" s="29" t="s">
         <v>90</v>
       </c>
-      <c r="AA4" s="36" t="s">
+      <c r="AA4" s="29" t="s">
         <v>91</v>
       </c>
-      <c r="AB4" s="36" t="s">
+      <c r="AB4" s="29" t="s">
         <v>92</v>
       </c>
-      <c r="AC4" s="36" t="s">
+      <c r="AC4" s="29" t="s">
         <v>135</v>
       </c>
-      <c r="AD4" s="36" t="s">
+      <c r="AD4" s="29" t="s">
         <v>136</v>
       </c>
-      <c r="AE4" s="34"/>
-      <c r="AF4" s="36" t="s">
+      <c r="AE4" s="17"/>
+      <c r="AF4" s="29" t="s">
         <v>90</v>
       </c>
-      <c r="AG4" s="36" t="s">
+      <c r="AG4" s="29" t="s">
         <v>91</v>
       </c>
-      <c r="AH4" s="36" t="s">
+      <c r="AH4" s="29" t="s">
         <v>92</v>
       </c>
-      <c r="AI4" s="36" t="s">
+      <c r="AI4" s="29" t="s">
         <v>135</v>
       </c>
-      <c r="AJ4" s="36" t="s">
+      <c r="AJ4" s="29" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A5" s="17" t="s">
         <v>85</v>
       </c>
@@ -2326,20 +2323,20 @@
       <c r="V5" s="16"/>
       <c r="W5" s="16"/>
       <c r="X5" s="16"/>
-      <c r="Y5" s="31"/>
+      <c r="Y5" s="16"/>
       <c r="Z5" s="16"/>
       <c r="AA5" s="16"/>
       <c r="AB5" s="16"/>
       <c r="AC5" s="16"/>
       <c r="AD5" s="16"/>
-      <c r="AE5" s="31"/>
+      <c r="AE5" s="16"/>
       <c r="AF5" s="16"/>
       <c r="AG5" s="16"/>
       <c r="AH5" s="16"/>
       <c r="AI5" s="16"/>
       <c r="AJ5" s="16"/>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A6" s="16" t="s">
         <v>96</v>
       </c>
@@ -2405,7 +2402,7 @@
       <c r="X6" s="16">
         <v>12.095000000000001</v>
       </c>
-      <c r="Y6" s="31"/>
+      <c r="Y6" s="16"/>
       <c r="Z6" s="16">
         <v>11.930999999999999</v>
       </c>
@@ -2421,7 +2418,7 @@
       <c r="AD6" s="16">
         <v>12.236000000000001</v>
       </c>
-      <c r="AE6" s="31"/>
+      <c r="AE6" s="16"/>
       <c r="AF6" s="16">
         <v>11.930999999999999</v>
       </c>
@@ -2438,7 +2435,7 @@
         <v>12.236000000000001</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A7" s="16" t="s">
         <v>97</v>
       </c>
@@ -2504,7 +2501,7 @@
       <c r="X7" s="16">
         <v>-7.7430000000000003</v>
       </c>
-      <c r="Y7" s="31"/>
+      <c r="Y7" s="16"/>
       <c r="Z7" s="16">
         <v>-8.8079999999999998</v>
       </c>
@@ -2520,7 +2517,7 @@
       <c r="AD7" s="16">
         <v>-7.7619999999999996</v>
       </c>
-      <c r="AE7" s="31"/>
+      <c r="AE7" s="16"/>
       <c r="AF7" s="16">
         <v>-8.8030000000000008</v>
       </c>
@@ -2537,7 +2534,7 @@
         <v>-7.7560000000000002</v>
       </c>
     </row>
-    <row r="8" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A8" s="16"/>
       <c r="B8" s="16"/>
       <c r="C8" s="16"/>
@@ -2551,8 +2548,8 @@
       <c r="K8" s="18"/>
       <c r="L8" s="16"/>
       <c r="M8" s="16"/>
-      <c r="N8" s="29"/>
-      <c r="O8" s="29"/>
+      <c r="N8" s="16"/>
+      <c r="O8" s="16"/>
       <c r="P8" s="18"/>
       <c r="Q8" s="18"/>
       <c r="R8" s="16"/>
@@ -2561,20 +2558,20 @@
       <c r="V8" s="18"/>
       <c r="W8" s="18"/>
       <c r="X8" s="21"/>
-      <c r="Y8" s="39"/>
+      <c r="Y8" s="21"/>
       <c r="Z8" s="16"/>
       <c r="AA8" s="16"/>
       <c r="AB8" s="18"/>
       <c r="AC8" s="18"/>
       <c r="AD8" s="16"/>
-      <c r="AE8" s="31"/>
+      <c r="AE8" s="16"/>
       <c r="AF8" s="16"/>
       <c r="AG8" s="16"/>
       <c r="AH8" s="18"/>
       <c r="AI8" s="18"/>
       <c r="AJ8" s="16"/>
     </row>
-    <row r="9" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A9" s="17" t="s">
         <v>86</v>
       </c>
@@ -2600,20 +2597,20 @@
       <c r="V9" s="16"/>
       <c r="W9" s="16"/>
       <c r="X9" s="21"/>
-      <c r="Y9" s="39"/>
+      <c r="Y9" s="21"/>
       <c r="Z9" s="16"/>
       <c r="AA9" s="16"/>
       <c r="AB9" s="16"/>
       <c r="AC9" s="16"/>
       <c r="AD9" s="16"/>
-      <c r="AE9" s="31"/>
+      <c r="AE9" s="16"/>
       <c r="AF9" s="16"/>
       <c r="AG9" s="16"/>
       <c r="AH9" s="16"/>
       <c r="AI9" s="16"/>
       <c r="AJ9" s="16"/>
     </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A10" s="16" t="s">
         <v>98</v>
       </c>
@@ -2679,7 +2676,7 @@
       <c r="X10" s="16">
         <v>-0.24</v>
       </c>
-      <c r="Y10" s="31"/>
+      <c r="Y10" s="16"/>
       <c r="Z10" s="16">
         <v>-0.30599999999999999</v>
       </c>
@@ -2695,7 +2692,7 @@
       <c r="AD10" s="16">
         <v>-0.24099999999999999</v>
       </c>
-      <c r="AE10" s="31"/>
+      <c r="AE10" s="16"/>
       <c r="AF10" s="16">
         <v>-0.30599999999999999</v>
       </c>
@@ -2712,7 +2709,7 @@
         <v>-0.24</v>
       </c>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A11" s="16" t="s">
         <v>99</v>
       </c>
@@ -2778,7 +2775,7 @@
       <c r="X11" s="16">
         <v>0.09</v>
       </c>
-      <c r="Y11" s="31"/>
+      <c r="Y11" s="16"/>
       <c r="Z11" s="16">
         <v>5.6000000000000001E-2</v>
       </c>
@@ -2794,7 +2791,7 @@
       <c r="AD11" s="16">
         <v>0.09</v>
       </c>
-      <c r="AE11" s="31"/>
+      <c r="AE11" s="16"/>
       <c r="AF11" s="16">
         <v>5.6000000000000001E-2</v>
       </c>
@@ -2811,7 +2808,7 @@
         <v>0.09</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A12" s="16" t="s">
         <v>100</v>
       </c>
@@ -2877,7 +2874,7 @@
       <c r="X12" s="16">
         <v>0.16900000000000001</v>
       </c>
-      <c r="Y12" s="31"/>
+      <c r="Y12" s="16"/>
       <c r="Z12" s="16">
         <v>0.114</v>
       </c>
@@ -2893,7 +2890,7 @@
       <c r="AD12" s="16">
         <v>0.14799999999999999</v>
       </c>
-      <c r="AE12" s="31"/>
+      <c r="AE12" s="16"/>
       <c r="AF12" s="16">
         <v>0.115</v>
       </c>
@@ -2910,7 +2907,7 @@
         <v>0.14899999999999999</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A13" s="16" t="s">
         <v>101</v>
       </c>
@@ -2976,7 +2973,7 @@
       <c r="X13" s="16">
         <v>3.1E-2</v>
       </c>
-      <c r="Y13" s="31"/>
+      <c r="Y13" s="16"/>
       <c r="Z13" s="16">
         <v>-2.8000000000000001E-2</v>
       </c>
@@ -2992,7 +2989,7 @@
       <c r="AD13" s="16">
         <v>3.5000000000000003E-2</v>
       </c>
-      <c r="AE13" s="31"/>
+      <c r="AE13" s="16"/>
       <c r="AF13" s="16">
         <v>-2.8000000000000001E-2</v>
       </c>
@@ -3009,7 +3006,7 @@
         <v>3.5999999999999997E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A14" s="16" t="s">
         <v>88</v>
       </c>
@@ -3075,7 +3072,7 @@
       <c r="X14" s="16">
         <v>0.28399999999999997</v>
       </c>
-      <c r="Y14" s="31"/>
+      <c r="Y14" s="16"/>
       <c r="Z14" s="16">
         <v>0.252</v>
       </c>
@@ -3091,7 +3088,7 @@
       <c r="AD14" s="16">
         <v>0.28699999999999998</v>
       </c>
-      <c r="AE14" s="31"/>
+      <c r="AE14" s="16"/>
       <c r="AF14" s="16">
         <v>0.252</v>
       </c>
@@ -3108,7 +3105,7 @@
         <v>0.28799999999999998</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A15" s="16"/>
       <c r="B15" s="16"/>
       <c r="C15" s="16"/>
@@ -3132,20 +3129,20 @@
       <c r="V15" s="18"/>
       <c r="W15" s="18"/>
       <c r="X15" s="21"/>
-      <c r="Y15" s="39"/>
+      <c r="Y15" s="21"/>
       <c r="Z15" s="16"/>
       <c r="AA15" s="16"/>
       <c r="AB15" s="18"/>
       <c r="AC15" s="18"/>
       <c r="AD15" s="16"/>
-      <c r="AE15" s="31"/>
+      <c r="AE15" s="16"/>
       <c r="AF15" s="16"/>
       <c r="AG15" s="16"/>
       <c r="AH15" s="18"/>
       <c r="AI15" s="18"/>
       <c r="AJ15" s="16"/>
     </row>
-    <row r="16" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A16" s="17" t="s">
         <v>87</v>
       </c>
@@ -3171,20 +3168,20 @@
       <c r="V16" s="16"/>
       <c r="W16" s="16"/>
       <c r="X16" s="21"/>
-      <c r="Y16" s="39"/>
+      <c r="Y16" s="21"/>
       <c r="Z16" s="16"/>
       <c r="AA16" s="16"/>
       <c r="AB16" s="16"/>
       <c r="AC16" s="16"/>
       <c r="AD16" s="16"/>
-      <c r="AE16" s="31"/>
+      <c r="AE16" s="16"/>
       <c r="AF16" s="16"/>
       <c r="AG16" s="16"/>
       <c r="AH16" s="16"/>
       <c r="AI16" s="16"/>
       <c r="AJ16" s="16"/>
     </row>
-    <row r="17" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A17" s="16" t="s">
         <v>102</v>
       </c>
@@ -3250,7 +3247,7 @@
       <c r="X17" s="16">
         <v>0.443</v>
       </c>
-      <c r="Y17" s="31"/>
+      <c r="Y17" s="16"/>
       <c r="Z17" s="16">
         <v>0.38300000000000001</v>
       </c>
@@ -3266,7 +3263,7 @@
       <c r="AD17" s="16">
         <v>0.443</v>
       </c>
-      <c r="AE17" s="31"/>
+      <c r="AE17" s="16"/>
       <c r="AF17" s="16">
         <v>0.38300000000000001</v>
       </c>
@@ -3283,7 +3280,7 @@
         <v>0.443</v>
       </c>
     </row>
-    <row r="18" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A18" s="16" t="s">
         <v>103</v>
       </c>
@@ -3349,7 +3346,7 @@
       <c r="X18" s="21" t="s">
         <v>94</v>
       </c>
-      <c r="Y18" s="39"/>
+      <c r="Y18" s="21"/>
       <c r="Z18" s="16">
         <v>-0.13900000000000001</v>
       </c>
@@ -3365,7 +3362,7 @@
       <c r="AD18" s="16">
         <v>-0.104</v>
       </c>
-      <c r="AE18" s="31"/>
+      <c r="AE18" s="16"/>
       <c r="AF18" s="16">
         <v>-0.13900000000000001</v>
       </c>
@@ -3382,7 +3379,7 @@
         <v>-0.10299999999999999</v>
       </c>
     </row>
-    <row r="19" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A19" s="16" t="s">
         <v>104</v>
       </c>
@@ -3448,7 +3445,7 @@
       <c r="X19" s="21" t="s">
         <v>94</v>
       </c>
-      <c r="Y19" s="39"/>
+      <c r="Y19" s="21"/>
       <c r="Z19" s="16">
         <v>2.5000000000000001E-2</v>
       </c>
@@ -3464,7 +3461,7 @@
       <c r="AD19" s="16">
         <v>9.1999999999999998E-2</v>
       </c>
-      <c r="AE19" s="31"/>
+      <c r="AE19" s="16"/>
       <c r="AF19" s="16">
         <v>2.4E-2</v>
       </c>
@@ -3477,11 +3474,11 @@
       <c r="AI19" s="16">
         <v>-4.2999999999999997E-2</v>
       </c>
-      <c r="AJ19" s="40">
+      <c r="AJ19" s="30">
         <v>9.0999999999999998E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A20" s="16" t="s">
         <v>107</v>
       </c>
@@ -3547,7 +3544,7 @@
       <c r="X20" s="21" t="s">
         <v>94</v>
       </c>
-      <c r="Y20" s="39"/>
+      <c r="Y20" s="21"/>
       <c r="Z20" s="16">
         <v>-0.17</v>
       </c>
@@ -3563,7 +3560,7 @@
       <c r="AD20" s="16">
         <v>3.2000000000000001E-2</v>
       </c>
-      <c r="AE20" s="31"/>
+      <c r="AE20" s="16"/>
       <c r="AF20" s="16">
         <v>-3.0000000000000001E-3</v>
       </c>
@@ -3580,7 +3577,7 @@
         <v>3.1E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A21" s="16" t="s">
         <v>108</v>
       </c>
@@ -3646,7 +3643,7 @@
       <c r="X21" s="21" t="s">
         <v>94</v>
       </c>
-      <c r="Y21" s="39"/>
+      <c r="Y21" s="21"/>
       <c r="Z21" s="16">
         <v>-3.0000000000000001E-3</v>
       </c>
@@ -3662,7 +3659,7 @@
       <c r="AD21" s="16">
         <v>-0.13600000000000001</v>
       </c>
-      <c r="AE21" s="31"/>
+      <c r="AE21" s="16"/>
       <c r="AF21" s="16">
         <v>-0.17100000000000001</v>
       </c>
@@ -3679,7 +3676,7 @@
         <v>-0.13600000000000001</v>
       </c>
     </row>
-    <row r="22" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A22" s="16" t="s">
         <v>105</v>
       </c>
@@ -3745,7 +3742,7 @@
       <c r="X22" s="21" t="s">
         <v>94</v>
       </c>
-      <c r="Y22" s="39"/>
+      <c r="Y22" s="21"/>
       <c r="Z22" s="16" t="s">
         <v>94</v>
       </c>
@@ -3759,7 +3756,7 @@
       <c r="AD22" s="16" t="s">
         <v>94</v>
       </c>
-      <c r="AE22" s="31"/>
+      <c r="AE22" s="16"/>
       <c r="AF22" s="16">
         <v>0.11700000000000001</v>
       </c>
@@ -3776,7 +3773,7 @@
         <v>0.156</v>
       </c>
     </row>
-    <row r="23" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A23" s="16" t="s">
         <v>106</v>
       </c>
@@ -3842,7 +3839,7 @@
       <c r="X23" s="21" t="s">
         <v>94</v>
       </c>
-      <c r="Y23" s="39"/>
+      <c r="Y23" s="21"/>
       <c r="Z23" s="16" t="s">
         <v>94</v>
       </c>
@@ -3856,7 +3853,7 @@
       <c r="AD23" s="16" t="s">
         <v>94</v>
       </c>
-      <c r="AE23" s="31"/>
+      <c r="AE23" s="16"/>
       <c r="AF23" s="16">
         <v>-8.8999999999999996E-2</v>
       </c>
@@ -3873,7 +3870,7 @@
         <v>-1.6E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A24" s="16" t="s">
         <v>110</v>
       </c>
@@ -3939,7 +3936,7 @@
       <c r="X24" s="21" t="s">
         <v>94</v>
       </c>
-      <c r="Y24" s="39"/>
+      <c r="Y24" s="21"/>
       <c r="Z24" s="16" t="s">
         <v>94</v>
       </c>
@@ -3953,7 +3950,7 @@
       <c r="AD24" s="16" t="s">
         <v>94</v>
       </c>
-      <c r="AE24" s="31"/>
+      <c r="AE24" s="16"/>
       <c r="AF24" s="16">
         <v>6.8000000000000005E-2</v>
       </c>
@@ -3970,7 +3967,7 @@
         <v>0.112</v>
       </c>
     </row>
-    <row r="25" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A25" s="16" t="s">
         <v>109</v>
       </c>
@@ -4036,7 +4033,7 @@
       <c r="X25" s="21" t="s">
         <v>94</v>
       </c>
-      <c r="Y25" s="39"/>
+      <c r="Y25" s="21"/>
       <c r="Z25" s="16" t="s">
         <v>94</v>
       </c>
@@ -4050,7 +4047,7 @@
       <c r="AD25" s="16" t="s">
         <v>94</v>
       </c>
-      <c r="AE25" s="31"/>
+      <c r="AE25" s="16"/>
       <c r="AF25" s="16">
         <v>0.125</v>
       </c>
@@ -4067,7 +4064,7 @@
         <v>0.16</v>
       </c>
     </row>
-    <row r="26" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A26" s="16" t="s">
         <v>111</v>
       </c>
@@ -4133,7 +4130,7 @@
       <c r="X26" s="21" t="s">
         <v>94</v>
       </c>
-      <c r="Y26" s="39"/>
+      <c r="Y26" s="21"/>
       <c r="Z26" s="16" t="s">
         <v>94</v>
       </c>
@@ -4147,7 +4144,7 @@
       <c r="AD26" s="16" t="s">
         <v>94</v>
       </c>
-      <c r="AE26" s="31"/>
+      <c r="AE26" s="16"/>
       <c r="AF26" s="16">
         <v>-8.3000000000000004E-2</v>
       </c>
@@ -4164,7 +4161,7 @@
         <v>-4.9000000000000002E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A27" s="16"/>
       <c r="B27" s="16"/>
       <c r="C27" s="16"/>
@@ -4188,20 +4185,20 @@
       <c r="V27" s="16"/>
       <c r="W27" s="16"/>
       <c r="X27" s="21"/>
-      <c r="Y27" s="39"/>
+      <c r="Y27" s="21"/>
       <c r="Z27" s="16"/>
       <c r="AA27" s="16"/>
       <c r="AB27" s="16"/>
       <c r="AC27" s="16"/>
       <c r="AD27" s="16"/>
-      <c r="AE27" s="31"/>
+      <c r="AE27" s="16"/>
       <c r="AF27" s="16"/>
       <c r="AG27" s="16"/>
       <c r="AH27" s="18"/>
       <c r="AI27" s="18"/>
       <c r="AJ27" s="16"/>
     </row>
-    <row r="28" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A28" s="17" t="s">
         <v>82</v>
       </c>
@@ -4227,20 +4224,20 @@
       <c r="V28" s="16"/>
       <c r="W28" s="16"/>
       <c r="X28" s="21"/>
-      <c r="Y28" s="39"/>
+      <c r="Y28" s="21"/>
       <c r="Z28" s="16"/>
       <c r="AA28" s="16"/>
       <c r="AB28" s="16"/>
       <c r="AC28" s="16"/>
       <c r="AD28" s="16"/>
-      <c r="AE28" s="31"/>
+      <c r="AE28" s="16"/>
       <c r="AF28" s="16"/>
       <c r="AG28" s="16"/>
       <c r="AH28" s="16"/>
       <c r="AI28" s="16"/>
       <c r="AJ28" s="16"/>
     </row>
-    <row r="29" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A29" s="16" t="s">
         <v>84</v>
       </c>
@@ -4306,7 +4303,7 @@
       <c r="X29" s="16">
         <v>14.16</v>
       </c>
-      <c r="Y29" s="31"/>
+      <c r="Y29" s="16"/>
       <c r="Z29" s="16">
         <v>13.832000000000001</v>
       </c>
@@ -4322,7 +4319,7 @@
       <c r="AD29" s="16">
         <v>14.164999999999999</v>
       </c>
-      <c r="AE29" s="31"/>
+      <c r="AE29" s="16"/>
       <c r="AF29" s="16">
         <v>13.832000000000001</v>
       </c>
@@ -4339,7 +4336,7 @@
         <v>14.164999999999999</v>
       </c>
     </row>
-    <row r="30" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A30" s="16" t="s">
         <v>89</v>
       </c>
@@ -4405,7 +4402,7 @@
       <c r="X30" s="16">
         <v>3.992</v>
       </c>
-      <c r="Y30" s="31"/>
+      <c r="Y30" s="16"/>
       <c r="Z30" s="16">
         <v>4.0620000000000003</v>
       </c>
@@ -4421,7 +4418,7 @@
       <c r="AD30" s="16">
         <v>4.1669999999999998</v>
       </c>
-      <c r="AE30" s="31"/>
+      <c r="AE30" s="16"/>
       <c r="AF30" s="16">
         <v>4.0609999999999999</v>
       </c>
@@ -4438,7 +4435,7 @@
         <v>4.1660000000000004</v>
       </c>
     </row>
-    <row r="31" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A31" s="16" t="s">
         <v>93</v>
       </c>
@@ -4504,7 +4501,7 @@
       <c r="X31" s="21" t="s">
         <v>94</v>
       </c>
-      <c r="Y31" s="39"/>
+      <c r="Y31" s="21"/>
       <c r="Z31" s="16">
         <v>1.026</v>
       </c>
@@ -4520,7 +4517,7 @@
       <c r="AD31" s="16">
         <v>1.0549999999999999</v>
       </c>
-      <c r="AE31" s="31"/>
+      <c r="AE31" s="16"/>
       <c r="AF31" s="16">
         <v>1.0269999999999999</v>
       </c>
@@ -4537,7 +4534,7 @@
         <v>1.0549999999999999</v>
       </c>
     </row>
-    <row r="32" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A32" s="16" t="s">
         <v>112</v>
       </c>
@@ -4556,7 +4553,7 @@
       <c r="F32" s="21" t="s">
         <v>94</v>
       </c>
-      <c r="G32" s="39"/>
+      <c r="G32" s="21"/>
       <c r="H32" s="16" t="s">
         <v>94</v>
       </c>
@@ -4570,7 +4567,7 @@
       <c r="L32" s="16" t="s">
         <v>94</v>
       </c>
-      <c r="M32" s="31"/>
+      <c r="M32" s="16"/>
       <c r="N32" s="16">
         <v>3.8239999999999998</v>
       </c>
@@ -4586,7 +4583,6 @@
       <c r="R32" s="16">
         <v>4.5410000000000004</v>
       </c>
-      <c r="S32" s="33"/>
       <c r="T32" s="16" t="s">
         <v>94</v>
       </c>
@@ -4602,7 +4598,7 @@
       <c r="X32" s="21" t="s">
         <v>94</v>
       </c>
-      <c r="Y32" s="39"/>
+      <c r="Y32" s="21"/>
       <c r="Z32" s="16" t="s">
         <v>94</v>
       </c>
@@ -4618,7 +4614,7 @@
       <c r="AD32" s="21" t="s">
         <v>94</v>
       </c>
-      <c r="AE32" s="31"/>
+      <c r="AE32" s="16"/>
       <c r="AF32" s="16">
         <v>3.387</v>
       </c>
@@ -4634,9 +4630,8 @@
       <c r="AJ32" s="16">
         <v>4.202</v>
       </c>
-      <c r="AK32" s="33"/>
-    </row>
-    <row r="33" spans="1:39" x14ac:dyDescent="0.25">
+    </row>
+    <row r="33" spans="1:39" x14ac:dyDescent="0.2">
       <c r="A33" s="20" t="s">
         <v>117</v>
       </c>
@@ -4645,108 +4640,1935 @@
       <c r="D33" s="14"/>
       <c r="E33" s="14"/>
       <c r="F33" s="14"/>
-      <c r="G33" s="31"/>
+      <c r="G33" s="16"/>
       <c r="H33" s="14"/>
       <c r="I33" s="14"/>
       <c r="J33" s="14"/>
       <c r="K33" s="14"/>
       <c r="L33" s="14"/>
-      <c r="M33" s="31"/>
+      <c r="M33" s="16"/>
       <c r="N33" s="14"/>
       <c r="O33" s="14"/>
       <c r="P33" s="14"/>
       <c r="Q33" s="14"/>
       <c r="R33" s="14"/>
-      <c r="S33" s="31"/>
+      <c r="S33" s="16"/>
       <c r="T33" s="14"/>
       <c r="U33" s="14"/>
       <c r="V33" s="14"/>
       <c r="W33" s="14"/>
       <c r="X33" s="14"/>
-      <c r="Y33" s="31"/>
+      <c r="Y33" s="16"/>
       <c r="Z33" s="14"/>
       <c r="AA33" s="14"/>
       <c r="AB33" s="14"/>
       <c r="AC33" s="14"/>
       <c r="AD33" s="14"/>
-      <c r="AE33" s="31"/>
+      <c r="AE33" s="16"/>
       <c r="AF33" s="14"/>
       <c r="AG33" s="14"/>
       <c r="AH33" s="14"/>
       <c r="AI33" s="14"/>
       <c r="AJ33" s="14"/>
-      <c r="AK33" s="31"/>
+      <c r="AK33" s="16"/>
       <c r="AL33" s="16"/>
       <c r="AM33" s="16"/>
     </row>
-    <row r="34" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:39" x14ac:dyDescent="0.2">
       <c r="A34" s="15" t="s">
         <v>118</v>
       </c>
-      <c r="B34" s="30">
+      <c r="B34" s="31">
         <v>74058.118000000002</v>
       </c>
-      <c r="C34" s="30"/>
-      <c r="D34" s="30"/>
-      <c r="E34" s="30"/>
-      <c r="F34" s="30"/>
-      <c r="G34" s="38"/>
-      <c r="H34" s="30">
+      <c r="C34" s="31"/>
+      <c r="D34" s="31"/>
+      <c r="E34" s="31"/>
+      <c r="F34" s="31"/>
+      <c r="G34" s="27"/>
+      <c r="H34" s="31">
         <v>83016.937999999995</v>
       </c>
-      <c r="I34" s="30"/>
-      <c r="J34" s="30"/>
-      <c r="K34" s="30"/>
-      <c r="L34" s="30"/>
-      <c r="M34" s="38"/>
-      <c r="N34" s="30">
+      <c r="I34" s="31"/>
+      <c r="J34" s="31"/>
+      <c r="K34" s="31"/>
+      <c r="L34" s="31"/>
+      <c r="M34" s="27"/>
+      <c r="N34" s="31">
         <v>94345.274999999994</v>
       </c>
-      <c r="O34" s="30"/>
-      <c r="P34" s="30"/>
-      <c r="Q34" s="30"/>
-      <c r="R34" s="30"/>
+      <c r="O34" s="31"/>
+      <c r="P34" s="31"/>
+      <c r="Q34" s="31"/>
+      <c r="R34" s="31"/>
       <c r="S34" s="15"/>
-      <c r="T34" s="30">
+      <c r="T34" s="31">
         <v>83167.763000000006</v>
       </c>
-      <c r="U34" s="30"/>
-      <c r="V34" s="30"/>
-      <c r="W34" s="30"/>
-      <c r="X34" s="30"/>
-      <c r="Y34" s="38"/>
-      <c r="Z34" s="30">
+      <c r="U34" s="31"/>
+      <c r="V34" s="31"/>
+      <c r="W34" s="31"/>
+      <c r="X34" s="31"/>
+      <c r="Y34" s="27"/>
+      <c r="Z34" s="31">
         <v>93083.505999999994</v>
       </c>
-      <c r="AA34" s="30"/>
-      <c r="AB34" s="30"/>
-      <c r="AC34" s="30"/>
-      <c r="AD34" s="30"/>
-      <c r="AE34" s="38"/>
-      <c r="AF34" s="30">
+      <c r="AA34" s="31"/>
+      <c r="AB34" s="31"/>
+      <c r="AC34" s="31"/>
+      <c r="AD34" s="31"/>
+      <c r="AE34" s="27"/>
+      <c r="AF34" s="31">
         <v>105770.462</v>
       </c>
-      <c r="AG34" s="30"/>
-      <c r="AH34" s="30"/>
-      <c r="AI34" s="30"/>
-      <c r="AJ34" s="30"/>
-      <c r="AK34" s="41"/>
+      <c r="AG34" s="31"/>
+      <c r="AH34" s="31"/>
+      <c r="AI34" s="31"/>
+      <c r="AJ34" s="31"/>
+      <c r="AK34" s="16"/>
       <c r="AL34" s="16"/>
       <c r="AM34" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B2:R2"/>
+    <mergeCell ref="H3:L3"/>
+    <mergeCell ref="N3:R3"/>
+    <mergeCell ref="T2:AJ2"/>
+    <mergeCell ref="T3:X3"/>
+    <mergeCell ref="Z3:AD3"/>
+    <mergeCell ref="AF3:AJ3"/>
     <mergeCell ref="AF34:AJ34"/>
     <mergeCell ref="B34:F34"/>
     <mergeCell ref="H34:L34"/>
     <mergeCell ref="T34:X34"/>
     <mergeCell ref="N34:R34"/>
     <mergeCell ref="Z34:AD34"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CD5CF7F-81D6-D24D-8228-B4C578C35D65}">
+  <dimension ref="A1:AM34"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="19.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="1.1640625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="6" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="5.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="5.6640625" style="1" customWidth="1"/>
+    <col min="11" max="11" width="6.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="6" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="1.1640625" style="1" customWidth="1"/>
+    <col min="14" max="14" width="6" style="1" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="5.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="5.6640625" style="1" customWidth="1"/>
+    <col min="17" max="17" width="6.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="6" style="1" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="0.83203125" style="1" customWidth="1"/>
+    <col min="20" max="20" width="6.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="5.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="6.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="5.6640625" style="1" customWidth="1"/>
+    <col min="24" max="24" width="6.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="1" style="1" customWidth="1"/>
+    <col min="26" max="26" width="6" style="1" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="5.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="5.6640625" style="1" customWidth="1"/>
+    <col min="29" max="30" width="6" style="1" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="1.1640625" style="1" customWidth="1"/>
+    <col min="32" max="32" width="7" style="1" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="5.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="5.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="5.6640625" style="1" customWidth="1"/>
+    <col min="36" max="36" width="6.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="37" max="16384" width="11" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:36" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="2" spans="1:36" x14ac:dyDescent="0.2">
+      <c r="A2" s="14"/>
+      <c r="B2" s="32" t="s">
+        <v>114</v>
+      </c>
+      <c r="C2" s="32"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
+      <c r="F2" s="32"/>
+      <c r="G2" s="32"/>
+      <c r="H2" s="32"/>
+      <c r="I2" s="32"/>
+      <c r="J2" s="32"/>
+      <c r="K2" s="32"/>
+      <c r="L2" s="32"/>
+      <c r="M2" s="32"/>
+      <c r="N2" s="32"/>
+      <c r="O2" s="32"/>
+      <c r="P2" s="32"/>
+      <c r="Q2" s="32"/>
+      <c r="R2" s="32"/>
+      <c r="S2" s="9"/>
+      <c r="T2" s="32" t="s">
+        <v>115</v>
+      </c>
+      <c r="U2" s="32"/>
+      <c r="V2" s="32"/>
+      <c r="W2" s="32"/>
+      <c r="X2" s="32"/>
+      <c r="Y2" s="32"/>
+      <c r="Z2" s="32"/>
+      <c r="AA2" s="32"/>
+      <c r="AB2" s="32"/>
+      <c r="AC2" s="32"/>
+      <c r="AD2" s="32"/>
+      <c r="AE2" s="32"/>
+      <c r="AF2" s="32"/>
+      <c r="AG2" s="32"/>
+      <c r="AH2" s="32"/>
+      <c r="AI2" s="32"/>
+      <c r="AJ2" s="32"/>
+    </row>
+    <row r="3" spans="1:36" x14ac:dyDescent="0.2">
+      <c r="A3" s="16"/>
+      <c r="B3" s="32" t="s">
+        <v>79</v>
+      </c>
+      <c r="C3" s="32"/>
+      <c r="D3" s="32"/>
+      <c r="E3" s="32"/>
+      <c r="F3" s="32"/>
+      <c r="G3" s="28"/>
+      <c r="H3" s="32" t="s">
+        <v>80</v>
+      </c>
+      <c r="I3" s="32"/>
+      <c r="J3" s="32"/>
+      <c r="K3" s="32"/>
+      <c r="L3" s="32"/>
+      <c r="M3" s="28"/>
+      <c r="N3" s="32" t="s">
+        <v>81</v>
+      </c>
+      <c r="O3" s="32"/>
+      <c r="P3" s="32"/>
+      <c r="Q3" s="32"/>
+      <c r="R3" s="32"/>
+      <c r="T3" s="33" t="s">
+        <v>79</v>
+      </c>
+      <c r="U3" s="33"/>
+      <c r="V3" s="33"/>
+      <c r="W3" s="33"/>
+      <c r="X3" s="33"/>
+      <c r="Y3" s="28"/>
+      <c r="Z3" s="32" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA3" s="32"/>
+      <c r="AB3" s="32"/>
+      <c r="AC3" s="32"/>
+      <c r="AD3" s="32"/>
+      <c r="AE3" s="28"/>
+      <c r="AF3" s="32" t="s">
+        <v>81</v>
+      </c>
+      <c r="AG3" s="32"/>
+      <c r="AH3" s="32"/>
+      <c r="AI3" s="32"/>
+      <c r="AJ3" s="32"/>
+    </row>
+    <row r="4" spans="1:36" x14ac:dyDescent="0.2">
+      <c r="A4" s="15"/>
+      <c r="B4" s="29" t="s">
+        <v>90</v>
+      </c>
+      <c r="C4" s="29" t="s">
+        <v>91</v>
+      </c>
+      <c r="D4" s="29" t="s">
+        <v>92</v>
+      </c>
+      <c r="E4" s="29" t="s">
+        <v>135</v>
+      </c>
+      <c r="F4" s="29" t="s">
+        <v>136</v>
+      </c>
+      <c r="G4" s="29"/>
+      <c r="H4" s="29" t="s">
+        <v>90</v>
+      </c>
+      <c r="I4" s="29" t="s">
+        <v>91</v>
+      </c>
+      <c r="J4" s="29" t="s">
+        <v>92</v>
+      </c>
+      <c r="K4" s="29" t="s">
+        <v>135</v>
+      </c>
+      <c r="L4" s="29" t="s">
+        <v>136</v>
+      </c>
+      <c r="M4" s="29"/>
+      <c r="N4" s="29" t="s">
+        <v>90</v>
+      </c>
+      <c r="O4" s="29" t="s">
+        <v>91</v>
+      </c>
+      <c r="P4" s="29" t="s">
+        <v>92</v>
+      </c>
+      <c r="Q4" s="29" t="s">
+        <v>135</v>
+      </c>
+      <c r="R4" s="29" t="s">
+        <v>136</v>
+      </c>
+      <c r="S4" s="6"/>
+      <c r="T4" s="29" t="s">
+        <v>90</v>
+      </c>
+      <c r="U4" s="29" t="s">
+        <v>91</v>
+      </c>
+      <c r="V4" s="29" t="s">
+        <v>92</v>
+      </c>
+      <c r="W4" s="29" t="s">
+        <v>135</v>
+      </c>
+      <c r="X4" s="29" t="s">
+        <v>136</v>
+      </c>
+      <c r="Y4" s="17"/>
+      <c r="Z4" s="29" t="s">
+        <v>90</v>
+      </c>
+      <c r="AA4" s="29" t="s">
+        <v>91</v>
+      </c>
+      <c r="AB4" s="29" t="s">
+        <v>92</v>
+      </c>
+      <c r="AC4" s="29" t="s">
+        <v>135</v>
+      </c>
+      <c r="AD4" s="29" t="s">
+        <v>136</v>
+      </c>
+      <c r="AE4" s="17"/>
+      <c r="AF4" s="29" t="s">
+        <v>90</v>
+      </c>
+      <c r="AG4" s="29" t="s">
+        <v>91</v>
+      </c>
+      <c r="AH4" s="29" t="s">
+        <v>92</v>
+      </c>
+      <c r="AI4" s="29" t="s">
+        <v>135</v>
+      </c>
+      <c r="AJ4" s="29" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="5" spans="1:36" x14ac:dyDescent="0.2">
+      <c r="A5" s="17" t="s">
+        <v>85</v>
+      </c>
+      <c r="B5" s="16"/>
+      <c r="C5" s="16"/>
+      <c r="D5" s="16"/>
+      <c r="E5" s="16"/>
+      <c r="F5" s="21"/>
+      <c r="G5" s="21"/>
+      <c r="H5" s="16"/>
+      <c r="I5" s="16"/>
+      <c r="J5" s="16"/>
+      <c r="K5" s="16"/>
+      <c r="L5" s="16"/>
+      <c r="M5" s="16"/>
+      <c r="N5" s="16"/>
+      <c r="O5" s="16"/>
+      <c r="P5" s="16"/>
+      <c r="Q5" s="16"/>
+      <c r="R5" s="16"/>
+      <c r="T5" s="16"/>
+      <c r="U5" s="16"/>
+      <c r="V5" s="16"/>
+      <c r="W5" s="16"/>
+      <c r="X5" s="16"/>
+      <c r="Y5" s="16"/>
+      <c r="Z5" s="16"/>
+      <c r="AA5" s="16"/>
+      <c r="AB5" s="16"/>
+      <c r="AC5" s="16"/>
+      <c r="AD5" s="16"/>
+      <c r="AE5" s="16"/>
+      <c r="AF5" s="16"/>
+      <c r="AG5" s="16"/>
+      <c r="AH5" s="16"/>
+      <c r="AI5" s="16"/>
+      <c r="AJ5" s="16"/>
+    </row>
+    <row r="6" spans="1:36" ht="17" x14ac:dyDescent="0.25">
+      <c r="A6" s="16" t="s">
+        <v>96</v>
+      </c>
+      <c r="B6" s="16"/>
+      <c r="C6" s="16"/>
+      <c r="D6" s="18"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="16"/>
+      <c r="G6" s="16"/>
+      <c r="H6" s="16"/>
+      <c r="I6" s="16"/>
+      <c r="J6" s="18"/>
+      <c r="K6" s="16"/>
+      <c r="L6" s="16"/>
+      <c r="M6" s="16"/>
+      <c r="N6" s="16"/>
+      <c r="O6" s="16"/>
+      <c r="P6" s="18"/>
+      <c r="Q6" s="16"/>
+      <c r="R6" s="16"/>
+      <c r="T6" s="16">
+        <v>13.391</v>
+      </c>
+      <c r="U6" s="16">
+        <v>0.215</v>
+      </c>
+      <c r="V6" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="W6" s="16"/>
+      <c r="X6" s="16"/>
+      <c r="Y6" s="16"/>
+      <c r="Z6" s="16"/>
+      <c r="AA6" s="16"/>
+      <c r="AB6" s="18"/>
+      <c r="AC6" s="16"/>
+      <c r="AD6" s="16"/>
+      <c r="AE6" s="16"/>
+      <c r="AF6" s="16"/>
+      <c r="AG6" s="16"/>
+      <c r="AH6" s="18"/>
+      <c r="AI6" s="16"/>
+      <c r="AJ6" s="16"/>
+    </row>
+    <row r="7" spans="1:36" ht="17" x14ac:dyDescent="0.25">
+      <c r="A7" s="16" t="s">
+        <v>97</v>
+      </c>
+      <c r="B7" s="16"/>
+      <c r="C7" s="16"/>
+      <c r="D7" s="18"/>
+      <c r="E7" s="16"/>
+      <c r="F7" s="16"/>
+      <c r="G7" s="16"/>
+      <c r="H7" s="16"/>
+      <c r="I7" s="16"/>
+      <c r="J7" s="18"/>
+      <c r="K7" s="16"/>
+      <c r="L7" s="16"/>
+      <c r="M7" s="16"/>
+      <c r="N7" s="16"/>
+      <c r="O7" s="16"/>
+      <c r="P7" s="18"/>
+      <c r="Q7" s="16"/>
+      <c r="R7" s="16"/>
+      <c r="T7" s="16">
+        <v>1.222</v>
+      </c>
+      <c r="U7" s="16">
+        <v>0.53400000000000003</v>
+      </c>
+      <c r="V7" s="18">
+        <v>2.1999999999999999E-2</v>
+      </c>
+      <c r="W7" s="16"/>
+      <c r="X7" s="16"/>
+      <c r="Y7" s="16"/>
+      <c r="Z7" s="16"/>
+      <c r="AA7" s="16"/>
+      <c r="AB7" s="18"/>
+      <c r="AC7" s="16"/>
+      <c r="AD7" s="16"/>
+      <c r="AE7" s="16"/>
+      <c r="AF7" s="16"/>
+      <c r="AG7" s="16"/>
+      <c r="AH7" s="18"/>
+      <c r="AI7" s="16"/>
+      <c r="AJ7" s="16"/>
+    </row>
+    <row r="8" spans="1:36" x14ac:dyDescent="0.2">
+      <c r="A8" s="16"/>
+      <c r="B8" s="16"/>
+      <c r="C8" s="16"/>
+      <c r="D8" s="18"/>
+      <c r="E8" s="18"/>
+      <c r="F8" s="21"/>
+      <c r="G8" s="21"/>
+      <c r="H8" s="16"/>
+      <c r="I8" s="16"/>
+      <c r="J8" s="18"/>
+      <c r="K8" s="18"/>
+      <c r="L8" s="16"/>
+      <c r="M8" s="16"/>
+      <c r="N8" s="16"/>
+      <c r="O8" s="16"/>
+      <c r="P8" s="18"/>
+      <c r="Q8" s="18"/>
+      <c r="R8" s="16"/>
+      <c r="T8" s="16"/>
+      <c r="U8" s="16"/>
+      <c r="V8" s="18"/>
+      <c r="W8" s="18"/>
+      <c r="X8" s="21"/>
+      <c r="Y8" s="21"/>
+      <c r="Z8" s="16"/>
+      <c r="AA8" s="16"/>
+      <c r="AB8" s="18"/>
+      <c r="AC8" s="18"/>
+      <c r="AD8" s="16"/>
+      <c r="AE8" s="16"/>
+      <c r="AF8" s="16"/>
+      <c r="AG8" s="16"/>
+      <c r="AH8" s="18"/>
+      <c r="AI8" s="18"/>
+      <c r="AJ8" s="16"/>
+    </row>
+    <row r="9" spans="1:36" x14ac:dyDescent="0.2">
+      <c r="A9" s="17" t="s">
+        <v>86</v>
+      </c>
+      <c r="B9" s="16"/>
+      <c r="C9" s="16"/>
+      <c r="D9" s="16"/>
+      <c r="E9" s="16"/>
+      <c r="F9" s="21"/>
+      <c r="G9" s="21"/>
+      <c r="H9" s="16"/>
+      <c r="I9" s="16"/>
+      <c r="J9" s="16"/>
+      <c r="K9" s="16"/>
+      <c r="L9" s="16"/>
+      <c r="M9" s="16"/>
+      <c r="N9" s="16"/>
+      <c r="O9" s="16"/>
+      <c r="P9" s="16"/>
+      <c r="Q9" s="16"/>
+      <c r="R9" s="16"/>
+      <c r="T9" s="16"/>
+      <c r="U9" s="16"/>
+      <c r="V9" s="16"/>
+      <c r="W9" s="16"/>
+      <c r="X9" s="21"/>
+      <c r="Y9" s="21"/>
+      <c r="Z9" s="16"/>
+      <c r="AA9" s="16"/>
+      <c r="AB9" s="16"/>
+      <c r="AC9" s="16"/>
+      <c r="AD9" s="16"/>
+      <c r="AE9" s="16"/>
+      <c r="AF9" s="16"/>
+      <c r="AG9" s="16"/>
+      <c r="AH9" s="16"/>
+      <c r="AI9" s="16"/>
+      <c r="AJ9" s="16"/>
+    </row>
+    <row r="10" spans="1:36" ht="17" x14ac:dyDescent="0.25">
+      <c r="A10" s="16" t="s">
+        <v>98</v>
+      </c>
+      <c r="B10" s="16"/>
+      <c r="C10" s="16"/>
+      <c r="D10" s="18"/>
+      <c r="E10" s="16"/>
+      <c r="F10" s="16"/>
+      <c r="G10" s="16"/>
+      <c r="H10" s="16"/>
+      <c r="I10" s="16"/>
+      <c r="J10" s="18"/>
+      <c r="K10" s="16"/>
+      <c r="L10" s="16"/>
+      <c r="M10" s="16"/>
+      <c r="N10" s="16"/>
+      <c r="O10" s="16"/>
+      <c r="P10" s="18"/>
+      <c r="Q10" s="16"/>
+      <c r="R10" s="16"/>
+      <c r="T10" s="16">
+        <v>0.318</v>
+      </c>
+      <c r="U10" s="16">
+        <v>0.05</v>
+      </c>
+      <c r="V10" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="W10" s="16"/>
+      <c r="X10" s="16"/>
+      <c r="Y10" s="16"/>
+      <c r="Z10" s="16"/>
+      <c r="AA10" s="16"/>
+      <c r="AB10" s="18"/>
+      <c r="AC10" s="16"/>
+      <c r="AD10" s="16"/>
+      <c r="AE10" s="16"/>
+      <c r="AF10" s="16"/>
+      <c r="AG10" s="16"/>
+      <c r="AH10" s="18"/>
+      <c r="AI10" s="16"/>
+      <c r="AJ10" s="16"/>
+    </row>
+    <row r="11" spans="1:36" ht="17" x14ac:dyDescent="0.25">
+      <c r="A11" s="16" t="s">
+        <v>99</v>
+      </c>
+      <c r="B11" s="16"/>
+      <c r="C11" s="16"/>
+      <c r="D11" s="18"/>
+      <c r="E11" s="16"/>
+      <c r="F11" s="16"/>
+      <c r="G11" s="16"/>
+      <c r="H11" s="16"/>
+      <c r="I11" s="16"/>
+      <c r="J11" s="18"/>
+      <c r="K11" s="16"/>
+      <c r="L11" s="16"/>
+      <c r="M11" s="16"/>
+      <c r="N11" s="16"/>
+      <c r="O11" s="16"/>
+      <c r="P11" s="18"/>
+      <c r="Q11" s="16"/>
+      <c r="R11" s="16"/>
+      <c r="T11" s="16">
+        <v>-0.01</v>
+      </c>
+      <c r="U11" s="16">
+        <v>2.1000000000000001E-2</v>
+      </c>
+      <c r="V11" s="18">
+        <v>0.63500000000000001</v>
+      </c>
+      <c r="W11" s="16"/>
+      <c r="X11" s="16"/>
+      <c r="Y11" s="16"/>
+      <c r="Z11" s="16"/>
+      <c r="AA11" s="16"/>
+      <c r="AB11" s="18"/>
+      <c r="AC11" s="16"/>
+      <c r="AD11" s="16"/>
+      <c r="AE11" s="16"/>
+      <c r="AF11" s="16"/>
+      <c r="AG11" s="16"/>
+      <c r="AH11" s="18"/>
+      <c r="AI11" s="16"/>
+      <c r="AJ11" s="16"/>
+    </row>
+    <row r="12" spans="1:36" ht="17" x14ac:dyDescent="0.25">
+      <c r="A12" s="16" t="s">
+        <v>100</v>
+      </c>
+      <c r="B12" s="16"/>
+      <c r="C12" s="16"/>
+      <c r="D12" s="18"/>
+      <c r="E12" s="16"/>
+      <c r="F12" s="16"/>
+      <c r="G12" s="16"/>
+      <c r="H12" s="16"/>
+      <c r="I12" s="16"/>
+      <c r="J12" s="18"/>
+      <c r="K12" s="16"/>
+      <c r="L12" s="16"/>
+      <c r="M12" s="16"/>
+      <c r="N12" s="16"/>
+      <c r="O12" s="16"/>
+      <c r="P12" s="18"/>
+      <c r="Q12" s="16"/>
+      <c r="R12" s="16"/>
+      <c r="T12" s="16">
+        <v>7.0999999999999994E-2</v>
+      </c>
+      <c r="U12" s="16">
+        <v>2.1000000000000001E-2</v>
+      </c>
+      <c r="V12" s="18">
+        <v>1E-3</v>
+      </c>
+      <c r="W12" s="16"/>
+      <c r="X12" s="16"/>
+      <c r="Y12" s="16"/>
+      <c r="Z12" s="16"/>
+      <c r="AA12" s="16"/>
+      <c r="AB12" s="18"/>
+      <c r="AC12" s="16"/>
+      <c r="AD12" s="16"/>
+      <c r="AE12" s="16"/>
+      <c r="AF12" s="16"/>
+      <c r="AG12" s="16"/>
+      <c r="AH12" s="18"/>
+      <c r="AI12" s="16"/>
+      <c r="AJ12" s="16"/>
+    </row>
+    <row r="13" spans="1:36" ht="17" x14ac:dyDescent="0.25">
+      <c r="A13" s="16" t="s">
+        <v>101</v>
+      </c>
+      <c r="B13" s="16"/>
+      <c r="C13" s="16"/>
+      <c r="D13" s="16"/>
+      <c r="E13" s="16"/>
+      <c r="F13" s="16"/>
+      <c r="G13" s="16"/>
+      <c r="H13" s="16"/>
+      <c r="I13" s="16"/>
+      <c r="J13" s="18"/>
+      <c r="K13" s="16"/>
+      <c r="L13" s="16"/>
+      <c r="M13" s="16"/>
+      <c r="N13" s="16"/>
+      <c r="O13" s="16"/>
+      <c r="P13" s="18"/>
+      <c r="Q13" s="16"/>
+      <c r="R13" s="16"/>
+      <c r="T13" s="16">
+        <v>0.16800000000000001</v>
+      </c>
+      <c r="U13" s="16">
+        <v>3.5999999999999997E-2</v>
+      </c>
+      <c r="V13" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="W13" s="16"/>
+      <c r="X13" s="16"/>
+      <c r="Y13" s="16"/>
+      <c r="Z13" s="16"/>
+      <c r="AA13" s="16"/>
+      <c r="AB13" s="16"/>
+      <c r="AC13" s="16"/>
+      <c r="AD13" s="16"/>
+      <c r="AE13" s="16"/>
+      <c r="AF13" s="16"/>
+      <c r="AG13" s="16"/>
+      <c r="AH13" s="18"/>
+      <c r="AI13" s="16"/>
+      <c r="AJ13" s="16"/>
+    </row>
+    <row r="14" spans="1:36" x14ac:dyDescent="0.2">
+      <c r="A14" s="16" t="s">
+        <v>88</v>
+      </c>
+      <c r="B14" s="16"/>
+      <c r="C14" s="16"/>
+      <c r="D14" s="18"/>
+      <c r="E14" s="16"/>
+      <c r="F14" s="16"/>
+      <c r="G14" s="16"/>
+      <c r="H14" s="16"/>
+      <c r="I14" s="16"/>
+      <c r="J14" s="18"/>
+      <c r="K14" s="16"/>
+      <c r="L14" s="16"/>
+      <c r="M14" s="16"/>
+      <c r="N14" s="16"/>
+      <c r="O14" s="16"/>
+      <c r="P14" s="18"/>
+      <c r="Q14" s="16"/>
+      <c r="R14" s="16"/>
+      <c r="T14" s="16">
+        <v>0.248</v>
+      </c>
+      <c r="U14" s="16">
+        <v>2.1999999999999999E-2</v>
+      </c>
+      <c r="V14" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="W14" s="16"/>
+      <c r="X14" s="16"/>
+      <c r="Y14" s="16"/>
+      <c r="Z14" s="16"/>
+      <c r="AA14" s="16"/>
+      <c r="AB14" s="18"/>
+      <c r="AC14" s="16"/>
+      <c r="AD14" s="16"/>
+      <c r="AE14" s="16"/>
+      <c r="AF14" s="16"/>
+      <c r="AG14" s="16"/>
+      <c r="AH14" s="18"/>
+      <c r="AI14" s="16"/>
+      <c r="AJ14" s="16"/>
+    </row>
+    <row r="15" spans="1:36" x14ac:dyDescent="0.2">
+      <c r="A15" s="16"/>
+      <c r="B15" s="16"/>
+      <c r="C15" s="16"/>
+      <c r="D15" s="18"/>
+      <c r="E15" s="18"/>
+      <c r="F15" s="21"/>
+      <c r="G15" s="21"/>
+      <c r="H15" s="16"/>
+      <c r="I15" s="16"/>
+      <c r="J15" s="18"/>
+      <c r="K15" s="18"/>
+      <c r="L15" s="16"/>
+      <c r="M15" s="16"/>
+      <c r="N15" s="16"/>
+      <c r="O15" s="16"/>
+      <c r="P15" s="18"/>
+      <c r="Q15" s="18"/>
+      <c r="R15" s="16"/>
+      <c r="T15" s="16"/>
+      <c r="U15" s="16"/>
+      <c r="V15" s="18"/>
+      <c r="W15" s="18"/>
+      <c r="X15" s="21"/>
+      <c r="Y15" s="21"/>
+      <c r="Z15" s="16"/>
+      <c r="AA15" s="16"/>
+      <c r="AB15" s="18"/>
+      <c r="AC15" s="18"/>
+      <c r="AD15" s="16"/>
+      <c r="AE15" s="16"/>
+      <c r="AF15" s="16"/>
+      <c r="AG15" s="16"/>
+      <c r="AH15" s="18"/>
+      <c r="AI15" s="18"/>
+      <c r="AJ15" s="16"/>
+    </row>
+    <row r="16" spans="1:36" x14ac:dyDescent="0.2">
+      <c r="A16" s="17" t="s">
+        <v>87</v>
+      </c>
+      <c r="B16" s="16"/>
+      <c r="C16" s="16"/>
+      <c r="D16" s="16"/>
+      <c r="E16" s="16"/>
+      <c r="F16" s="21"/>
+      <c r="G16" s="21"/>
+      <c r="H16" s="16"/>
+      <c r="I16" s="16"/>
+      <c r="J16" s="16"/>
+      <c r="K16" s="16"/>
+      <c r="L16" s="16"/>
+      <c r="M16" s="16"/>
+      <c r="N16" s="16"/>
+      <c r="O16" s="16"/>
+      <c r="P16" s="16"/>
+      <c r="Q16" s="16"/>
+      <c r="R16" s="16"/>
+      <c r="T16" s="16"/>
+      <c r="U16" s="16"/>
+      <c r="V16" s="16"/>
+      <c r="W16" s="16"/>
+      <c r="X16" s="21"/>
+      <c r="Y16" s="21"/>
+      <c r="Z16" s="16"/>
+      <c r="AA16" s="16"/>
+      <c r="AB16" s="16"/>
+      <c r="AC16" s="16"/>
+      <c r="AD16" s="16"/>
+      <c r="AE16" s="16"/>
+      <c r="AF16" s="16"/>
+      <c r="AG16" s="16"/>
+      <c r="AH16" s="16"/>
+      <c r="AI16" s="16"/>
+      <c r="AJ16" s="16"/>
+    </row>
+    <row r="17" spans="1:36" ht="17" x14ac:dyDescent="0.25">
+      <c r="A17" s="16" t="s">
+        <v>102</v>
+      </c>
+      <c r="B17" s="16"/>
+      <c r="C17" s="16"/>
+      <c r="D17" s="18"/>
+      <c r="E17" s="16"/>
+      <c r="F17" s="16"/>
+      <c r="G17" s="16"/>
+      <c r="H17" s="16"/>
+      <c r="I17" s="16"/>
+      <c r="J17" s="18"/>
+      <c r="K17" s="16"/>
+      <c r="L17" s="16"/>
+      <c r="M17" s="16"/>
+      <c r="N17" s="16"/>
+      <c r="O17" s="16"/>
+      <c r="P17" s="18"/>
+      <c r="Q17" s="16"/>
+      <c r="R17" s="16"/>
+      <c r="T17" s="16">
+        <v>8.5000000000000006E-2</v>
+      </c>
+      <c r="U17" s="16">
+        <v>3.6999999999999998E-2</v>
+      </c>
+      <c r="V17" s="18">
+        <v>2.1000000000000001E-2</v>
+      </c>
+      <c r="W17" s="16"/>
+      <c r="X17" s="16"/>
+      <c r="Y17" s="16"/>
+      <c r="Z17" s="16"/>
+      <c r="AA17" s="16"/>
+      <c r="AB17" s="18"/>
+      <c r="AC17" s="16"/>
+      <c r="AD17" s="16"/>
+      <c r="AE17" s="16"/>
+      <c r="AF17" s="16"/>
+      <c r="AG17" s="16"/>
+      <c r="AH17" s="18"/>
+      <c r="AI17" s="16"/>
+      <c r="AJ17" s="16"/>
+    </row>
+    <row r="18" spans="1:36" ht="17" x14ac:dyDescent="0.25">
+      <c r="A18" s="16" t="s">
+        <v>103</v>
+      </c>
+      <c r="B18" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="C18" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="D18" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="E18" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="F18" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="G18" s="21"/>
+      <c r="H18" s="16"/>
+      <c r="I18" s="16"/>
+      <c r="J18" s="18"/>
+      <c r="K18" s="16"/>
+      <c r="L18" s="16"/>
+      <c r="M18" s="16"/>
+      <c r="N18" s="16"/>
+      <c r="O18" s="16"/>
+      <c r="P18" s="18"/>
+      <c r="Q18" s="16"/>
+      <c r="R18" s="16"/>
+      <c r="T18" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="U18" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="V18" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="W18" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="X18" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="Y18" s="21"/>
+      <c r="Z18" s="16"/>
+      <c r="AA18" s="16"/>
+      <c r="AB18" s="18"/>
+      <c r="AC18" s="16"/>
+      <c r="AD18" s="16"/>
+      <c r="AE18" s="16"/>
+      <c r="AF18" s="16"/>
+      <c r="AG18" s="16"/>
+      <c r="AH18" s="18"/>
+      <c r="AI18" s="16"/>
+      <c r="AJ18" s="16"/>
+    </row>
+    <row r="19" spans="1:36" ht="17" x14ac:dyDescent="0.25">
+      <c r="A19" s="16" t="s">
+        <v>104</v>
+      </c>
+      <c r="B19" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="C19" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="D19" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="E19" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="F19" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="G19" s="21"/>
+      <c r="H19" s="22"/>
+      <c r="I19" s="22"/>
+      <c r="J19" s="16"/>
+      <c r="K19" s="16"/>
+      <c r="L19" s="16"/>
+      <c r="M19" s="16"/>
+      <c r="N19" s="16"/>
+      <c r="O19" s="16"/>
+      <c r="P19" s="18"/>
+      <c r="Q19" s="16"/>
+      <c r="R19" s="16"/>
+      <c r="T19" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="U19" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="V19" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="W19" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="X19" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="Y19" s="21"/>
+      <c r="Z19" s="16"/>
+      <c r="AA19" s="16"/>
+      <c r="AB19" s="16"/>
+      <c r="AC19" s="16"/>
+      <c r="AD19" s="16"/>
+      <c r="AE19" s="16"/>
+      <c r="AF19" s="16"/>
+      <c r="AG19" s="16"/>
+      <c r="AH19" s="16"/>
+      <c r="AI19" s="16"/>
+      <c r="AJ19" s="30"/>
+    </row>
+    <row r="20" spans="1:36" x14ac:dyDescent="0.2">
+      <c r="A20" s="16" t="s">
+        <v>107</v>
+      </c>
+      <c r="B20" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="C20" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="D20" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="E20" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="F20" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="G20" s="21"/>
+      <c r="H20" s="16"/>
+      <c r="I20" s="16"/>
+      <c r="J20" s="18"/>
+      <c r="K20" s="16"/>
+      <c r="L20" s="16"/>
+      <c r="M20" s="16"/>
+      <c r="N20" s="16"/>
+      <c r="O20" s="16"/>
+      <c r="P20" s="18"/>
+      <c r="Q20" s="16"/>
+      <c r="R20" s="16"/>
+      <c r="T20" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="U20" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="V20" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="W20" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="X20" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="Y20" s="21"/>
+      <c r="Z20" s="16"/>
+      <c r="AA20" s="16"/>
+      <c r="AB20" s="18"/>
+      <c r="AC20" s="16"/>
+      <c r="AD20" s="16"/>
+      <c r="AE20" s="16"/>
+      <c r="AF20" s="16"/>
+      <c r="AG20" s="16"/>
+      <c r="AH20" s="16"/>
+      <c r="AI20" s="16"/>
+      <c r="AJ20" s="16"/>
+    </row>
+    <row r="21" spans="1:36" x14ac:dyDescent="0.2">
+      <c r="A21" s="16" t="s">
+        <v>108</v>
+      </c>
+      <c r="B21" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="C21" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="D21" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="E21" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="F21" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="G21" s="21"/>
+      <c r="H21" s="16"/>
+      <c r="I21" s="16"/>
+      <c r="J21" s="18"/>
+      <c r="K21" s="16"/>
+      <c r="L21" s="16"/>
+      <c r="M21" s="16"/>
+      <c r="N21" s="16"/>
+      <c r="O21" s="16"/>
+      <c r="P21" s="18"/>
+      <c r="Q21" s="16"/>
+      <c r="R21" s="16"/>
+      <c r="T21" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="U21" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="V21" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="W21" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="X21" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="Y21" s="21"/>
+      <c r="Z21" s="16"/>
+      <c r="AA21" s="16"/>
+      <c r="AB21" s="16"/>
+      <c r="AC21" s="16"/>
+      <c r="AD21" s="16"/>
+      <c r="AE21" s="16"/>
+      <c r="AF21" s="16"/>
+      <c r="AG21" s="16"/>
+      <c r="AH21" s="18"/>
+      <c r="AI21" s="16"/>
+      <c r="AJ21" s="16"/>
+    </row>
+    <row r="22" spans="1:36" ht="17" x14ac:dyDescent="0.25">
+      <c r="A22" s="16" t="s">
+        <v>105</v>
+      </c>
+      <c r="B22" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="C22" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="D22" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="E22" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="F22" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="G22" s="21"/>
+      <c r="H22" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="I22" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="J22" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="K22" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="L22" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="M22" s="16"/>
+      <c r="N22" s="16"/>
+      <c r="O22" s="16"/>
+      <c r="P22" s="18"/>
+      <c r="Q22" s="16"/>
+      <c r="R22" s="16"/>
+      <c r="T22" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="U22" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="V22" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="W22" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="X22" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="Y22" s="21"/>
+      <c r="Z22" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="AA22" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="AB22" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="AC22" s="16"/>
+      <c r="AD22" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="AE22" s="16"/>
+      <c r="AF22" s="16"/>
+      <c r="AG22" s="16"/>
+      <c r="AH22" s="18"/>
+      <c r="AI22" s="16"/>
+      <c r="AJ22" s="16"/>
+    </row>
+    <row r="23" spans="1:36" ht="17" x14ac:dyDescent="0.25">
+      <c r="A23" s="16" t="s">
+        <v>106</v>
+      </c>
+      <c r="B23" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="C23" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="D23" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="E23" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="F23" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="G23" s="21"/>
+      <c r="H23" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="I23" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="J23" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="K23" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="L23" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="M23" s="16"/>
+      <c r="N23" s="16"/>
+      <c r="O23" s="16"/>
+      <c r="P23" s="18"/>
+      <c r="Q23" s="16"/>
+      <c r="R23" s="16"/>
+      <c r="T23" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="U23" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="V23" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="W23" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="X23" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="Y23" s="21"/>
+      <c r="Z23" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="AA23" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="AB23" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="AC23" s="16"/>
+      <c r="AD23" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="AE23" s="16"/>
+      <c r="AF23" s="16"/>
+      <c r="AG23" s="16"/>
+      <c r="AH23" s="16"/>
+      <c r="AI23" s="16"/>
+      <c r="AJ23" s="16"/>
+    </row>
+    <row r="24" spans="1:36" x14ac:dyDescent="0.2">
+      <c r="A24" s="16" t="s">
+        <v>110</v>
+      </c>
+      <c r="B24" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="C24" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="D24" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="E24" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="F24" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="G24" s="21"/>
+      <c r="H24" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="I24" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="J24" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="K24" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="L24" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="M24" s="16"/>
+      <c r="N24" s="16"/>
+      <c r="O24" s="16"/>
+      <c r="P24" s="18"/>
+      <c r="Q24" s="16"/>
+      <c r="R24" s="16"/>
+      <c r="T24" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="U24" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="V24" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="W24" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="X24" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="Y24" s="21"/>
+      <c r="Z24" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="AA24" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="AB24" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="AC24" s="16"/>
+      <c r="AD24" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="AE24" s="16"/>
+      <c r="AF24" s="16"/>
+      <c r="AG24" s="16"/>
+      <c r="AH24" s="18"/>
+      <c r="AI24" s="16"/>
+      <c r="AJ24" s="16"/>
+    </row>
+    <row r="25" spans="1:36" x14ac:dyDescent="0.2">
+      <c r="A25" s="16" t="s">
+        <v>109</v>
+      </c>
+      <c r="B25" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="C25" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="D25" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="E25" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="F25" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="G25" s="21"/>
+      <c r="H25" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="I25" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="J25" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="K25" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="L25" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="M25" s="16"/>
+      <c r="N25" s="16"/>
+      <c r="O25" s="16"/>
+      <c r="P25" s="18"/>
+      <c r="Q25" s="16"/>
+      <c r="R25" s="16"/>
+      <c r="T25" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="U25" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="V25" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="W25" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="X25" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="Y25" s="21"/>
+      <c r="Z25" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="AA25" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="AB25" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="AC25" s="16"/>
+      <c r="AD25" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="AE25" s="16"/>
+      <c r="AF25" s="16"/>
+      <c r="AG25" s="16"/>
+      <c r="AH25" s="16"/>
+      <c r="AI25" s="16"/>
+      <c r="AJ25" s="16"/>
+    </row>
+    <row r="26" spans="1:36" x14ac:dyDescent="0.2">
+      <c r="A26" s="16" t="s">
+        <v>111</v>
+      </c>
+      <c r="B26" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="C26" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="D26" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="E26" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="F26" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="G26" s="21"/>
+      <c r="H26" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="I26" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="J26" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="K26" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="L26" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="M26" s="16"/>
+      <c r="N26" s="16"/>
+      <c r="O26" s="16"/>
+      <c r="P26" s="18"/>
+      <c r="Q26" s="16"/>
+      <c r="R26" s="16"/>
+      <c r="T26" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="U26" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="V26" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="W26" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="X26" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="Y26" s="21"/>
+      <c r="Z26" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="AA26" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="AB26" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="AC26" s="16"/>
+      <c r="AD26" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="AE26" s="16"/>
+      <c r="AF26" s="16"/>
+      <c r="AG26" s="16"/>
+      <c r="AH26" s="18"/>
+      <c r="AI26" s="16"/>
+      <c r="AJ26" s="16"/>
+    </row>
+    <row r="27" spans="1:36" x14ac:dyDescent="0.2">
+      <c r="A27" s="16"/>
+      <c r="B27" s="16"/>
+      <c r="C27" s="16"/>
+      <c r="D27" s="16"/>
+      <c r="E27" s="16"/>
+      <c r="F27" s="21"/>
+      <c r="G27" s="21"/>
+      <c r="H27" s="16"/>
+      <c r="I27" s="16"/>
+      <c r="J27" s="16"/>
+      <c r="K27" s="16"/>
+      <c r="L27" s="16"/>
+      <c r="M27" s="16"/>
+      <c r="N27" s="16"/>
+      <c r="O27" s="16"/>
+      <c r="P27" s="18"/>
+      <c r="Q27" s="18"/>
+      <c r="R27" s="16"/>
+      <c r="T27" s="16"/>
+      <c r="U27" s="16"/>
+      <c r="V27" s="16"/>
+      <c r="W27" s="16"/>
+      <c r="X27" s="21"/>
+      <c r="Y27" s="21"/>
+      <c r="Z27" s="16"/>
+      <c r="AA27" s="16"/>
+      <c r="AB27" s="16"/>
+      <c r="AC27" s="16"/>
+      <c r="AD27" s="16"/>
+      <c r="AE27" s="16"/>
+      <c r="AF27" s="16"/>
+      <c r="AG27" s="16"/>
+      <c r="AH27" s="18"/>
+      <c r="AI27" s="18"/>
+      <c r="AJ27" s="16"/>
+    </row>
+    <row r="28" spans="1:36" x14ac:dyDescent="0.2">
+      <c r="A28" s="17" t="s">
+        <v>82</v>
+      </c>
+      <c r="B28" s="16"/>
+      <c r="C28" s="16"/>
+      <c r="D28" s="16"/>
+      <c r="E28" s="16"/>
+      <c r="F28" s="21"/>
+      <c r="G28" s="21"/>
+      <c r="H28" s="16"/>
+      <c r="I28" s="16"/>
+      <c r="J28" s="16"/>
+      <c r="K28" s="16"/>
+      <c r="L28" s="16"/>
+      <c r="M28" s="16"/>
+      <c r="N28" s="16"/>
+      <c r="O28" s="16"/>
+      <c r="P28" s="16"/>
+      <c r="Q28" s="16"/>
+      <c r="R28" s="16"/>
+      <c r="T28" s="16"/>
+      <c r="U28" s="16"/>
+      <c r="V28" s="16"/>
+      <c r="W28" s="16"/>
+      <c r="X28" s="21"/>
+      <c r="Y28" s="21"/>
+      <c r="Z28" s="16"/>
+      <c r="AA28" s="16"/>
+      <c r="AB28" s="16"/>
+      <c r="AC28" s="16"/>
+      <c r="AD28" s="16"/>
+      <c r="AE28" s="16"/>
+      <c r="AF28" s="16"/>
+      <c r="AG28" s="16"/>
+      <c r="AH28" s="16"/>
+      <c r="AI28" s="16"/>
+      <c r="AJ28" s="16"/>
+    </row>
+    <row r="29" spans="1:36" x14ac:dyDescent="0.2">
+      <c r="A29" s="16" t="s">
+        <v>84</v>
+      </c>
+      <c r="B29" s="16"/>
+      <c r="C29" s="16"/>
+      <c r="D29" s="18"/>
+      <c r="E29" s="16"/>
+      <c r="F29" s="16"/>
+      <c r="G29" s="16"/>
+      <c r="H29" s="16"/>
+      <c r="I29" s="16"/>
+      <c r="J29" s="18"/>
+      <c r="K29" s="16"/>
+      <c r="L29" s="16"/>
+      <c r="M29" s="16"/>
+      <c r="N29" s="16"/>
+      <c r="O29" s="16"/>
+      <c r="P29" s="18"/>
+      <c r="Q29" s="16"/>
+      <c r="R29" s="16"/>
+      <c r="T29" s="16">
+        <v>13.827</v>
+      </c>
+      <c r="U29" s="16">
+        <v>0.20100000000000001</v>
+      </c>
+      <c r="V29" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="W29" s="16"/>
+      <c r="X29" s="16"/>
+      <c r="Y29" s="16"/>
+      <c r="Z29" s="16"/>
+      <c r="AA29" s="16"/>
+      <c r="AB29" s="18"/>
+      <c r="AC29" s="16"/>
+      <c r="AD29" s="16"/>
+      <c r="AE29" s="16"/>
+      <c r="AF29" s="16"/>
+      <c r="AG29" s="16"/>
+      <c r="AH29" s="18"/>
+      <c r="AI29" s="16"/>
+      <c r="AJ29" s="16"/>
+    </row>
+    <row r="30" spans="1:36" x14ac:dyDescent="0.2">
+      <c r="A30" s="16" t="s">
+        <v>89</v>
+      </c>
+      <c r="B30" s="16"/>
+      <c r="C30" s="16"/>
+      <c r="D30" s="18"/>
+      <c r="E30" s="16"/>
+      <c r="F30" s="16"/>
+      <c r="G30" s="16"/>
+      <c r="H30" s="16"/>
+      <c r="I30" s="16"/>
+      <c r="J30" s="18"/>
+      <c r="K30" s="16"/>
+      <c r="L30" s="16"/>
+      <c r="M30" s="16"/>
+      <c r="N30" s="16"/>
+      <c r="O30" s="16"/>
+      <c r="P30" s="18"/>
+      <c r="Q30" s="16"/>
+      <c r="R30" s="16"/>
+      <c r="T30" s="16">
+        <v>3.8889999999999998</v>
+      </c>
+      <c r="U30" s="16">
+        <v>6.3E-2</v>
+      </c>
+      <c r="V30" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="W30" s="16"/>
+      <c r="X30" s="16"/>
+      <c r="Y30" s="16"/>
+      <c r="Z30" s="16"/>
+      <c r="AA30" s="16"/>
+      <c r="AB30" s="18"/>
+      <c r="AC30" s="16"/>
+      <c r="AD30" s="16"/>
+      <c r="AE30" s="16"/>
+      <c r="AF30" s="16"/>
+      <c r="AG30" s="16"/>
+      <c r="AH30" s="18"/>
+      <c r="AI30" s="16"/>
+      <c r="AJ30" s="16"/>
+    </row>
+    <row r="31" spans="1:36" x14ac:dyDescent="0.2">
+      <c r="A31" s="16" t="s">
+        <v>93</v>
+      </c>
+      <c r="B31" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="C31" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="D31" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="E31" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="F31" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="G31" s="21"/>
+      <c r="H31" s="16"/>
+      <c r="I31" s="16"/>
+      <c r="J31" s="18"/>
+      <c r="K31" s="16"/>
+      <c r="L31" s="16"/>
+      <c r="M31" s="16"/>
+      <c r="N31" s="16"/>
+      <c r="O31" s="16"/>
+      <c r="P31" s="18"/>
+      <c r="Q31" s="16"/>
+      <c r="R31" s="16"/>
+      <c r="T31" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="U31" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="V31" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="W31" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="X31" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="Y31" s="21"/>
+      <c r="Z31" s="16"/>
+      <c r="AA31" s="16"/>
+      <c r="AB31" s="18"/>
+      <c r="AC31" s="16"/>
+      <c r="AD31" s="16"/>
+      <c r="AE31" s="16"/>
+      <c r="AF31" s="16"/>
+      <c r="AG31" s="16"/>
+      <c r="AH31" s="18"/>
+      <c r="AI31" s="16"/>
+      <c r="AJ31" s="16"/>
+    </row>
+    <row r="32" spans="1:36" x14ac:dyDescent="0.2">
+      <c r="A32" s="16" t="s">
+        <v>112</v>
+      </c>
+      <c r="B32" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="C32" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="D32" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="E32" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="F32" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="G32" s="21"/>
+      <c r="H32" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="I32" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="J32" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="K32" s="16"/>
+      <c r="L32" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="M32" s="16"/>
+      <c r="N32" s="16"/>
+      <c r="O32" s="16"/>
+      <c r="P32" s="18"/>
+      <c r="Q32" s="16"/>
+      <c r="R32" s="16"/>
+      <c r="T32" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="U32" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="V32" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="W32" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="X32" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="Y32" s="21"/>
+      <c r="Z32" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="AA32" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="AB32" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="AC32" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="AD32" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="AE32" s="16"/>
+      <c r="AF32" s="16"/>
+      <c r="AG32" s="16"/>
+      <c r="AH32" s="18"/>
+      <c r="AI32" s="16"/>
+      <c r="AJ32" s="16"/>
+    </row>
+    <row r="33" spans="1:39" x14ac:dyDescent="0.2">
+      <c r="A33" s="20" t="s">
+        <v>117</v>
+      </c>
+      <c r="B33" s="14"/>
+      <c r="C33" s="14"/>
+      <c r="D33" s="14"/>
+      <c r="E33" s="14"/>
+      <c r="F33" s="14"/>
+      <c r="G33" s="16"/>
+      <c r="H33" s="14"/>
+      <c r="I33" s="14"/>
+      <c r="J33" s="14"/>
+      <c r="K33" s="14"/>
+      <c r="L33" s="14"/>
+      <c r="M33" s="16"/>
+      <c r="N33" s="14"/>
+      <c r="O33" s="14"/>
+      <c r="P33" s="14"/>
+      <c r="Q33" s="14"/>
+      <c r="R33" s="14"/>
+      <c r="S33" s="16"/>
+      <c r="T33" s="14"/>
+      <c r="U33" s="14"/>
+      <c r="V33" s="14"/>
+      <c r="W33" s="14"/>
+      <c r="X33" s="14"/>
+      <c r="Y33" s="16"/>
+      <c r="Z33" s="14"/>
+      <c r="AA33" s="14"/>
+      <c r="AB33" s="14"/>
+      <c r="AC33" s="14"/>
+      <c r="AD33" s="14"/>
+      <c r="AE33" s="16"/>
+      <c r="AF33" s="14"/>
+      <c r="AG33" s="14"/>
+      <c r="AH33" s="14"/>
+      <c r="AI33" s="14"/>
+      <c r="AJ33" s="14"/>
+      <c r="AK33" s="16"/>
+      <c r="AL33" s="16"/>
+      <c r="AM33" s="16"/>
+    </row>
+    <row r="34" spans="1:39" x14ac:dyDescent="0.2">
+      <c r="A34" s="15" t="s">
+        <v>118</v>
+      </c>
+      <c r="B34" s="31">
+        <v>74058.118000000002</v>
+      </c>
+      <c r="C34" s="31"/>
+      <c r="D34" s="31"/>
+      <c r="E34" s="31"/>
+      <c r="F34" s="31"/>
+      <c r="G34" s="27"/>
+      <c r="H34" s="31">
+        <v>83016.937999999995</v>
+      </c>
+      <c r="I34" s="31"/>
+      <c r="J34" s="31"/>
+      <c r="K34" s="31"/>
+      <c r="L34" s="31"/>
+      <c r="M34" s="27"/>
+      <c r="N34" s="31">
+        <v>94345.274999999994</v>
+      </c>
+      <c r="O34" s="31"/>
+      <c r="P34" s="31"/>
+      <c r="Q34" s="31"/>
+      <c r="R34" s="31"/>
+      <c r="S34" s="15"/>
+      <c r="T34" s="36">
+        <v>37782.404000000002</v>
+      </c>
+      <c r="U34" s="36"/>
+      <c r="V34" s="36"/>
+      <c r="W34" s="36"/>
+      <c r="X34" s="36"/>
+      <c r="Y34" s="27"/>
+      <c r="Z34" s="31"/>
+      <c r="AA34" s="31"/>
+      <c r="AB34" s="31"/>
+      <c r="AC34" s="31"/>
+      <c r="AD34" s="31"/>
+      <c r="AE34" s="27"/>
+      <c r="AF34" s="31"/>
+      <c r="AG34" s="31"/>
+      <c r="AH34" s="31"/>
+      <c r="AI34" s="31"/>
+      <c r="AJ34" s="31"/>
+      <c r="AK34" s="16"/>
+      <c r="AL34" s="16"/>
+      <c r="AM34" s="16"/>
+    </row>
+  </sheetData>
+  <mergeCells count="14">
+    <mergeCell ref="B34:F34"/>
+    <mergeCell ref="H34:L34"/>
+    <mergeCell ref="N34:R34"/>
+    <mergeCell ref="T34:X34"/>
+    <mergeCell ref="Z34:AD34"/>
+    <mergeCell ref="AF34:AJ34"/>
+    <mergeCell ref="B2:R2"/>
+    <mergeCell ref="T2:AJ2"/>
     <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B2:R2"/>
     <mergeCell ref="H3:L3"/>
     <mergeCell ref="N3:R3"/>
-    <mergeCell ref="T2:AJ2"/>
     <mergeCell ref="T3:X3"/>
     <mergeCell ref="Z3:AD3"/>
     <mergeCell ref="AF3:AJ3"/>
@@ -4756,56 +6578,56 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57A86273-0E84-8246-B3ED-A023C6721217}">
   <dimension ref="A1:M38"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="4.625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="5.875" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.1640625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="4.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="5.83203125" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="7.5" style="1" customWidth="1"/>
     <col min="7" max="7" width="7" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="5.125" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="5.625" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="6.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="5.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="5.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="6.1640625" style="1" bestFit="1" customWidth="1"/>
     <col min="11" max="16384" width="11" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" s="14"/>
-      <c r="B2" s="28"/>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
-      <c r="G2" s="28"/>
-      <c r="H2" s="28"/>
-      <c r="I2" s="28"/>
-      <c r="J2" s="28"/>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B2" s="34"/>
+      <c r="C2" s="34"/>
+      <c r="D2" s="34"/>
+      <c r="E2" s="34"/>
+      <c r="G2" s="34"/>
+      <c r="H2" s="34"/>
+      <c r="I2" s="34"/>
+      <c r="J2" s="34"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" s="15"/>
-      <c r="B3" s="27" t="s">
+      <c r="B3" s="35" t="s">
         <v>81</v>
       </c>
-      <c r="C3" s="27"/>
-      <c r="D3" s="27"/>
-      <c r="E3" s="27"/>
-      <c r="G3" s="27" t="s">
+      <c r="C3" s="35"/>
+      <c r="D3" s="35"/>
+      <c r="E3" s="35"/>
+      <c r="G3" s="35" t="s">
         <v>81</v>
       </c>
-      <c r="H3" s="27"/>
-      <c r="I3" s="27"/>
-      <c r="J3" s="27"/>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="H3" s="35"/>
+      <c r="I3" s="35"/>
+      <c r="J3" s="35"/>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" s="16"/>
       <c r="B4" s="17" t="s">
         <v>90</v>
@@ -4832,7 +6654,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" s="17" t="s">
         <v>85</v>
       </c>
@@ -4845,7 +6667,7 @@
       <c r="I5" s="16"/>
       <c r="J5" s="16"/>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" ht="17" x14ac:dyDescent="0.25">
       <c r="A6" s="16" t="s">
         <v>96</v>
       </c>
@@ -4858,7 +6680,7 @@
       <c r="I6" s="18"/>
       <c r="J6" s="16"/>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" ht="17" x14ac:dyDescent="0.25">
       <c r="A7" s="16" t="s">
         <v>97</v>
       </c>
@@ -4871,7 +6693,7 @@
       <c r="I7" s="18"/>
       <c r="J7" s="16"/>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" s="17" t="s">
         <v>86</v>
       </c>
@@ -4884,7 +6706,7 @@
       <c r="I8" s="16"/>
       <c r="J8" s="16"/>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" ht="17" x14ac:dyDescent="0.25">
       <c r="A9" s="16" t="s">
         <v>98</v>
       </c>
@@ -4897,7 +6719,7 @@
       <c r="I9" s="18"/>
       <c r="J9" s="16"/>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" ht="17" x14ac:dyDescent="0.25">
       <c r="A10" s="16" t="s">
         <v>99</v>
       </c>
@@ -4914,7 +6736,7 @@
       <c r="I10" s="18"/>
       <c r="J10" s="16"/>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" ht="17" x14ac:dyDescent="0.25">
       <c r="A11" s="16" t="s">
         <v>100</v>
       </c>
@@ -4931,7 +6753,7 @@
       <c r="I11" s="18"/>
       <c r="J11" s="16"/>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" ht="17" x14ac:dyDescent="0.25">
       <c r="A12" s="25" t="s">
         <v>101</v>
       </c>
@@ -4948,7 +6770,7 @@
       <c r="I12" s="18"/>
       <c r="J12" s="16"/>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" s="16" t="s">
         <v>88</v>
       </c>
@@ -4965,7 +6787,7 @@
       <c r="I13" s="18"/>
       <c r="J13" s="16"/>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14" s="17" t="s">
         <v>87</v>
       </c>
@@ -4978,7 +6800,7 @@
       <c r="I14" s="16"/>
       <c r="J14" s="16"/>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" ht="17" x14ac:dyDescent="0.25">
       <c r="A15" s="16" t="s">
         <v>102</v>
       </c>
@@ -4995,7 +6817,7 @@
       <c r="I15" s="18"/>
       <c r="J15" s="16"/>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" ht="17" x14ac:dyDescent="0.25">
       <c r="A16" s="16" t="s">
         <v>103</v>
       </c>
@@ -5008,7 +6830,7 @@
       <c r="I16" s="18"/>
       <c r="J16" s="16"/>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" ht="17" x14ac:dyDescent="0.25">
       <c r="A17" s="16" t="s">
         <v>104</v>
       </c>
@@ -5021,7 +6843,7 @@
       <c r="I17" s="18"/>
       <c r="J17" s="16"/>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" s="16" t="s">
         <v>107</v>
       </c>
@@ -5038,7 +6860,7 @@
       <c r="I18" s="18"/>
       <c r="J18" s="16"/>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A19" s="16" t="s">
         <v>108</v>
       </c>
@@ -5055,7 +6877,7 @@
       <c r="I19" s="18"/>
       <c r="J19" s="16"/>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" ht="17" x14ac:dyDescent="0.25">
       <c r="A20" s="16" t="s">
         <v>105</v>
       </c>
@@ -5068,7 +6890,7 @@
       <c r="I20" s="18"/>
       <c r="J20" s="16"/>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" ht="17" x14ac:dyDescent="0.25">
       <c r="A21" s="16" t="s">
         <v>106</v>
       </c>
@@ -5081,7 +6903,7 @@
       <c r="I21" s="18"/>
       <c r="J21" s="16"/>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A22" s="16" t="s">
         <v>110</v>
       </c>
@@ -5098,7 +6920,7 @@
       <c r="I22" s="18"/>
       <c r="J22" s="16"/>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A23" s="16" t="s">
         <v>109</v>
       </c>
@@ -5115,7 +6937,7 @@
       <c r="I23" s="18"/>
       <c r="J23" s="16"/>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A24" s="16" t="s">
         <v>111</v>
       </c>
@@ -5128,7 +6950,7 @@
       <c r="I24" s="18"/>
       <c r="J24" s="16"/>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A25" s="17" t="s">
         <v>82</v>
       </c>
@@ -5141,7 +6963,7 @@
       <c r="I25" s="16"/>
       <c r="J25" s="16"/>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A26" s="16" t="s">
         <v>84</v>
       </c>
@@ -5158,7 +6980,7 @@
       <c r="I26" s="18"/>
       <c r="J26" s="16"/>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A27" s="16" t="s">
         <v>89</v>
       </c>
@@ -5175,7 +6997,7 @@
       <c r="I27" s="18"/>
       <c r="J27" s="16"/>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A28" s="16" t="s">
         <v>93</v>
       </c>
@@ -5194,7 +7016,7 @@
       <c r="I28" s="18"/>
       <c r="J28" s="16"/>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A29" s="16" t="s">
         <v>112</v>
       </c>
@@ -5207,7 +7029,7 @@
       <c r="I29" s="18"/>
       <c r="J29" s="16"/>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A30" s="17" t="s">
         <v>83</v>
       </c>
@@ -5220,7 +7042,7 @@
       <c r="I30" s="16"/>
       <c r="J30" s="16"/>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10" ht="17" x14ac:dyDescent="0.25">
       <c r="A31" s="16" t="s">
         <v>96</v>
       </c>
@@ -5239,7 +7061,7 @@
       <c r="I31" s="18"/>
       <c r="J31" s="16"/>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:10" ht="17" x14ac:dyDescent="0.25">
       <c r="A32" s="16" t="s">
         <v>97</v>
       </c>
@@ -5258,7 +7080,7 @@
       <c r="I32" s="18"/>
       <c r="J32" s="16"/>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A33" s="16" t="s">
         <v>84</v>
       </c>
@@ -5275,7 +7097,7 @@
       <c r="I33" s="18"/>
       <c r="J33" s="16"/>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A34" s="16" t="s">
         <v>89</v>
       </c>
@@ -5292,7 +7114,7 @@
       <c r="I34" s="18"/>
       <c r="J34" s="16"/>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A35" s="16" t="s">
         <v>93</v>
       </c>
@@ -5305,7 +7127,7 @@
       <c r="I35" s="18"/>
       <c r="J35" s="16"/>
     </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A36" s="16" t="s">
         <v>112</v>
       </c>
@@ -5316,7 +7138,7 @@
       <c r="H36" s="16"/>
       <c r="I36" s="18"/>
     </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A37" s="20" t="s">
         <v>117</v>
       </c>
@@ -5333,7 +7155,7 @@
       <c r="L37" s="16"/>
       <c r="M37" s="16"/>
     </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A38" s="15" t="s">
         <v>118</v>
       </c>
@@ -5361,57 +7183,57 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{540507A6-720C-0B43-804E-087FEE710926}">
   <dimension ref="A1:E25"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.875" customWidth="1"/>
-    <col min="2" max="2" width="18.875" customWidth="1"/>
-    <col min="3" max="3" width="19.125" customWidth="1"/>
+    <col min="1" max="1" width="19.83203125" customWidth="1"/>
+    <col min="2" max="2" width="18.83203125" customWidth="1"/>
+    <col min="3" max="3" width="19.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="23" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="2" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A2" s="24"/>
     </row>
-    <row r="3" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A3" s="24" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="4" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A4" s="24" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="5" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A5" s="24"/>
     </row>
-    <row r="6" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A6" s="24"/>
     </row>
-    <row r="7" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="8" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="8" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A8" s="23" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" s="24" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" s="24" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="B11" s="23" t="s">
         <v>129</v>
       </c>
@@ -5419,7 +7241,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>126</v>
       </c>
@@ -5430,7 +7252,7 @@
         <v>-1.4E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>127</v>
       </c>
@@ -5441,7 +7263,7 @@
         <v>-8.0000000000000002E-3</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>128</v>
       </c>
@@ -5452,7 +7274,7 @@
         <v>-7.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>133</v>
       </c>
@@ -5463,17 +7285,17 @@
         <v>-8.0000000000000002E-3</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" s="23" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" s="24" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B19" s="23" t="s">
         <v>129</v>
       </c>
@@ -5481,7 +7303,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>126</v>
       </c>
@@ -5492,7 +7314,7 @@
         <v>-1.0999999999999999E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>127</v>
       </c>
@@ -5503,7 +7325,7 @@
         <v>-1.2999999999999999E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>128</v>
       </c>
@@ -5514,7 +7336,7 @@
         <v>9.7000000000000003E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>133</v>
       </c>
@@ -5525,7 +7347,7 @@
         <v>-1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="E25" s="23" t="s">
         <v>132</v>
       </c>

</xml_diff>

<commit_message>
rerun models and updated table
</commit_message>
<xml_diff>
--- a/Tables.xlsx
+++ b/Tables.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10208"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nchaku/Documents/GitHub/pubertybrain/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nchaku\Documents\GitHub\pubertybrain\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DF775CB-4F28-1742-9002-F940C250CB44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF0C5C2D-21F6-4142-814F-EFC173B4BD72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13360" yWindow="500" windowWidth="15440" windowHeight="16400" firstSheet="1" activeTab="5" xr2:uid="{E0F15479-AA73-0644-8B08-3949D67CD8FE}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="5" xr2:uid="{E0F15479-AA73-0644-8B08-3949D67CD8FE}"/>
   </bookViews>
   <sheets>
     <sheet name="Descriptive table" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="723" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="805" uniqueCount="143">
   <si>
     <t>16.10 (2.98)</t>
   </si>
@@ -722,6 +722,119 @@
   </si>
   <si>
     <t>ULCI</t>
+  </si>
+  <si>
+    <t>Table 3. Subcortical volume by sex</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Timing on Quadratic Slope</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">   Intercept</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="subscript"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>b</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> with Quadratic Slope</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="subscript"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>b</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">   Quadratic Slope</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="subscript"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>b</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">   Slope</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="subscript"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>b</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">      with Quadratic Slope</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="subscript"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>b</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">   Quadratic Slope</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="subscript"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">b </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>with Tempo</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -885,7 +998,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -933,23 +1046,20 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1531,20 +1641,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39987BE7-3659-524A-81AE-D479F97EF698}">
   <dimension ref="A1:F29"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="28.83203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="4" width="20.1640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.83203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28.875" bestFit="1" customWidth="1"/>
+    <col min="2" max="4" width="20.125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="9"/>
       <c r="B2" s="10" t="s">
         <v>63</v>
@@ -1562,7 +1672,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="6"/>
       <c r="B3" s="11" t="s">
         <v>69</v>
@@ -1576,7 +1686,7 @@
       <c r="E3" s="11"/>
       <c r="F3" s="6"/>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>60</v>
       </c>
@@ -1586,7 +1696,7 @@
       <c r="E4" s="2"/>
       <c r="F4" s="1"/>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>61</v>
       </c>
@@ -1606,7 +1716,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>62</v>
       </c>
@@ -1626,7 +1736,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>58</v>
       </c>
@@ -1646,7 +1756,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
         <v>59</v>
       </c>
@@ -1656,7 +1766,7 @@
       <c r="E8" s="12"/>
       <c r="F8" s="1"/>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>61</v>
       </c>
@@ -1676,7 +1786,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>66</v>
       </c>
@@ -1696,7 +1806,7 @@
         <v>0.06</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>67</v>
       </c>
@@ -1716,7 +1826,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>62</v>
       </c>
@@ -1736,7 +1846,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
         <v>68</v>
       </c>
@@ -1746,7 +1856,7 @@
       <c r="E13" s="12"/>
       <c r="F13" s="1"/>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>73</v>
       </c>
@@ -1766,7 +1876,7 @@
         <v>1.74</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>74</v>
       </c>
@@ -1786,7 +1896,7 @@
         <v>1.93</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>75</v>
       </c>
@@ -1806,7 +1916,7 @@
         <v>1.69</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>76</v>
       </c>
@@ -1824,7 +1934,7 @@
       </c>
       <c r="F17" s="19"/>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
         <v>71</v>
       </c>
@@ -1834,7 +1944,7 @@
       <c r="E18" s="12"/>
       <c r="F18" s="1"/>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>61</v>
       </c>
@@ -1854,7 +1964,7 @@
         <v>0.87</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
         <v>66</v>
       </c>
@@ -1874,7 +1984,7 @@
         <v>0.93</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
         <v>67</v>
       </c>
@@ -1894,7 +2004,7 @@
         <v>1.18</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
         <v>62</v>
       </c>
@@ -1914,7 +2024,7 @@
         <v>1.24</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="8" t="s">
         <v>72</v>
       </c>
@@ -1924,7 +2034,7 @@
       <c r="E23" s="12"/>
       <c r="F23" s="1"/>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
         <v>61</v>
       </c>
@@ -1944,7 +2054,7 @@
         <v>0.88</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
         <v>66</v>
       </c>
@@ -1964,7 +2074,7 @@
         <v>0.88</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
         <v>67</v>
       </c>
@@ -1984,7 +2094,7 @@
         <v>1.1299999999999999</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="7" t="s">
         <v>62</v>
       </c>
@@ -2004,7 +2114,7 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="28" spans="1:6" ht="18" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:6" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A28" s="4"/>
       <c r="B28" s="1"/>
       <c r="C28" s="1"/>
@@ -2012,7 +2122,7 @@
       <c r="E28" s="1"/>
       <c r="F28" s="1"/>
     </row>
-    <row r="29" spans="1:6" ht="18" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:6" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A29" s="4"/>
       <c r="B29" s="1"/>
       <c r="C29" s="1"/>
@@ -2028,9 +2138,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A749072B-F938-0F49-BE23-243603B2B3D0}">
   <dimension ref="M2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="2" spans="13:13" x14ac:dyDescent="0.2">
+    <row r="2" spans="13:13" x14ac:dyDescent="0.25">
       <c r="M2" t="s">
         <v>113</v>
       </c>
@@ -2044,7 +2154,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45875D41-9C56-AA4E-A18A-2D3A4CE169B3}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2054,7 +2164,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A2A5153E-6E5C-054A-8ACA-5118463B96C5}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2064,142 +2174,142 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BBA86F85-A8D4-F648-84C3-730F1A42C846}">
   <dimension ref="A1:AM34"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.625" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.625" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="6.5" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="1.1640625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="1.125" style="1" customWidth="1"/>
     <col min="8" max="8" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="5.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="5.6640625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="5.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="5.625" style="1" customWidth="1"/>
     <col min="11" max="11" width="6.5" style="1" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="1.1640625" style="1" customWidth="1"/>
+    <col min="13" max="13" width="1.125" style="1" customWidth="1"/>
     <col min="14" max="14" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="5.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="5.6640625" style="1" customWidth="1"/>
+    <col min="15" max="15" width="5.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="5.625" style="1" customWidth="1"/>
     <col min="17" max="17" width="6.5" style="1" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="0.83203125" style="1" customWidth="1"/>
+    <col min="19" max="19" width="0.875" style="1" customWidth="1"/>
     <col min="20" max="20" width="8.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="5.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="22" max="23" width="5.6640625" style="1" customWidth="1"/>
-    <col min="24" max="24" width="6.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="5.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="22" max="23" width="5.625" style="1" customWidth="1"/>
+    <col min="24" max="24" width="6.125" style="1" bestFit="1" customWidth="1"/>
     <col min="25" max="25" width="1" style="1" customWidth="1"/>
     <col min="26" max="26" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="5.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="5.6640625" style="1" customWidth="1"/>
+    <col min="27" max="27" width="5.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="5.625" style="1" customWidth="1"/>
     <col min="29" max="30" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="1.1640625" style="1" customWidth="1"/>
+    <col min="31" max="31" width="1.125" style="1" customWidth="1"/>
     <col min="32" max="32" width="7" style="1" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="5.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="5.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="5.6640625" style="1" customWidth="1"/>
-    <col min="36" max="36" width="6.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="5.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="5.625" style="1" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="5.625" style="1" customWidth="1"/>
+    <col min="36" max="36" width="6.125" style="1" bestFit="1" customWidth="1"/>
     <col min="37" max="16384" width="11" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="14"/>
-      <c r="B2" s="32" t="s">
+      <c r="B2" s="31" t="s">
         <v>114</v>
       </c>
-      <c r="C2" s="32"/>
-      <c r="D2" s="32"/>
-      <c r="E2" s="32"/>
-      <c r="F2" s="32"/>
-      <c r="G2" s="32"/>
-      <c r="H2" s="32"/>
-      <c r="I2" s="32"/>
-      <c r="J2" s="32"/>
-      <c r="K2" s="32"/>
-      <c r="L2" s="32"/>
-      <c r="M2" s="32"/>
-      <c r="N2" s="32"/>
-      <c r="O2" s="32"/>
-      <c r="P2" s="32"/>
-      <c r="Q2" s="32"/>
-      <c r="R2" s="32"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
+      <c r="G2" s="31"/>
+      <c r="H2" s="31"/>
+      <c r="I2" s="31"/>
+      <c r="J2" s="31"/>
+      <c r="K2" s="31"/>
+      <c r="L2" s="31"/>
+      <c r="M2" s="31"/>
+      <c r="N2" s="31"/>
+      <c r="O2" s="31"/>
+      <c r="P2" s="31"/>
+      <c r="Q2" s="31"/>
+      <c r="R2" s="31"/>
       <c r="S2" s="9"/>
-      <c r="T2" s="32" t="s">
+      <c r="T2" s="31" t="s">
         <v>115</v>
       </c>
-      <c r="U2" s="32"/>
-      <c r="V2" s="32"/>
-      <c r="W2" s="32"/>
-      <c r="X2" s="32"/>
-      <c r="Y2" s="32"/>
-      <c r="Z2" s="32"/>
-      <c r="AA2" s="32"/>
-      <c r="AB2" s="32"/>
-      <c r="AC2" s="32"/>
-      <c r="AD2" s="32"/>
-      <c r="AE2" s="32"/>
-      <c r="AF2" s="32"/>
-      <c r="AG2" s="32"/>
-      <c r="AH2" s="32"/>
-      <c r="AI2" s="32"/>
-      <c r="AJ2" s="32"/>
-    </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.2">
+      <c r="U2" s="31"/>
+      <c r="V2" s="31"/>
+      <c r="W2" s="31"/>
+      <c r="X2" s="31"/>
+      <c r="Y2" s="31"/>
+      <c r="Z2" s="31"/>
+      <c r="AA2" s="31"/>
+      <c r="AB2" s="31"/>
+      <c r="AC2" s="31"/>
+      <c r="AD2" s="31"/>
+      <c r="AE2" s="31"/>
+      <c r="AF2" s="31"/>
+      <c r="AG2" s="31"/>
+      <c r="AH2" s="31"/>
+      <c r="AI2" s="31"/>
+      <c r="AJ2" s="31"/>
+    </row>
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="16"/>
-      <c r="B3" s="32" t="s">
+      <c r="B3" s="31" t="s">
         <v>79</v>
       </c>
-      <c r="C3" s="32"/>
-      <c r="D3" s="32"/>
-      <c r="E3" s="32"/>
-      <c r="F3" s="32"/>
+      <c r="C3" s="31"/>
+      <c r="D3" s="31"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="31"/>
       <c r="G3" s="28"/>
-      <c r="H3" s="32" t="s">
+      <c r="H3" s="31" t="s">
         <v>80</v>
       </c>
-      <c r="I3" s="32"/>
-      <c r="J3" s="32"/>
-      <c r="K3" s="32"/>
-      <c r="L3" s="32"/>
+      <c r="I3" s="31"/>
+      <c r="J3" s="31"/>
+      <c r="K3" s="31"/>
+      <c r="L3" s="31"/>
       <c r="M3" s="28"/>
-      <c r="N3" s="32" t="s">
+      <c r="N3" s="31" t="s">
         <v>81</v>
       </c>
-      <c r="O3" s="32"/>
-      <c r="P3" s="32"/>
-      <c r="Q3" s="32"/>
-      <c r="R3" s="32"/>
-      <c r="T3" s="33" t="s">
+      <c r="O3" s="31"/>
+      <c r="P3" s="31"/>
+      <c r="Q3" s="31"/>
+      <c r="R3" s="31"/>
+      <c r="T3" s="32" t="s">
         <v>79</v>
       </c>
-      <c r="U3" s="33"/>
-      <c r="V3" s="33"/>
-      <c r="W3" s="33"/>
-      <c r="X3" s="33"/>
+      <c r="U3" s="32"/>
+      <c r="V3" s="32"/>
+      <c r="W3" s="32"/>
+      <c r="X3" s="32"/>
       <c r="Y3" s="28"/>
-      <c r="Z3" s="32" t="s">
+      <c r="Z3" s="31" t="s">
         <v>80</v>
       </c>
-      <c r="AA3" s="32"/>
-      <c r="AB3" s="32"/>
-      <c r="AC3" s="32"/>
-      <c r="AD3" s="32"/>
+      <c r="AA3" s="31"/>
+      <c r="AB3" s="31"/>
+      <c r="AC3" s="31"/>
+      <c r="AD3" s="31"/>
       <c r="AE3" s="28"/>
-      <c r="AF3" s="32" t="s">
+      <c r="AF3" s="31" t="s">
         <v>81</v>
       </c>
-      <c r="AG3" s="32"/>
-      <c r="AH3" s="32"/>
-      <c r="AI3" s="32"/>
-      <c r="AJ3" s="32"/>
-    </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.2">
+      <c r="AG3" s="31"/>
+      <c r="AH3" s="31"/>
+      <c r="AI3" s="31"/>
+      <c r="AJ3" s="31"/>
+    </row>
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="15"/>
       <c r="B4" s="29" t="s">
         <v>90</v>
@@ -2297,7 +2407,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="17" t="s">
         <v>85</v>
       </c>
@@ -2336,7 +2446,7 @@
       <c r="AI5" s="16"/>
       <c r="AJ5" s="16"/>
     </row>
-    <row r="6" spans="1:36" ht="17" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="16" t="s">
         <v>96</v>
       </c>
@@ -2435,7 +2545,7 @@
         <v>12.236000000000001</v>
       </c>
     </row>
-    <row r="7" spans="1:36" ht="17" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="16" t="s">
         <v>97</v>
       </c>
@@ -2534,7 +2644,7 @@
         <v>-7.7560000000000002</v>
       </c>
     </row>
-    <row r="8" spans="1:36" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A8" s="16"/>
       <c r="B8" s="16"/>
       <c r="C8" s="16"/>
@@ -2571,7 +2681,7 @@
       <c r="AI8" s="18"/>
       <c r="AJ8" s="16"/>
     </row>
-    <row r="9" spans="1:36" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A9" s="17" t="s">
         <v>86</v>
       </c>
@@ -2610,7 +2720,7 @@
       <c r="AI9" s="16"/>
       <c r="AJ9" s="16"/>
     </row>
-    <row r="10" spans="1:36" ht="17" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A10" s="16" t="s">
         <v>98</v>
       </c>
@@ -2709,7 +2819,7 @@
         <v>-0.24</v>
       </c>
     </row>
-    <row r="11" spans="1:36" ht="17" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A11" s="16" t="s">
         <v>99</v>
       </c>
@@ -2808,7 +2918,7 @@
         <v>0.09</v>
       </c>
     </row>
-    <row r="12" spans="1:36" ht="17" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A12" s="16" t="s">
         <v>100</v>
       </c>
@@ -2907,7 +3017,7 @@
         <v>0.14899999999999999</v>
       </c>
     </row>
-    <row r="13" spans="1:36" ht="17" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="16" t="s">
         <v>101</v>
       </c>
@@ -3006,7 +3116,7 @@
         <v>3.5999999999999997E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A14" s="16" t="s">
         <v>88</v>
       </c>
@@ -3105,7 +3215,7 @@
         <v>0.28799999999999998</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A15" s="16"/>
       <c r="B15" s="16"/>
       <c r="C15" s="16"/>
@@ -3142,7 +3252,7 @@
       <c r="AI15" s="18"/>
       <c r="AJ15" s="16"/>
     </row>
-    <row r="16" spans="1:36" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A16" s="17" t="s">
         <v>87</v>
       </c>
@@ -3181,7 +3291,7 @@
       <c r="AI16" s="16"/>
       <c r="AJ16" s="16"/>
     </row>
-    <row r="17" spans="1:36" ht="17" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A17" s="16" t="s">
         <v>102</v>
       </c>
@@ -3280,7 +3390,7 @@
         <v>0.443</v>
       </c>
     </row>
-    <row r="18" spans="1:36" ht="17" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A18" s="16" t="s">
         <v>103</v>
       </c>
@@ -3379,7 +3489,7 @@
         <v>-0.10299999999999999</v>
       </c>
     </row>
-    <row r="19" spans="1:36" ht="17" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A19" s="16" t="s">
         <v>104</v>
       </c>
@@ -3478,7 +3588,7 @@
         <v>9.0999999999999998E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:36" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A20" s="16" t="s">
         <v>107</v>
       </c>
@@ -3577,7 +3687,7 @@
         <v>3.1E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:36" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A21" s="16" t="s">
         <v>108</v>
       </c>
@@ -3676,7 +3786,7 @@
         <v>-0.13600000000000001</v>
       </c>
     </row>
-    <row r="22" spans="1:36" ht="17" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A22" s="16" t="s">
         <v>105</v>
       </c>
@@ -3773,7 +3883,7 @@
         <v>0.156</v>
       </c>
     </row>
-    <row r="23" spans="1:36" ht="17" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A23" s="16" t="s">
         <v>106</v>
       </c>
@@ -3870,7 +3980,7 @@
         <v>-1.6E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:36" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A24" s="16" t="s">
         <v>110</v>
       </c>
@@ -3967,7 +4077,7 @@
         <v>0.112</v>
       </c>
     </row>
-    <row r="25" spans="1:36" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A25" s="16" t="s">
         <v>109</v>
       </c>
@@ -4064,7 +4174,7 @@
         <v>0.16</v>
       </c>
     </row>
-    <row r="26" spans="1:36" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A26" s="16" t="s">
         <v>111</v>
       </c>
@@ -4161,7 +4271,7 @@
         <v>-4.9000000000000002E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:36" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A27" s="16"/>
       <c r="B27" s="16"/>
       <c r="C27" s="16"/>
@@ -4198,7 +4308,7 @@
       <c r="AI27" s="18"/>
       <c r="AJ27" s="16"/>
     </row>
-    <row r="28" spans="1:36" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A28" s="17" t="s">
         <v>82</v>
       </c>
@@ -4237,7 +4347,7 @@
       <c r="AI28" s="16"/>
       <c r="AJ28" s="16"/>
     </row>
-    <row r="29" spans="1:36" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A29" s="16" t="s">
         <v>84</v>
       </c>
@@ -4336,7 +4446,7 @@
         <v>14.164999999999999</v>
       </c>
     </row>
-    <row r="30" spans="1:36" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A30" s="16" t="s">
         <v>89</v>
       </c>
@@ -4435,7 +4545,7 @@
         <v>4.1660000000000004</v>
       </c>
     </row>
-    <row r="31" spans="1:36" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A31" s="16" t="s">
         <v>93</v>
       </c>
@@ -4534,7 +4644,7 @@
         <v>1.0549999999999999</v>
       </c>
     </row>
-    <row r="32" spans="1:36" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A32" s="16" t="s">
         <v>112</v>
       </c>
@@ -4631,7 +4741,7 @@
         <v>4.202</v>
       </c>
     </row>
-    <row r="33" spans="1:39" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A33" s="20" t="s">
         <v>117</v>
       </c>
@@ -4674,63 +4784,69 @@
       <c r="AL33" s="16"/>
       <c r="AM33" s="16"/>
     </row>
-    <row r="34" spans="1:39" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A34" s="15" t="s">
         <v>118</v>
       </c>
-      <c r="B34" s="31">
+      <c r="B34" s="33">
         <v>74058.118000000002</v>
       </c>
-      <c r="C34" s="31"/>
-      <c r="D34" s="31"/>
-      <c r="E34" s="31"/>
-      <c r="F34" s="31"/>
+      <c r="C34" s="33"/>
+      <c r="D34" s="33"/>
+      <c r="E34" s="33"/>
+      <c r="F34" s="33"/>
       <c r="G34" s="27"/>
-      <c r="H34" s="31">
+      <c r="H34" s="33">
         <v>83016.937999999995</v>
       </c>
-      <c r="I34" s="31"/>
-      <c r="J34" s="31"/>
-      <c r="K34" s="31"/>
-      <c r="L34" s="31"/>
+      <c r="I34" s="33"/>
+      <c r="J34" s="33"/>
+      <c r="K34" s="33"/>
+      <c r="L34" s="33"/>
       <c r="M34" s="27"/>
-      <c r="N34" s="31">
+      <c r="N34" s="33">
         <v>94345.274999999994</v>
       </c>
-      <c r="O34" s="31"/>
-      <c r="P34" s="31"/>
-      <c r="Q34" s="31"/>
-      <c r="R34" s="31"/>
+      <c r="O34" s="33"/>
+      <c r="P34" s="33"/>
+      <c r="Q34" s="33"/>
+      <c r="R34" s="33"/>
       <c r="S34" s="15"/>
-      <c r="T34" s="31">
+      <c r="T34" s="33">
         <v>83167.763000000006</v>
       </c>
-      <c r="U34" s="31"/>
-      <c r="V34" s="31"/>
-      <c r="W34" s="31"/>
-      <c r="X34" s="31"/>
+      <c r="U34" s="33"/>
+      <c r="V34" s="33"/>
+      <c r="W34" s="33"/>
+      <c r="X34" s="33"/>
       <c r="Y34" s="27"/>
-      <c r="Z34" s="31">
+      <c r="Z34" s="33">
         <v>93083.505999999994</v>
       </c>
-      <c r="AA34" s="31"/>
-      <c r="AB34" s="31"/>
-      <c r="AC34" s="31"/>
-      <c r="AD34" s="31"/>
+      <c r="AA34" s="33"/>
+      <c r="AB34" s="33"/>
+      <c r="AC34" s="33"/>
+      <c r="AD34" s="33"/>
       <c r="AE34" s="27"/>
-      <c r="AF34" s="31">
+      <c r="AF34" s="33">
         <v>105770.462</v>
       </c>
-      <c r="AG34" s="31"/>
-      <c r="AH34" s="31"/>
-      <c r="AI34" s="31"/>
-      <c r="AJ34" s="31"/>
+      <c r="AG34" s="33"/>
+      <c r="AH34" s="33"/>
+      <c r="AI34" s="33"/>
+      <c r="AJ34" s="33"/>
       <c r="AK34" s="16"/>
       <c r="AL34" s="16"/>
       <c r="AM34" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="AF34:AJ34"/>
+    <mergeCell ref="B34:F34"/>
+    <mergeCell ref="H34:L34"/>
+    <mergeCell ref="T34:X34"/>
+    <mergeCell ref="N34:R34"/>
+    <mergeCell ref="Z34:AD34"/>
     <mergeCell ref="B3:F3"/>
     <mergeCell ref="B2:R2"/>
     <mergeCell ref="H3:L3"/>
@@ -4739,12 +4855,6 @@
     <mergeCell ref="T3:X3"/>
     <mergeCell ref="Z3:AD3"/>
     <mergeCell ref="AF3:AJ3"/>
-    <mergeCell ref="AF34:AJ34"/>
-    <mergeCell ref="B34:F34"/>
-    <mergeCell ref="H34:L34"/>
-    <mergeCell ref="T34:X34"/>
-    <mergeCell ref="N34:R34"/>
-    <mergeCell ref="Z34:AD34"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
@@ -4753,144 +4863,142 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CD5CF7F-81D6-D24D-8228-B4C578C35D65}">
-  <dimension ref="A1:AM34"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:AM39"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24" style="1" customWidth="1"/>
     <col min="2" max="2" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="1.1640625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="5.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.625" style="1" customWidth="1"/>
+    <col min="5" max="6" width="6" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="1.125" style="1" customWidth="1"/>
     <col min="8" max="8" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="5.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="5.6640625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="5.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="5.625" style="1" customWidth="1"/>
     <col min="11" max="11" width="6.5" style="1" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="1.1640625" style="1" customWidth="1"/>
+    <col min="13" max="13" width="1.125" style="1" customWidth="1"/>
     <col min="14" max="14" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="5.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="5.6640625" style="1" customWidth="1"/>
+    <col min="15" max="15" width="5.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="5.625" style="1" customWidth="1"/>
     <col min="17" max="17" width="6.5" style="1" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="0.83203125" style="1" customWidth="1"/>
-    <col min="20" max="20" width="6.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="5.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="6.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="5.6640625" style="1" customWidth="1"/>
-    <col min="24" max="24" width="6.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="0.875" style="1" customWidth="1"/>
+    <col min="20" max="20" width="6" style="1" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="5.875" style="1" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="6.375" style="1" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="5.625" style="1" customWidth="1"/>
+    <col min="24" max="24" width="6" style="1" bestFit="1" customWidth="1"/>
     <col min="25" max="25" width="1" style="1" customWidth="1"/>
     <col min="26" max="26" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="5.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="5.6640625" style="1" customWidth="1"/>
+    <col min="27" max="27" width="5.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="5.625" style="1" bestFit="1" customWidth="1"/>
     <col min="29" max="30" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="1.1640625" style="1" customWidth="1"/>
-    <col min="32" max="32" width="7" style="1" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="5.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="5.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="5.6640625" style="1" customWidth="1"/>
-    <col min="36" max="36" width="6.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="1.125" style="1" customWidth="1"/>
+    <col min="32" max="32" width="6" style="1" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="5.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="5.625" style="1" customWidth="1"/>
+    <col min="35" max="36" width="6" style="1" bestFit="1" customWidth="1"/>
     <col min="37" max="16384" width="11" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.2">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="14"/>
-      <c r="B2" s="32" t="s">
+      <c r="B2" s="31" t="s">
         <v>114</v>
       </c>
-      <c r="C2" s="32"/>
-      <c r="D2" s="32"/>
-      <c r="E2" s="32"/>
-      <c r="F2" s="32"/>
-      <c r="G2" s="32"/>
-      <c r="H2" s="32"/>
-      <c r="I2" s="32"/>
-      <c r="J2" s="32"/>
-      <c r="K2" s="32"/>
-      <c r="L2" s="32"/>
-      <c r="M2" s="32"/>
-      <c r="N2" s="32"/>
-      <c r="O2" s="32"/>
-      <c r="P2" s="32"/>
-      <c r="Q2" s="32"/>
-      <c r="R2" s="32"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
+      <c r="G2" s="31"/>
+      <c r="H2" s="31"/>
+      <c r="I2" s="31"/>
+      <c r="J2" s="31"/>
+      <c r="K2" s="31"/>
+      <c r="L2" s="31"/>
+      <c r="M2" s="31"/>
+      <c r="N2" s="31"/>
+      <c r="O2" s="31"/>
+      <c r="P2" s="31"/>
+      <c r="Q2" s="31"/>
+      <c r="R2" s="31"/>
       <c r="S2" s="9"/>
-      <c r="T2" s="32" t="s">
+      <c r="T2" s="31" t="s">
         <v>115</v>
       </c>
-      <c r="U2" s="32"/>
-      <c r="V2" s="32"/>
-      <c r="W2" s="32"/>
-      <c r="X2" s="32"/>
-      <c r="Y2" s="32"/>
-      <c r="Z2" s="32"/>
-      <c r="AA2" s="32"/>
-      <c r="AB2" s="32"/>
-      <c r="AC2" s="32"/>
-      <c r="AD2" s="32"/>
-      <c r="AE2" s="32"/>
-      <c r="AF2" s="32"/>
-      <c r="AG2" s="32"/>
-      <c r="AH2" s="32"/>
-      <c r="AI2" s="32"/>
-      <c r="AJ2" s="32"/>
-    </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.2">
+      <c r="U2" s="31"/>
+      <c r="V2" s="31"/>
+      <c r="W2" s="31"/>
+      <c r="X2" s="31"/>
+      <c r="Y2" s="31"/>
+      <c r="Z2" s="31"/>
+      <c r="AA2" s="31"/>
+      <c r="AB2" s="31"/>
+      <c r="AC2" s="31"/>
+      <c r="AD2" s="31"/>
+      <c r="AE2" s="31"/>
+      <c r="AF2" s="31"/>
+      <c r="AG2" s="31"/>
+      <c r="AH2" s="31"/>
+      <c r="AI2" s="31"/>
+      <c r="AJ2" s="31"/>
+    </row>
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="16"/>
-      <c r="B3" s="32" t="s">
+      <c r="B3" s="31" t="s">
         <v>79</v>
       </c>
-      <c r="C3" s="32"/>
-      <c r="D3" s="32"/>
-      <c r="E3" s="32"/>
-      <c r="F3" s="32"/>
+      <c r="C3" s="31"/>
+      <c r="D3" s="31"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="31"/>
       <c r="G3" s="28"/>
-      <c r="H3" s="32" t="s">
+      <c r="H3" s="31" t="s">
         <v>80</v>
       </c>
-      <c r="I3" s="32"/>
-      <c r="J3" s="32"/>
-      <c r="K3" s="32"/>
-      <c r="L3" s="32"/>
+      <c r="I3" s="31"/>
+      <c r="J3" s="31"/>
+      <c r="K3" s="31"/>
+      <c r="L3" s="31"/>
       <c r="M3" s="28"/>
-      <c r="N3" s="32" t="s">
+      <c r="N3" s="31" t="s">
         <v>81</v>
       </c>
-      <c r="O3" s="32"/>
-      <c r="P3" s="32"/>
-      <c r="Q3" s="32"/>
-      <c r="R3" s="32"/>
-      <c r="T3" s="33" t="s">
+      <c r="O3" s="31"/>
+      <c r="P3" s="31"/>
+      <c r="Q3" s="31"/>
+      <c r="R3" s="31"/>
+      <c r="T3" s="32" t="s">
         <v>79</v>
       </c>
-      <c r="U3" s="33"/>
-      <c r="V3" s="33"/>
-      <c r="W3" s="33"/>
-      <c r="X3" s="33"/>
+      <c r="U3" s="32"/>
+      <c r="V3" s="32"/>
+      <c r="W3" s="32"/>
+      <c r="X3" s="32"/>
       <c r="Y3" s="28"/>
-      <c r="Z3" s="32" t="s">
+      <c r="Z3" s="31" t="s">
         <v>80</v>
       </c>
-      <c r="AA3" s="32"/>
-      <c r="AB3" s="32"/>
-      <c r="AC3" s="32"/>
-      <c r="AD3" s="32"/>
+      <c r="AA3" s="31"/>
+      <c r="AB3" s="31"/>
+      <c r="AC3" s="31"/>
+      <c r="AD3" s="31"/>
       <c r="AE3" s="28"/>
-      <c r="AF3" s="32" t="s">
+      <c r="AF3" s="31" t="s">
         <v>81</v>
       </c>
-      <c r="AG3" s="32"/>
-      <c r="AH3" s="32"/>
-      <c r="AI3" s="32"/>
-      <c r="AJ3" s="32"/>
-    </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.2">
+      <c r="AG3" s="31"/>
+      <c r="AH3" s="31"/>
+      <c r="AI3" s="31"/>
+      <c r="AJ3" s="31"/>
+    </row>
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="15"/>
       <c r="B4" s="29" t="s">
         <v>90</v>
@@ -4988,7 +5096,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="17" t="s">
         <v>85</v>
       </c>
@@ -5027,15 +5135,25 @@
       <c r="AI5" s="16"/>
       <c r="AJ5" s="16"/>
     </row>
-    <row r="6" spans="1:36" ht="17" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="16" t="s">
         <v>96</v>
       </c>
-      <c r="B6" s="16"/>
-      <c r="C6" s="16"/>
-      <c r="D6" s="18"/>
-      <c r="E6" s="16"/>
-      <c r="F6" s="16"/>
+      <c r="B6" s="16">
+        <v>13.944000000000001</v>
+      </c>
+      <c r="C6" s="16">
+        <v>0.247</v>
+      </c>
+      <c r="D6" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="E6" s="16">
+        <v>13.538</v>
+      </c>
+      <c r="F6" s="16">
+        <v>14.35</v>
+      </c>
       <c r="G6" s="16"/>
       <c r="H6" s="16"/>
       <c r="I6" s="16"/>
@@ -5057,30 +5175,64 @@
       <c r="V6" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="W6" s="16"/>
-      <c r="X6" s="16"/>
+      <c r="W6" s="16">
+        <v>13.037000000000001</v>
+      </c>
+      <c r="X6" s="16">
+        <v>13.746</v>
+      </c>
       <c r="Y6" s="16"/>
-      <c r="Z6" s="16"/>
-      <c r="AA6" s="16"/>
-      <c r="AB6" s="18"/>
-      <c r="AC6" s="16"/>
-      <c r="AD6" s="16"/>
+      <c r="Z6" s="16">
+        <v>13.525</v>
+      </c>
+      <c r="AA6" s="16">
+        <v>0.21299999999999999</v>
+      </c>
+      <c r="AB6" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="AC6" s="16">
+        <v>13.173999999999999</v>
+      </c>
+      <c r="AD6" s="16">
+        <v>13.875999999999999</v>
+      </c>
       <c r="AE6" s="16"/>
-      <c r="AF6" s="16"/>
-      <c r="AG6" s="16"/>
-      <c r="AH6" s="18"/>
-      <c r="AI6" s="16"/>
-      <c r="AJ6" s="16"/>
-    </row>
-    <row r="7" spans="1:36" ht="17" x14ac:dyDescent="0.25">
+      <c r="AF6" s="16">
+        <v>13.525</v>
+      </c>
+      <c r="AG6" s="16">
+        <v>0.21299999999999999</v>
+      </c>
+      <c r="AH6" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="AI6" s="16">
+        <v>13.173999999999999</v>
+      </c>
+      <c r="AJ6" s="16">
+        <v>13.875999999999999</v>
+      </c>
+    </row>
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="16" t="s">
         <v>97</v>
       </c>
-      <c r="B7" s="16"/>
-      <c r="C7" s="16"/>
-      <c r="D7" s="18"/>
-      <c r="E7" s="16"/>
-      <c r="F7" s="16"/>
+      <c r="B7" s="16">
+        <v>-7.5229999999999997</v>
+      </c>
+      <c r="C7" s="16">
+        <v>0.48599999999999999</v>
+      </c>
+      <c r="D7" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="E7" s="16">
+        <v>-8.3209999999999997</v>
+      </c>
+      <c r="F7" s="16">
+        <v>-6.7240000000000002</v>
+      </c>
       <c r="G7" s="16"/>
       <c r="H7" s="16"/>
       <c r="I7" s="16"/>
@@ -5102,196 +5254,288 @@
       <c r="V7" s="18">
         <v>2.1999999999999999E-2</v>
       </c>
-      <c r="W7" s="16"/>
-      <c r="X7" s="16"/>
+      <c r="W7" s="16">
+        <v>0.34300000000000003</v>
+      </c>
+      <c r="X7" s="16">
+        <v>2.1</v>
+      </c>
       <c r="Y7" s="16"/>
-      <c r="Z7" s="16"/>
-      <c r="AA7" s="16"/>
-      <c r="AB7" s="18"/>
-      <c r="AC7" s="16"/>
-      <c r="AD7" s="16"/>
+      <c r="Z7" s="16">
+        <v>1.236</v>
+      </c>
+      <c r="AA7" s="16">
+        <v>0.53800000000000003</v>
+      </c>
+      <c r="AB7" s="16">
+        <v>2.1999999999999999E-2</v>
+      </c>
+      <c r="AC7" s="16">
+        <v>0.35099999999999998</v>
+      </c>
+      <c r="AD7" s="16">
+        <v>2.121</v>
+      </c>
       <c r="AE7" s="16"/>
-      <c r="AF7" s="16"/>
-      <c r="AG7" s="16"/>
-      <c r="AH7" s="18"/>
-      <c r="AI7" s="16"/>
-      <c r="AJ7" s="16"/>
-    </row>
-    <row r="8" spans="1:36" x14ac:dyDescent="0.2">
-      <c r="A8" s="16"/>
-      <c r="B8" s="16"/>
-      <c r="C8" s="16"/>
-      <c r="D8" s="18"/>
-      <c r="E8" s="18"/>
-      <c r="F8" s="21"/>
-      <c r="G8" s="21"/>
+      <c r="AF7" s="16">
+        <v>1.2370000000000001</v>
+      </c>
+      <c r="AG7" s="16">
+        <v>0.53800000000000003</v>
+      </c>
+      <c r="AH7" s="16">
+        <v>2.1000000000000001E-2</v>
+      </c>
+      <c r="AI7" s="16">
+        <v>0.35199999999999998</v>
+      </c>
+      <c r="AJ7" s="16">
+        <v>2.1219999999999999</v>
+      </c>
+    </row>
+    <row r="8" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A8" s="16" t="s">
+        <v>140</v>
+      </c>
+      <c r="B8" s="16">
+        <v>-0.253</v>
+      </c>
+      <c r="C8" s="16">
+        <v>1.236</v>
+      </c>
+      <c r="D8" s="18">
+        <v>0.83699999999999997</v>
+      </c>
+      <c r="E8" s="16">
+        <v>-2.286</v>
+      </c>
+      <c r="F8" s="16">
+        <v>1.7789999999999999</v>
+      </c>
+      <c r="G8" s="16"/>
       <c r="H8" s="16"/>
       <c r="I8" s="16"/>
       <c r="J8" s="18"/>
-      <c r="K8" s="18"/>
+      <c r="K8" s="16"/>
       <c r="L8" s="16"/>
       <c r="M8" s="16"/>
       <c r="N8" s="16"/>
       <c r="O8" s="16"/>
       <c r="P8" s="18"/>
-      <c r="Q8" s="18"/>
+      <c r="Q8" s="16"/>
       <c r="R8" s="16"/>
       <c r="T8" s="16"/>
       <c r="U8" s="16"/>
       <c r="V8" s="18"/>
-      <c r="W8" s="18"/>
-      <c r="X8" s="21"/>
-      <c r="Y8" s="21"/>
+      <c r="W8" s="16"/>
+      <c r="X8" s="16"/>
+      <c r="Y8" s="16"/>
       <c r="Z8" s="16"/>
       <c r="AA8" s="16"/>
-      <c r="AB8" s="18"/>
-      <c r="AC8" s="18"/>
+      <c r="AB8" s="16"/>
+      <c r="AC8" s="16"/>
       <c r="AD8" s="16"/>
       <c r="AE8" s="16"/>
       <c r="AF8" s="16"/>
       <c r="AG8" s="16"/>
-      <c r="AH8" s="18"/>
-      <c r="AI8" s="18"/>
+      <c r="AH8" s="16"/>
+      <c r="AI8" s="16"/>
       <c r="AJ8" s="16"/>
     </row>
-    <row r="9" spans="1:36" x14ac:dyDescent="0.2">
-      <c r="A9" s="17" t="s">
-        <v>86</v>
-      </c>
+    <row r="9" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A9" s="16"/>
       <c r="B9" s="16"/>
       <c r="C9" s="16"/>
-      <c r="D9" s="16"/>
-      <c r="E9" s="16"/>
+      <c r="D9" s="18"/>
+      <c r="E9" s="18"/>
       <c r="F9" s="21"/>
       <c r="G9" s="21"/>
       <c r="H9" s="16"/>
       <c r="I9" s="16"/>
-      <c r="J9" s="16"/>
-      <c r="K9" s="16"/>
+      <c r="J9" s="18"/>
+      <c r="K9" s="18"/>
       <c r="L9" s="16"/>
       <c r="M9" s="16"/>
       <c r="N9" s="16"/>
       <c r="O9" s="16"/>
-      <c r="P9" s="16"/>
-      <c r="Q9" s="16"/>
+      <c r="P9" s="18"/>
+      <c r="Q9" s="18"/>
       <c r="R9" s="16"/>
       <c r="T9" s="16"/>
       <c r="U9" s="16"/>
-      <c r="V9" s="16"/>
-      <c r="W9" s="16"/>
+      <c r="V9" s="18"/>
+      <c r="W9" s="18"/>
       <c r="X9" s="21"/>
       <c r="Y9" s="21"/>
       <c r="Z9" s="16"/>
       <c r="AA9" s="16"/>
-      <c r="AB9" s="16"/>
-      <c r="AC9" s="16"/>
+      <c r="AB9" s="18"/>
+      <c r="AC9" s="18"/>
       <c r="AD9" s="16"/>
       <c r="AE9" s="16"/>
       <c r="AF9" s="16"/>
       <c r="AG9" s="16"/>
-      <c r="AH9" s="16"/>
-      <c r="AI9" s="16"/>
+      <c r="AH9" s="18"/>
+      <c r="AI9" s="18"/>
       <c r="AJ9" s="16"/>
     </row>
-    <row r="10" spans="1:36" ht="17" x14ac:dyDescent="0.25">
-      <c r="A10" s="16" t="s">
-        <v>98</v>
+    <row r="10" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A10" s="17" t="s">
+        <v>86</v>
       </c>
       <c r="B10" s="16"/>
       <c r="C10" s="16"/>
-      <c r="D10" s="18"/>
+      <c r="D10" s="16"/>
       <c r="E10" s="16"/>
-      <c r="F10" s="16"/>
-      <c r="G10" s="16"/>
+      <c r="F10" s="21"/>
+      <c r="G10" s="21"/>
       <c r="H10" s="16"/>
       <c r="I10" s="16"/>
-      <c r="J10" s="18"/>
+      <c r="J10" s="16"/>
       <c r="K10" s="16"/>
       <c r="L10" s="16"/>
       <c r="M10" s="16"/>
       <c r="N10" s="16"/>
       <c r="O10" s="16"/>
-      <c r="P10" s="18"/>
+      <c r="P10" s="16"/>
       <c r="Q10" s="16"/>
       <c r="R10" s="16"/>
-      <c r="T10" s="16">
-        <v>0.318</v>
-      </c>
-      <c r="U10" s="16">
-        <v>0.05</v>
-      </c>
-      <c r="V10" s="18" t="s">
-        <v>24</v>
-      </c>
+      <c r="T10" s="16"/>
+      <c r="U10" s="16"/>
+      <c r="V10" s="16"/>
       <c r="W10" s="16"/>
-      <c r="X10" s="16"/>
-      <c r="Y10" s="16"/>
+      <c r="X10" s="21"/>
+      <c r="Y10" s="21"/>
       <c r="Z10" s="16"/>
       <c r="AA10" s="16"/>
-      <c r="AB10" s="18"/>
+      <c r="AB10" s="16"/>
       <c r="AC10" s="16"/>
       <c r="AD10" s="16"/>
       <c r="AE10" s="16"/>
       <c r="AF10" s="16"/>
       <c r="AG10" s="16"/>
-      <c r="AH10" s="18"/>
+      <c r="AH10" s="16"/>
       <c r="AI10" s="16"/>
       <c r="AJ10" s="16"/>
     </row>
-    <row r="11" spans="1:36" ht="17" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A11" s="16" t="s">
-        <v>99</v>
-      </c>
-      <c r="B11" s="16"/>
-      <c r="C11" s="16"/>
-      <c r="D11" s="18"/>
-      <c r="E11" s="16"/>
-      <c r="F11" s="16"/>
+        <v>98</v>
+      </c>
+      <c r="B11" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="C11" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="D11" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="E11" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="F11" s="21" t="s">
+        <v>94</v>
+      </c>
       <c r="G11" s="16"/>
-      <c r="H11" s="16"/>
-      <c r="I11" s="16"/>
-      <c r="J11" s="18"/>
-      <c r="K11" s="16"/>
-      <c r="L11" s="16"/>
+      <c r="H11" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="I11" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="J11" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="K11" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="L11" s="21" t="s">
+        <v>94</v>
+      </c>
       <c r="M11" s="16"/>
-      <c r="N11" s="16"/>
-      <c r="O11" s="16"/>
-      <c r="P11" s="18"/>
-      <c r="Q11" s="16"/>
-      <c r="R11" s="16"/>
+      <c r="N11" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="O11" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="P11" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="Q11" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="R11" s="21" t="s">
+        <v>94</v>
+      </c>
       <c r="T11" s="16">
-        <v>-0.01</v>
+        <v>0.318</v>
       </c>
       <c r="U11" s="16">
+        <v>0.05</v>
+      </c>
+      <c r="V11" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="W11" s="16">
+        <v>0.23599999999999999</v>
+      </c>
+      <c r="X11" s="16">
+        <v>0.40100000000000002</v>
+      </c>
+      <c r="Y11" s="16"/>
+      <c r="Z11" s="16">
+        <v>0.32</v>
+      </c>
+      <c r="AA11" s="16">
+        <v>0.05</v>
+      </c>
+      <c r="AB11" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="AC11" s="16">
+        <v>0.23699999999999999</v>
+      </c>
+      <c r="AD11" s="16">
+        <v>0.40300000000000002</v>
+      </c>
+      <c r="AE11" s="16"/>
+      <c r="AF11" s="16">
+        <v>0.32</v>
+      </c>
+      <c r="AG11" s="16">
+        <v>0.05</v>
+      </c>
+      <c r="AH11" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="AI11" s="16">
+        <v>0.23699999999999999</v>
+      </c>
+      <c r="AJ11" s="16">
+        <v>0.40300000000000002</v>
+      </c>
+    </row>
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A12" s="16" t="s">
+        <v>139</v>
+      </c>
+      <c r="B12" s="16">
+        <v>0.11700000000000001</v>
+      </c>
+      <c r="C12" s="16">
+        <v>5.8000000000000003E-2</v>
+      </c>
+      <c r="D12" s="16">
+        <v>4.4999999999999998E-2</v>
+      </c>
+      <c r="E12" s="16">
         <v>2.1000000000000001E-2</v>
       </c>
-      <c r="V11" s="18">
-        <v>0.63500000000000001</v>
-      </c>
-      <c r="W11" s="16"/>
-      <c r="X11" s="16"/>
-      <c r="Y11" s="16"/>
-      <c r="Z11" s="16"/>
-      <c r="AA11" s="16"/>
-      <c r="AB11" s="18"/>
-      <c r="AC11" s="16"/>
-      <c r="AD11" s="16"/>
-      <c r="AE11" s="16"/>
-      <c r="AF11" s="16"/>
-      <c r="AG11" s="16"/>
-      <c r="AH11" s="18"/>
-      <c r="AI11" s="16"/>
-      <c r="AJ11" s="16"/>
-    </row>
-    <row r="12" spans="1:36" ht="17" x14ac:dyDescent="0.25">
-      <c r="A12" s="16" t="s">
-        <v>100</v>
-      </c>
-      <c r="B12" s="16"/>
-      <c r="C12" s="16"/>
-      <c r="D12" s="18"/>
-      <c r="E12" s="16"/>
-      <c r="F12" s="16"/>
+      <c r="F12" s="16">
+        <v>0.21299999999999999</v>
+      </c>
       <c r="G12" s="16"/>
       <c r="H12" s="16"/>
       <c r="I12" s="16"/>
@@ -5304,15 +5548,9 @@
       <c r="P12" s="18"/>
       <c r="Q12" s="16"/>
       <c r="R12" s="16"/>
-      <c r="T12" s="16">
-        <v>7.0999999999999994E-2</v>
-      </c>
-      <c r="U12" s="16">
-        <v>2.1000000000000001E-2</v>
-      </c>
-      <c r="V12" s="18">
-        <v>1E-3</v>
-      </c>
+      <c r="T12" s="16"/>
+      <c r="U12" s="16"/>
+      <c r="V12" s="18"/>
       <c r="W12" s="16"/>
       <c r="X12" s="16"/>
       <c r="Y12" s="16"/>
@@ -5328,15 +5566,25 @@
       <c r="AI12" s="16"/>
       <c r="AJ12" s="16"/>
     </row>
-    <row r="13" spans="1:36" ht="17" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="16" t="s">
-        <v>101</v>
-      </c>
-      <c r="B13" s="16"/>
-      <c r="C13" s="16"/>
-      <c r="D13" s="16"/>
-      <c r="E13" s="16"/>
-      <c r="F13" s="16"/>
+        <v>99</v>
+      </c>
+      <c r="B13" s="16">
+        <v>0.02</v>
+      </c>
+      <c r="C13" s="16">
+        <v>2.1999999999999999E-2</v>
+      </c>
+      <c r="D13" s="16">
+        <v>0.35199999999999998</v>
+      </c>
+      <c r="E13" s="16">
+        <v>-1.4999999999999999E-2</v>
+      </c>
+      <c r="F13" s="16">
+        <v>5.6000000000000001E-2</v>
+      </c>
       <c r="G13" s="16"/>
       <c r="H13" s="16"/>
       <c r="I13" s="16"/>
@@ -5350,38 +5598,72 @@
       <c r="Q13" s="16"/>
       <c r="R13" s="16"/>
       <c r="T13" s="16">
-        <v>0.16800000000000001</v>
+        <v>-0.01</v>
       </c>
       <c r="U13" s="16">
-        <v>3.5999999999999997E-2</v>
-      </c>
-      <c r="V13" s="18" t="s">
-        <v>24</v>
-      </c>
-      <c r="W13" s="16"/>
-      <c r="X13" s="16"/>
+        <v>2.1000000000000001E-2</v>
+      </c>
+      <c r="V13" s="18">
+        <v>0.63500000000000001</v>
+      </c>
+      <c r="W13" s="16">
+        <v>-4.4999999999999998E-2</v>
+      </c>
+      <c r="X13" s="16">
+        <v>2.5000000000000001E-2</v>
+      </c>
       <c r="Y13" s="16"/>
-      <c r="Z13" s="16"/>
-      <c r="AA13" s="16"/>
-      <c r="AB13" s="16"/>
-      <c r="AC13" s="16"/>
-      <c r="AD13" s="16"/>
+      <c r="Z13" s="16">
+        <v>-0.01</v>
+      </c>
+      <c r="AA13" s="16">
+        <v>2.1000000000000001E-2</v>
+      </c>
+      <c r="AB13" s="16">
+        <v>0.625</v>
+      </c>
+      <c r="AC13" s="16">
+        <v>-4.4999999999999998E-2</v>
+      </c>
+      <c r="AD13" s="16">
+        <v>2.4E-2</v>
+      </c>
       <c r="AE13" s="16"/>
-      <c r="AF13" s="16"/>
-      <c r="AG13" s="16"/>
-      <c r="AH13" s="18"/>
-      <c r="AI13" s="16"/>
-      <c r="AJ13" s="16"/>
-    </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.2">
+      <c r="AF13" s="16">
+        <v>-0.01</v>
+      </c>
+      <c r="AG13" s="16">
+        <v>2.1000000000000001E-2</v>
+      </c>
+      <c r="AH13" s="16">
+        <v>0.621</v>
+      </c>
+      <c r="AI13" s="16">
+        <v>-4.4999999999999998E-2</v>
+      </c>
+      <c r="AJ13" s="16">
+        <v>2.4E-2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A14" s="16" t="s">
-        <v>88</v>
-      </c>
-      <c r="B14" s="16"/>
-      <c r="C14" s="16"/>
-      <c r="D14" s="18"/>
-      <c r="E14" s="16"/>
-      <c r="F14" s="16"/>
+        <v>100</v>
+      </c>
+      <c r="B14" s="16">
+        <v>6.9000000000000006E-2</v>
+      </c>
+      <c r="C14" s="16">
+        <v>2.3E-2</v>
+      </c>
+      <c r="D14" s="16">
+        <v>3.0000000000000001E-3</v>
+      </c>
+      <c r="E14" s="16">
+        <v>3.1E-2</v>
+      </c>
+      <c r="F14" s="16">
+        <v>0.106</v>
+      </c>
       <c r="G14" s="16"/>
       <c r="H14" s="16"/>
       <c r="I14" s="16"/>
@@ -5395,114 +5677,220 @@
       <c r="Q14" s="16"/>
       <c r="R14" s="16"/>
       <c r="T14" s="16">
-        <v>0.248</v>
+        <v>7.0999999999999994E-2</v>
       </c>
       <c r="U14" s="16">
-        <v>2.1999999999999999E-2</v>
-      </c>
-      <c r="V14" s="18" t="s">
-        <v>24</v>
-      </c>
-      <c r="W14" s="16"/>
-      <c r="X14" s="16"/>
+        <v>2.1000000000000001E-2</v>
+      </c>
+      <c r="V14" s="18">
+        <v>1E-3</v>
+      </c>
+      <c r="W14" s="16">
+        <v>3.6999999999999998E-2</v>
+      </c>
+      <c r="X14" s="16">
+        <v>0.106</v>
+      </c>
       <c r="Y14" s="16"/>
-      <c r="Z14" s="16"/>
-      <c r="AA14" s="16"/>
-      <c r="AB14" s="18"/>
-      <c r="AC14" s="16"/>
-      <c r="AD14" s="16"/>
+      <c r="Z14" s="16">
+        <v>5.0999999999999997E-2</v>
+      </c>
+      <c r="AA14" s="16">
+        <v>2.1000000000000001E-2</v>
+      </c>
+      <c r="AB14" s="16">
+        <v>1.7000000000000001E-2</v>
+      </c>
+      <c r="AC14" s="16">
+        <v>1.6E-2</v>
+      </c>
+      <c r="AD14" s="16">
+        <v>8.5999999999999993E-2</v>
+      </c>
       <c r="AE14" s="16"/>
-      <c r="AF14" s="16"/>
-      <c r="AG14" s="16"/>
-      <c r="AH14" s="18"/>
-      <c r="AI14" s="16"/>
-      <c r="AJ14" s="16"/>
-    </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.2">
-      <c r="A15" s="16"/>
-      <c r="B15" s="16"/>
-      <c r="C15" s="16"/>
-      <c r="D15" s="18"/>
-      <c r="E15" s="18"/>
-      <c r="F15" s="21"/>
+      <c r="AF14" s="16">
+        <v>5.0999999999999997E-2</v>
+      </c>
+      <c r="AG14" s="16">
+        <v>2.1000000000000001E-2</v>
+      </c>
+      <c r="AH14" s="16">
+        <v>1.7000000000000001E-2</v>
+      </c>
+      <c r="AI14" s="16">
+        <v>1.6E-2</v>
+      </c>
+      <c r="AJ14" s="16">
+        <v>8.5999999999999993E-2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A15" s="16" t="s">
+        <v>141</v>
+      </c>
+      <c r="B15" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="C15" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="D15" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="E15" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="F15" s="21" t="s">
+        <v>94</v>
+      </c>
       <c r="G15" s="21"/>
-      <c r="H15" s="16"/>
-      <c r="I15" s="16"/>
-      <c r="J15" s="18"/>
-      <c r="K15" s="18"/>
-      <c r="L15" s="16"/>
+      <c r="H15" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="I15" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="J15" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="K15" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="L15" s="21" t="s">
+        <v>94</v>
+      </c>
       <c r="M15" s="16"/>
-      <c r="N15" s="16"/>
-      <c r="O15" s="16"/>
-      <c r="P15" s="18"/>
-      <c r="Q15" s="18"/>
-      <c r="R15" s="16"/>
+      <c r="N15" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="O15" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="P15" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="Q15" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="R15" s="21" t="s">
+        <v>94</v>
+      </c>
       <c r="T15" s="16"/>
       <c r="U15" s="16"/>
       <c r="V15" s="18"/>
-      <c r="W15" s="18"/>
-      <c r="X15" s="21"/>
-      <c r="Y15" s="21"/>
+      <c r="W15" s="16"/>
+      <c r="X15" s="16"/>
+      <c r="Y15" s="16"/>
       <c r="Z15" s="16"/>
       <c r="AA15" s="16"/>
-      <c r="AB15" s="18"/>
-      <c r="AC15" s="18"/>
+      <c r="AB15" s="16"/>
+      <c r="AC15" s="16"/>
       <c r="AD15" s="16"/>
       <c r="AE15" s="16"/>
       <c r="AF15" s="16"/>
       <c r="AG15" s="16"/>
-      <c r="AH15" s="18"/>
-      <c r="AI15" s="18"/>
+      <c r="AH15" s="16"/>
+      <c r="AI15" s="16"/>
       <c r="AJ15" s="16"/>
     </row>
-    <row r="16" spans="1:36" x14ac:dyDescent="0.2">
-      <c r="A16" s="17" t="s">
-        <v>87</v>
-      </c>
-      <c r="B16" s="16"/>
-      <c r="C16" s="16"/>
-      <c r="D16" s="16"/>
-      <c r="E16" s="16"/>
-      <c r="F16" s="21"/>
-      <c r="G16" s="21"/>
+    <row r="16" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A16" s="16" t="s">
+        <v>101</v>
+      </c>
+      <c r="B16" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="C16" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="D16" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="E16" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="F16" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="G16" s="16"/>
       <c r="H16" s="16"/>
       <c r="I16" s="16"/>
-      <c r="J16" s="16"/>
+      <c r="J16" s="18"/>
       <c r="K16" s="16"/>
       <c r="L16" s="16"/>
       <c r="M16" s="16"/>
       <c r="N16" s="16"/>
       <c r="O16" s="16"/>
-      <c r="P16" s="16"/>
+      <c r="P16" s="18"/>
       <c r="Q16" s="16"/>
       <c r="R16" s="16"/>
-      <c r="T16" s="16"/>
-      <c r="U16" s="16"/>
-      <c r="V16" s="16"/>
-      <c r="W16" s="16"/>
-      <c r="X16" s="21"/>
-      <c r="Y16" s="21"/>
-      <c r="Z16" s="16"/>
-      <c r="AA16" s="16"/>
-      <c r="AB16" s="16"/>
-      <c r="AC16" s="16"/>
-      <c r="AD16" s="16"/>
+      <c r="T16" s="16">
+        <v>0.16800000000000001</v>
+      </c>
+      <c r="U16" s="16">
+        <v>3.5999999999999997E-2</v>
+      </c>
+      <c r="V16" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="W16" s="16">
+        <v>0.108</v>
+      </c>
+      <c r="X16" s="16">
+        <v>0.22800000000000001</v>
+      </c>
+      <c r="Y16" s="16"/>
+      <c r="Z16" s="16">
+        <v>0.16800000000000001</v>
+      </c>
+      <c r="AA16" s="16">
+        <v>3.6999999999999998E-2</v>
+      </c>
+      <c r="AB16" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="AC16" s="16">
+        <v>0.108</v>
+      </c>
+      <c r="AD16" s="16">
+        <v>0.22900000000000001</v>
+      </c>
       <c r="AE16" s="16"/>
-      <c r="AF16" s="16"/>
-      <c r="AG16" s="16"/>
-      <c r="AH16" s="16"/>
-      <c r="AI16" s="16"/>
-      <c r="AJ16" s="16"/>
-    </row>
-    <row r="17" spans="1:36" ht="17" x14ac:dyDescent="0.25">
+      <c r="AF16" s="16">
+        <v>0.16900000000000001</v>
+      </c>
+      <c r="AG16" s="16">
+        <v>3.5999999999999997E-2</v>
+      </c>
+      <c r="AH16" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="AI16" s="16">
+        <v>0.109</v>
+      </c>
+      <c r="AJ16" s="16">
+        <v>0.22900000000000001</v>
+      </c>
+    </row>
+    <row r="17" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A17" s="16" t="s">
-        <v>102</v>
-      </c>
-      <c r="B17" s="16"/>
-      <c r="C17" s="16"/>
-      <c r="D17" s="18"/>
-      <c r="E17" s="16"/>
-      <c r="F17" s="16"/>
+        <v>142</v>
+      </c>
+      <c r="B17" s="16">
+        <v>-0.45300000000000001</v>
+      </c>
+      <c r="C17" s="16">
+        <v>0.13900000000000001</v>
+      </c>
+      <c r="D17" s="16">
+        <v>1E-3</v>
+      </c>
+      <c r="E17" s="16">
+        <v>-0.68100000000000005</v>
+      </c>
+      <c r="F17" s="16">
+        <v>-0.22500000000000001</v>
+      </c>
       <c r="G17" s="16"/>
       <c r="H17" s="16"/>
       <c r="I17" s="16"/>
@@ -5515,15 +5903,9 @@
       <c r="P17" s="18"/>
       <c r="Q17" s="16"/>
       <c r="R17" s="16"/>
-      <c r="T17" s="16">
-        <v>8.5000000000000006E-2</v>
-      </c>
-      <c r="U17" s="16">
-        <v>3.6999999999999998E-2</v>
-      </c>
-      <c r="V17" s="18">
-        <v>2.1000000000000001E-2</v>
-      </c>
+      <c r="T17" s="16"/>
+      <c r="U17" s="16"/>
+      <c r="V17" s="18"/>
       <c r="W17" s="16"/>
       <c r="X17" s="16"/>
       <c r="Y17" s="16"/>
@@ -5539,26 +5921,26 @@
       <c r="AI17" s="16"/>
       <c r="AJ17" s="16"/>
     </row>
-    <row r="18" spans="1:36" ht="17" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A18" s="16" t="s">
-        <v>103</v>
-      </c>
-      <c r="B18" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="C18" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="D18" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="E18" s="21" t="s">
-        <v>94</v>
-      </c>
-      <c r="F18" s="21" t="s">
-        <v>94</v>
-      </c>
-      <c r="G18" s="21"/>
+        <v>88</v>
+      </c>
+      <c r="B18" s="16">
+        <v>0.318</v>
+      </c>
+      <c r="C18" s="16">
+        <v>0.02</v>
+      </c>
+      <c r="D18" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="E18" s="16">
+        <v>0.28499999999999998</v>
+      </c>
+      <c r="F18" s="16">
+        <v>0.35099999999999998</v>
+      </c>
+      <c r="G18" s="16"/>
       <c r="H18" s="16"/>
       <c r="I18" s="16"/>
       <c r="J18" s="18"/>
@@ -5570,143 +5952,121 @@
       <c r="P18" s="18"/>
       <c r="Q18" s="16"/>
       <c r="R18" s="16"/>
-      <c r="T18" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="U18" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="V18" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="W18" s="21" t="s">
-        <v>94</v>
-      </c>
-      <c r="X18" s="21" t="s">
-        <v>94</v>
-      </c>
-      <c r="Y18" s="21"/>
-      <c r="Z18" s="16"/>
-      <c r="AA18" s="16"/>
-      <c r="AB18" s="18"/>
-      <c r="AC18" s="16"/>
-      <c r="AD18" s="16"/>
+      <c r="T18" s="16">
+        <v>0.248</v>
+      </c>
+      <c r="U18" s="16">
+        <v>2.1999999999999999E-2</v>
+      </c>
+      <c r="V18" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="W18" s="16">
+        <v>0.21199999999999999</v>
+      </c>
+      <c r="X18" s="16">
+        <v>0.28399999999999997</v>
+      </c>
+      <c r="Y18" s="16"/>
+      <c r="Z18" s="16">
+        <v>0.252</v>
+      </c>
+      <c r="AA18" s="16">
+        <v>2.1999999999999999E-2</v>
+      </c>
+      <c r="AB18" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="AC18" s="16">
+        <v>0.216</v>
+      </c>
+      <c r="AD18" s="16">
+        <v>0.28799999999999998</v>
+      </c>
       <c r="AE18" s="16"/>
-      <c r="AF18" s="16"/>
-      <c r="AG18" s="16"/>
-      <c r="AH18" s="18"/>
-      <c r="AI18" s="16"/>
-      <c r="AJ18" s="16"/>
-    </row>
-    <row r="19" spans="1:36" ht="17" x14ac:dyDescent="0.25">
-      <c r="A19" s="16" t="s">
-        <v>104</v>
-      </c>
-      <c r="B19" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="C19" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="D19" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="E19" s="21" t="s">
-        <v>94</v>
-      </c>
-      <c r="F19" s="21" t="s">
-        <v>94</v>
-      </c>
+      <c r="AF18" s="16">
+        <v>0.252</v>
+      </c>
+      <c r="AG18" s="16">
+        <v>2.1999999999999999E-2</v>
+      </c>
+      <c r="AH18" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="AI18" s="16">
+        <v>0.216</v>
+      </c>
+      <c r="AJ18" s="16">
+        <v>0.28799999999999998</v>
+      </c>
+    </row>
+    <row r="19" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A19" s="16"/>
+      <c r="B19" s="16"/>
+      <c r="C19" s="16"/>
+      <c r="D19" s="18"/>
+      <c r="E19" s="18"/>
+      <c r="F19" s="21"/>
       <c r="G19" s="21"/>
-      <c r="H19" s="22"/>
-      <c r="I19" s="22"/>
-      <c r="J19" s="16"/>
-      <c r="K19" s="16"/>
+      <c r="H19" s="16"/>
+      <c r="I19" s="16"/>
+      <c r="J19" s="18"/>
+      <c r="K19" s="18"/>
       <c r="L19" s="16"/>
       <c r="M19" s="16"/>
       <c r="N19" s="16"/>
       <c r="O19" s="16"/>
       <c r="P19" s="18"/>
-      <c r="Q19" s="16"/>
+      <c r="Q19" s="18"/>
       <c r="R19" s="16"/>
-      <c r="T19" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="U19" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="V19" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="W19" s="21" t="s">
-        <v>94</v>
-      </c>
-      <c r="X19" s="21" t="s">
-        <v>94</v>
-      </c>
+      <c r="T19" s="16"/>
+      <c r="U19" s="16"/>
+      <c r="V19" s="18"/>
+      <c r="W19" s="18"/>
+      <c r="X19" s="21"/>
       <c r="Y19" s="21"/>
       <c r="Z19" s="16"/>
       <c r="AA19" s="16"/>
-      <c r="AB19" s="16"/>
-      <c r="AC19" s="16"/>
+      <c r="AB19" s="18"/>
+      <c r="AC19" s="18"/>
       <c r="AD19" s="16"/>
       <c r="AE19" s="16"/>
       <c r="AF19" s="16"/>
       <c r="AG19" s="16"/>
-      <c r="AH19" s="16"/>
-      <c r="AI19" s="16"/>
-      <c r="AJ19" s="30"/>
-    </row>
-    <row r="20" spans="1:36" x14ac:dyDescent="0.2">
-      <c r="A20" s="16" t="s">
-        <v>107</v>
-      </c>
-      <c r="B20" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="C20" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="D20" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="E20" s="21" t="s">
-        <v>94</v>
-      </c>
-      <c r="F20" s="21" t="s">
-        <v>94</v>
-      </c>
+      <c r="AH19" s="18"/>
+      <c r="AI19" s="18"/>
+      <c r="AJ19" s="16"/>
+    </row>
+    <row r="20" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A20" s="17" t="s">
+        <v>87</v>
+      </c>
+      <c r="B20" s="16"/>
+      <c r="C20" s="16"/>
+      <c r="D20" s="16"/>
+      <c r="E20" s="16"/>
+      <c r="F20" s="21"/>
       <c r="G20" s="21"/>
       <c r="H20" s="16"/>
       <c r="I20" s="16"/>
-      <c r="J20" s="18"/>
+      <c r="J20" s="16"/>
       <c r="K20" s="16"/>
       <c r="L20" s="16"/>
       <c r="M20" s="16"/>
       <c r="N20" s="16"/>
       <c r="O20" s="16"/>
-      <c r="P20" s="18"/>
+      <c r="P20" s="16"/>
       <c r="Q20" s="16"/>
       <c r="R20" s="16"/>
-      <c r="T20" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="U20" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="V20" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="W20" s="21" t="s">
-        <v>94</v>
-      </c>
-      <c r="X20" s="21" t="s">
-        <v>94</v>
-      </c>
+      <c r="T20" s="16"/>
+      <c r="U20" s="16"/>
+      <c r="V20" s="16"/>
+      <c r="W20" s="16"/>
+      <c r="X20" s="21"/>
       <c r="Y20" s="21"/>
       <c r="Z20" s="16"/>
       <c r="AA20" s="16"/>
-      <c r="AB20" s="18"/>
+      <c r="AB20" s="16"/>
       <c r="AC20" s="16"/>
       <c r="AD20" s="16"/>
       <c r="AE20" s="16"/>
@@ -5716,52 +6076,42 @@
       <c r="AI20" s="16"/>
       <c r="AJ20" s="16"/>
     </row>
-    <row r="21" spans="1:36" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A21" s="16" t="s">
-        <v>108</v>
-      </c>
-      <c r="B21" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="C21" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="D21" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="E21" s="21" t="s">
-        <v>94</v>
-      </c>
-      <c r="F21" s="21" t="s">
-        <v>94</v>
+        <v>138</v>
+      </c>
+      <c r="B21" s="16">
+        <v>-0.29099999999999998</v>
+      </c>
+      <c r="C21" s="16">
+        <v>0.106</v>
+      </c>
+      <c r="D21" s="16">
+        <v>6.0000000000000001E-3</v>
+      </c>
+      <c r="E21" s="16">
+        <v>-0.46500000000000002</v>
+      </c>
+      <c r="F21" s="16">
+        <v>-0.11700000000000001</v>
       </c>
       <c r="G21" s="21"/>
       <c r="H21" s="16"/>
       <c r="I21" s="16"/>
-      <c r="J21" s="18"/>
+      <c r="J21" s="16"/>
       <c r="K21" s="16"/>
       <c r="L21" s="16"/>
       <c r="M21" s="16"/>
       <c r="N21" s="16"/>
       <c r="O21" s="16"/>
-      <c r="P21" s="18"/>
+      <c r="P21" s="16"/>
       <c r="Q21" s="16"/>
       <c r="R21" s="16"/>
-      <c r="T21" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="U21" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="V21" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="W21" s="21" t="s">
-        <v>94</v>
-      </c>
-      <c r="X21" s="21" t="s">
-        <v>94</v>
-      </c>
+      <c r="T21" s="16"/>
+      <c r="U21" s="16"/>
+      <c r="V21" s="16"/>
+      <c r="W21" s="16"/>
+      <c r="X21" s="21"/>
       <c r="Y21" s="21"/>
       <c r="Z21" s="16"/>
       <c r="AA21" s="16"/>
@@ -5771,13 +6121,13 @@
       <c r="AE21" s="16"/>
       <c r="AF21" s="16"/>
       <c r="AG21" s="16"/>
-      <c r="AH21" s="18"/>
+      <c r="AH21" s="16"/>
       <c r="AI21" s="16"/>
       <c r="AJ21" s="16"/>
     </row>
-    <row r="22" spans="1:36" ht="17" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A22" s="16" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B22" s="16" t="s">
         <v>94</v>
@@ -5794,7 +6144,7 @@
       <c r="F22" s="21" t="s">
         <v>94</v>
       </c>
-      <c r="G22" s="21"/>
+      <c r="G22" s="16"/>
       <c r="H22" s="16" t="s">
         <v>94</v>
       </c>
@@ -5804,57 +6154,79 @@
       <c r="J22" s="16" t="s">
         <v>94</v>
       </c>
-      <c r="K22" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="L22" s="16" t="s">
+      <c r="K22" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="L22" s="21" t="s">
         <v>94</v>
       </c>
       <c r="M22" s="16"/>
-      <c r="N22" s="16"/>
-      <c r="O22" s="16"/>
-      <c r="P22" s="18"/>
-      <c r="Q22" s="16"/>
-      <c r="R22" s="16"/>
-      <c r="T22" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="U22" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="V22" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="W22" s="21" t="s">
-        <v>94</v>
-      </c>
-      <c r="X22" s="21" t="s">
-        <v>94</v>
-      </c>
-      <c r="Y22" s="21"/>
-      <c r="Z22" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="AA22" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="AB22" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="AC22" s="16"/>
-      <c r="AD22" s="16" t="s">
-        <v>94</v>
+      <c r="N22" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="O22" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="P22" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="Q22" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="R22" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="T22" s="16">
+        <v>8.5000000000000006E-2</v>
+      </c>
+      <c r="U22" s="16">
+        <v>3.6999999999999998E-2</v>
+      </c>
+      <c r="V22" s="18">
+        <v>2.1000000000000001E-2</v>
+      </c>
+      <c r="W22" s="16">
+        <v>2.4E-2</v>
+      </c>
+      <c r="X22" s="16">
+        <v>0.14499999999999999</v>
+      </c>
+      <c r="Y22" s="16"/>
+      <c r="Z22" s="16">
+        <v>8.4000000000000005E-2</v>
+      </c>
+      <c r="AA22" s="16">
+        <v>3.6999999999999998E-2</v>
+      </c>
+      <c r="AB22" s="16">
+        <v>2.1999999999999999E-2</v>
+      </c>
+      <c r="AC22" s="16">
+        <v>2.4E-2</v>
+      </c>
+      <c r="AD22" s="16">
+        <v>0.14499999999999999</v>
       </c>
       <c r="AE22" s="16"/>
-      <c r="AF22" s="16"/>
-      <c r="AG22" s="16"/>
-      <c r="AH22" s="18"/>
-      <c r="AI22" s="16"/>
-      <c r="AJ22" s="16"/>
-    </row>
-    <row r="23" spans="1:36" ht="17" x14ac:dyDescent="0.25">
+      <c r="AF22" s="16">
+        <v>8.4000000000000005E-2</v>
+      </c>
+      <c r="AG22" s="16">
+        <v>3.6999999999999998E-2</v>
+      </c>
+      <c r="AH22" s="16">
+        <v>2.1999999999999999E-2</v>
+      </c>
+      <c r="AI22" s="16">
+        <v>2.4E-2</v>
+      </c>
+      <c r="AJ22" s="16">
+        <v>0.14499999999999999</v>
+      </c>
+    </row>
+    <row r="23" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A23" s="16" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="B23" s="16" t="s">
         <v>94</v>
@@ -5872,21 +6244,11 @@
         <v>94</v>
       </c>
       <c r="G23" s="21"/>
-      <c r="H23" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="I23" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="J23" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="K23" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="L23" s="16" t="s">
-        <v>94</v>
-      </c>
+      <c r="H23" s="16"/>
+      <c r="I23" s="16"/>
+      <c r="J23" s="18"/>
+      <c r="K23" s="16"/>
+      <c r="L23" s="16"/>
       <c r="M23" s="16"/>
       <c r="N23" s="16"/>
       <c r="O23" s="16"/>
@@ -5909,29 +6271,41 @@
         <v>94</v>
       </c>
       <c r="Y23" s="21"/>
-      <c r="Z23" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="AA23" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="AB23" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="AC23" s="16"/>
-      <c r="AD23" s="16" t="s">
-        <v>94</v>
+      <c r="Z23" s="16">
+        <v>-0.13100000000000001</v>
+      </c>
+      <c r="AA23" s="16">
+        <v>2.1999999999999999E-2</v>
+      </c>
+      <c r="AB23" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="AC23" s="16">
+        <v>-0.16600000000000001</v>
+      </c>
+      <c r="AD23" s="16">
+        <v>-9.5000000000000001E-2</v>
       </c>
       <c r="AE23" s="16"/>
-      <c r="AF23" s="16"/>
-      <c r="AG23" s="16"/>
-      <c r="AH23" s="16"/>
-      <c r="AI23" s="16"/>
-      <c r="AJ23" s="16"/>
-    </row>
-    <row r="24" spans="1:36" x14ac:dyDescent="0.2">
+      <c r="AF23" s="16">
+        <v>-0.13100000000000001</v>
+      </c>
+      <c r="AG23" s="16">
+        <v>2.1999999999999999E-2</v>
+      </c>
+      <c r="AH23" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="AI23" s="16">
+        <v>-0.16600000000000001</v>
+      </c>
+      <c r="AJ23" s="16">
+        <v>-9.5000000000000001E-2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A24" s="16" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="B24" s="16" t="s">
         <v>94</v>
@@ -5949,21 +6323,11 @@
         <v>94</v>
       </c>
       <c r="G24" s="21"/>
-      <c r="H24" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="I24" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="J24" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="K24" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="L24" s="16" t="s">
-        <v>94</v>
-      </c>
+      <c r="H24" s="22"/>
+      <c r="I24" s="22"/>
+      <c r="J24" s="16"/>
+      <c r="K24" s="16"/>
+      <c r="L24" s="16"/>
       <c r="M24" s="16"/>
       <c r="N24" s="16"/>
       <c r="O24" s="16"/>
@@ -5986,29 +6350,41 @@
         <v>94</v>
       </c>
       <c r="Y24" s="21"/>
-      <c r="Z24" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="AA24" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="AB24" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="AC24" s="16"/>
-      <c r="AD24" s="16" t="s">
-        <v>94</v>
+      <c r="Z24" s="16">
+        <v>-8.9999999999999993E-3</v>
+      </c>
+      <c r="AA24" s="16">
+        <v>3.6999999999999998E-2</v>
+      </c>
+      <c r="AB24" s="16">
+        <v>0.81399999999999995</v>
+      </c>
+      <c r="AC24" s="16">
+        <v>-6.9000000000000006E-2</v>
+      </c>
+      <c r="AD24" s="16">
+        <v>5.1999999999999998E-2</v>
       </c>
       <c r="AE24" s="16"/>
-      <c r="AF24" s="16"/>
-      <c r="AG24" s="16"/>
-      <c r="AH24" s="18"/>
-      <c r="AI24" s="16"/>
-      <c r="AJ24" s="16"/>
-    </row>
-    <row r="25" spans="1:36" x14ac:dyDescent="0.2">
+      <c r="AF24" s="16">
+        <v>-0.01</v>
+      </c>
+      <c r="AG24" s="16">
+        <v>3.6999999999999998E-2</v>
+      </c>
+      <c r="AH24" s="16">
+        <v>0.79300000000000004</v>
+      </c>
+      <c r="AI24" s="16">
+        <v>-7.0000000000000007E-2</v>
+      </c>
+      <c r="AJ24" s="16">
+        <v>5.0999999999999997E-2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A25" s="16" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="B25" s="16" t="s">
         <v>94</v>
@@ -6026,21 +6402,11 @@
         <v>94</v>
       </c>
       <c r="G25" s="21"/>
-      <c r="H25" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="I25" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="J25" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="K25" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="L25" s="16" t="s">
-        <v>94</v>
-      </c>
+      <c r="H25" s="16"/>
+      <c r="I25" s="16"/>
+      <c r="J25" s="18"/>
+      <c r="K25" s="16"/>
+      <c r="L25" s="16"/>
       <c r="M25" s="16"/>
       <c r="N25" s="16"/>
       <c r="O25" s="16"/>
@@ -6063,29 +6429,41 @@
         <v>94</v>
       </c>
       <c r="Y25" s="21"/>
-      <c r="Z25" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="AA25" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="AB25" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="AC25" s="16"/>
-      <c r="AD25" s="16" t="s">
-        <v>94</v>
+      <c r="Z25" s="16">
+        <v>-2E-3</v>
+      </c>
+      <c r="AA25" s="16">
+        <v>2.1000000000000001E-2</v>
+      </c>
+      <c r="AB25" s="16">
+        <v>0.92900000000000005</v>
+      </c>
+      <c r="AC25" s="16">
+        <v>-3.5999999999999997E-2</v>
+      </c>
+      <c r="AD25" s="16">
+        <v>3.3000000000000002E-2</v>
       </c>
       <c r="AE25" s="16"/>
-      <c r="AF25" s="16"/>
-      <c r="AG25" s="16"/>
-      <c r="AH25" s="16"/>
-      <c r="AI25" s="16"/>
-      <c r="AJ25" s="16"/>
-    </row>
-    <row r="26" spans="1:36" x14ac:dyDescent="0.2">
+      <c r="AF25" s="16">
+        <v>-3.0000000000000001E-3</v>
+      </c>
+      <c r="AG25" s="16">
+        <v>2.1000000000000001E-2</v>
+      </c>
+      <c r="AH25" s="16">
+        <v>0.90400000000000003</v>
+      </c>
+      <c r="AI25" s="16">
+        <v>-3.6999999999999998E-2</v>
+      </c>
+      <c r="AJ25" s="16">
+        <v>3.2000000000000001E-2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A26" s="16" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="B26" s="16" t="s">
         <v>94</v>
@@ -6103,21 +6481,11 @@
         <v>94</v>
       </c>
       <c r="G26" s="21"/>
-      <c r="H26" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="I26" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="J26" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="K26" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="L26" s="16" t="s">
-        <v>94</v>
-      </c>
+      <c r="H26" s="16"/>
+      <c r="I26" s="16"/>
+      <c r="J26" s="18"/>
+      <c r="K26" s="16"/>
+      <c r="L26" s="16"/>
       <c r="M26" s="16"/>
       <c r="N26" s="16"/>
       <c r="O26" s="16"/>
@@ -6140,195 +6508,389 @@
         <v>94</v>
       </c>
       <c r="Y26" s="21"/>
-      <c r="Z26" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="AA26" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="AB26" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="AC26" s="16"/>
-      <c r="AD26" s="16" t="s">
-        <v>94</v>
+      <c r="Z26" s="16">
+        <v>-0.17</v>
+      </c>
+      <c r="AA26" s="16">
+        <v>2.1000000000000001E-2</v>
+      </c>
+      <c r="AB26" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="AC26" s="16">
+        <v>-0.20399999999999999</v>
+      </c>
+      <c r="AD26" s="16">
+        <v>-0.13500000000000001</v>
       </c>
       <c r="AE26" s="16"/>
-      <c r="AF26" s="16"/>
-      <c r="AG26" s="16"/>
-      <c r="AH26" s="18"/>
-      <c r="AI26" s="16"/>
-      <c r="AJ26" s="16"/>
-    </row>
-    <row r="27" spans="1:36" x14ac:dyDescent="0.2">
-      <c r="A27" s="16"/>
-      <c r="B27" s="16"/>
-      <c r="C27" s="16"/>
-      <c r="D27" s="16"/>
-      <c r="E27" s="16"/>
-      <c r="F27" s="21"/>
+      <c r="AF26" s="16">
+        <v>-0.17</v>
+      </c>
+      <c r="AG26" s="16">
+        <v>2.1000000000000001E-2</v>
+      </c>
+      <c r="AH26" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="AI26" s="16">
+        <v>-0.20399999999999999</v>
+      </c>
+      <c r="AJ26" s="16">
+        <v>-0.13600000000000001</v>
+      </c>
+    </row>
+    <row r="27" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A27" s="16" t="s">
+        <v>105</v>
+      </c>
+      <c r="B27" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="C27" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="D27" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="E27" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="F27" s="21" t="s">
+        <v>94</v>
+      </c>
       <c r="G27" s="21"/>
-      <c r="H27" s="16"/>
-      <c r="I27" s="16"/>
-      <c r="J27" s="16"/>
-      <c r="K27" s="16"/>
-      <c r="L27" s="16"/>
+      <c r="H27" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="I27" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="J27" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="K27" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="L27" s="16" t="s">
+        <v>94</v>
+      </c>
       <c r="M27" s="16"/>
       <c r="N27" s="16"/>
       <c r="O27" s="16"/>
       <c r="P27" s="18"/>
-      <c r="Q27" s="18"/>
+      <c r="Q27" s="16"/>
       <c r="R27" s="16"/>
-      <c r="T27" s="16"/>
-      <c r="U27" s="16"/>
-      <c r="V27" s="16"/>
-      <c r="W27" s="16"/>
-      <c r="X27" s="21"/>
+      <c r="T27" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="U27" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="V27" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="W27" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="X27" s="21" t="s">
+        <v>94</v>
+      </c>
       <c r="Y27" s="21"/>
-      <c r="Z27" s="16"/>
-      <c r="AA27" s="16"/>
-      <c r="AB27" s="16"/>
+      <c r="Z27" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="AA27" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="AB27" s="16" t="s">
+        <v>94</v>
+      </c>
       <c r="AC27" s="16"/>
-      <c r="AD27" s="16"/>
+      <c r="AD27" s="16" t="s">
+        <v>94</v>
+      </c>
       <c r="AE27" s="16"/>
-      <c r="AF27" s="16"/>
-      <c r="AG27" s="16"/>
-      <c r="AH27" s="18"/>
-      <c r="AI27" s="18"/>
-      <c r="AJ27" s="16"/>
-    </row>
-    <row r="28" spans="1:36" x14ac:dyDescent="0.2">
-      <c r="A28" s="17" t="s">
-        <v>82</v>
-      </c>
-      <c r="B28" s="16"/>
-      <c r="C28" s="16"/>
-      <c r="D28" s="16"/>
-      <c r="E28" s="16"/>
-      <c r="F28" s="21"/>
+      <c r="AF27" s="16">
+        <v>-3.7999999999999999E-2</v>
+      </c>
+      <c r="AG27" s="16">
+        <v>4.4999999999999998E-2</v>
+      </c>
+      <c r="AH27" s="16">
+        <v>0.39900000000000002</v>
+      </c>
+      <c r="AI27" s="16">
+        <v>8.6999999999999994E-2</v>
+      </c>
+      <c r="AJ27" s="16">
+        <v>0.17199999999999999</v>
+      </c>
+    </row>
+    <row r="28" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A28" s="16" t="s">
+        <v>106</v>
+      </c>
+      <c r="B28" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="C28" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="D28" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="E28" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="F28" s="21" t="s">
+        <v>94</v>
+      </c>
       <c r="G28" s="21"/>
-      <c r="H28" s="16"/>
-      <c r="I28" s="16"/>
-      <c r="J28" s="16"/>
-      <c r="K28" s="16"/>
-      <c r="L28" s="16"/>
+      <c r="H28" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="I28" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="J28" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="K28" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="L28" s="16" t="s">
+        <v>94</v>
+      </c>
       <c r="M28" s="16"/>
       <c r="N28" s="16"/>
       <c r="O28" s="16"/>
-      <c r="P28" s="16"/>
+      <c r="P28" s="18"/>
       <c r="Q28" s="16"/>
       <c r="R28" s="16"/>
-      <c r="T28" s="16"/>
-      <c r="U28" s="16"/>
-      <c r="V28" s="16"/>
-      <c r="W28" s="16"/>
-      <c r="X28" s="21"/>
+      <c r="T28" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="U28" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="V28" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="W28" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="X28" s="21" t="s">
+        <v>94</v>
+      </c>
       <c r="Y28" s="21"/>
-      <c r="Z28" s="16"/>
-      <c r="AA28" s="16"/>
-      <c r="AB28" s="16"/>
+      <c r="Z28" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="AA28" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="AB28" s="16" t="s">
+        <v>94</v>
+      </c>
       <c r="AC28" s="16"/>
-      <c r="AD28" s="16"/>
+      <c r="AD28" s="16" t="s">
+        <v>94</v>
+      </c>
       <c r="AE28" s="16"/>
-      <c r="AF28" s="16"/>
-      <c r="AG28" s="16"/>
-      <c r="AH28" s="16"/>
-      <c r="AI28" s="16"/>
-      <c r="AJ28" s="16"/>
-    </row>
-    <row r="29" spans="1:36" x14ac:dyDescent="0.2">
+      <c r="AF28" s="16">
+        <v>0.129</v>
+      </c>
+      <c r="AG28" s="16">
+        <v>2.5999999999999999E-2</v>
+      </c>
+      <c r="AH28" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="AI28" s="16">
+        <v>-0.111</v>
+      </c>
+      <c r="AJ28" s="16">
+        <v>3.5999999999999997E-2</v>
+      </c>
+    </row>
+    <row r="29" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A29" s="16" t="s">
-        <v>84</v>
-      </c>
-      <c r="B29" s="16"/>
-      <c r="C29" s="16"/>
-      <c r="D29" s="18"/>
-      <c r="E29" s="16"/>
-      <c r="F29" s="16"/>
-      <c r="G29" s="16"/>
-      <c r="H29" s="16"/>
-      <c r="I29" s="16"/>
-      <c r="J29" s="18"/>
-      <c r="K29" s="16"/>
-      <c r="L29" s="16"/>
+        <v>110</v>
+      </c>
+      <c r="B29" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="C29" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="D29" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="E29" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="F29" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="G29" s="21"/>
+      <c r="H29" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="I29" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="J29" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="K29" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="L29" s="16" t="s">
+        <v>94</v>
+      </c>
       <c r="M29" s="16"/>
       <c r="N29" s="16"/>
       <c r="O29" s="16"/>
       <c r="P29" s="18"/>
       <c r="Q29" s="16"/>
       <c r="R29" s="16"/>
-      <c r="T29" s="16">
-        <v>13.827</v>
-      </c>
-      <c r="U29" s="16">
-        <v>0.20100000000000001</v>
-      </c>
-      <c r="V29" s="18" t="s">
-        <v>24</v>
-      </c>
-      <c r="W29" s="16"/>
-      <c r="X29" s="16"/>
-      <c r="Y29" s="16"/>
-      <c r="Z29" s="16"/>
-      <c r="AA29" s="16"/>
-      <c r="AB29" s="18"/>
+      <c r="T29" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="U29" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="V29" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="W29" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="X29" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="Y29" s="21"/>
+      <c r="Z29" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="AA29" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="AB29" s="16" t="s">
+        <v>94</v>
+      </c>
       <c r="AC29" s="16"/>
-      <c r="AD29" s="16"/>
+      <c r="AD29" s="16" t="s">
+        <v>94</v>
+      </c>
       <c r="AE29" s="16"/>
-      <c r="AF29" s="16"/>
-      <c r="AG29" s="16"/>
-      <c r="AH29" s="18"/>
-      <c r="AI29" s="16"/>
-      <c r="AJ29" s="16"/>
-    </row>
-    <row r="30" spans="1:36" x14ac:dyDescent="0.2">
+      <c r="AF29" s="16">
+        <v>4.2000000000000003E-2</v>
+      </c>
+      <c r="AG29" s="16">
+        <v>0.02</v>
+      </c>
+      <c r="AH29" s="16">
+        <v>3.5000000000000003E-2</v>
+      </c>
+      <c r="AI29" s="16">
+        <v>8.9999999999999993E-3</v>
+      </c>
+      <c r="AJ29" s="16">
+        <v>7.4999999999999997E-2</v>
+      </c>
+    </row>
+    <row r="30" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A30" s="16" t="s">
-        <v>89</v>
-      </c>
-      <c r="B30" s="16"/>
-      <c r="C30" s="16"/>
-      <c r="D30" s="18"/>
-      <c r="E30" s="16"/>
-      <c r="F30" s="16"/>
-      <c r="G30" s="16"/>
-      <c r="H30" s="16"/>
-      <c r="I30" s="16"/>
-      <c r="J30" s="18"/>
-      <c r="K30" s="16"/>
-      <c r="L30" s="16"/>
+        <v>109</v>
+      </c>
+      <c r="B30" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="C30" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="D30" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="E30" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="F30" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="G30" s="21"/>
+      <c r="H30" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="I30" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="J30" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="K30" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="L30" s="16" t="s">
+        <v>94</v>
+      </c>
       <c r="M30" s="16"/>
       <c r="N30" s="16"/>
       <c r="O30" s="16"/>
       <c r="P30" s="18"/>
       <c r="Q30" s="16"/>
       <c r="R30" s="16"/>
-      <c r="T30" s="16">
-        <v>3.8889999999999998</v>
-      </c>
-      <c r="U30" s="16">
-        <v>6.3E-2</v>
-      </c>
-      <c r="V30" s="18" t="s">
-        <v>24</v>
-      </c>
-      <c r="W30" s="16"/>
-      <c r="X30" s="16"/>
-      <c r="Y30" s="16"/>
-      <c r="Z30" s="16"/>
-      <c r="AA30" s="16"/>
-      <c r="AB30" s="18"/>
+      <c r="T30" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="U30" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="V30" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="W30" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="X30" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="Y30" s="21"/>
+      <c r="Z30" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="AA30" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="AB30" s="16" t="s">
+        <v>94</v>
+      </c>
       <c r="AC30" s="16"/>
-      <c r="AD30" s="16"/>
+      <c r="AD30" s="16" t="s">
+        <v>94</v>
+      </c>
       <c r="AE30" s="16"/>
-      <c r="AF30" s="16"/>
-      <c r="AG30" s="16"/>
-      <c r="AH30" s="18"/>
-      <c r="AI30" s="16"/>
-      <c r="AJ30" s="16"/>
-    </row>
-    <row r="31" spans="1:36" x14ac:dyDescent="0.2">
+      <c r="AF30" s="16">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="AG30" s="16">
+        <v>2.1999999999999999E-2</v>
+      </c>
+      <c r="AH30" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="AI30" s="16">
+        <v>0.104</v>
+      </c>
+      <c r="AJ30" s="16">
+        <v>0.17499999999999999</v>
+      </c>
+    </row>
+    <row r="31" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A31" s="16" t="s">
-        <v>93</v>
+        <v>111</v>
       </c>
       <c r="B31" s="16" t="s">
         <v>94</v>
@@ -6339,18 +6901,28 @@
       <c r="D31" s="16" t="s">
         <v>94</v>
       </c>
-      <c r="E31" s="16" t="s">
+      <c r="E31" s="21" t="s">
         <v>94</v>
       </c>
       <c r="F31" s="21" t="s">
         <v>94</v>
       </c>
       <c r="G31" s="21"/>
-      <c r="H31" s="16"/>
-      <c r="I31" s="16"/>
-      <c r="J31" s="18"/>
-      <c r="K31" s="16"/>
-      <c r="L31" s="16"/>
+      <c r="H31" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="I31" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="J31" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="K31" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="L31" s="16" t="s">
+        <v>94</v>
+      </c>
       <c r="M31" s="16"/>
       <c r="N31" s="16"/>
       <c r="O31" s="16"/>
@@ -6366,204 +6938,540 @@
       <c r="V31" s="16" t="s">
         <v>94</v>
       </c>
-      <c r="W31" s="16" t="s">
+      <c r="W31" s="21" t="s">
         <v>94</v>
       </c>
       <c r="X31" s="21" t="s">
         <v>94</v>
       </c>
       <c r="Y31" s="21"/>
-      <c r="Z31" s="16"/>
-      <c r="AA31" s="16"/>
-      <c r="AB31" s="18"/>
+      <c r="Z31" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="AA31" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="AB31" s="16" t="s">
+        <v>94</v>
+      </c>
       <c r="AC31" s="16"/>
-      <c r="AD31" s="16"/>
+      <c r="AD31" s="16" t="s">
+        <v>94</v>
+      </c>
       <c r="AE31" s="16"/>
-      <c r="AF31" s="16"/>
-      <c r="AG31" s="16"/>
-      <c r="AH31" s="18"/>
-      <c r="AI31" s="16"/>
-      <c r="AJ31" s="16"/>
-    </row>
-    <row r="32" spans="1:36" x14ac:dyDescent="0.2">
-      <c r="A32" s="16" t="s">
-        <v>112</v>
-      </c>
-      <c r="B32" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="C32" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="D32" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="E32" s="21" t="s">
-        <v>94</v>
-      </c>
-      <c r="F32" s="21" t="s">
-        <v>94</v>
-      </c>
+      <c r="AF31" s="16">
+        <v>-8.4000000000000005E-2</v>
+      </c>
+      <c r="AG31" s="16">
+        <v>0.02</v>
+      </c>
+      <c r="AH31" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="AI31" s="16">
+        <v>-0.11700000000000001</v>
+      </c>
+      <c r="AJ31" s="16">
+        <v>-0.05</v>
+      </c>
+    </row>
+    <row r="32" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A32" s="16"/>
+      <c r="B32" s="16"/>
+      <c r="C32" s="16"/>
+      <c r="D32" s="16"/>
+      <c r="E32" s="16"/>
+      <c r="F32" s="21"/>
       <c r="G32" s="21"/>
-      <c r="H32" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="I32" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="J32" s="16" t="s">
-        <v>94</v>
-      </c>
+      <c r="H32" s="16"/>
+      <c r="I32" s="16"/>
+      <c r="J32" s="16"/>
       <c r="K32" s="16"/>
-      <c r="L32" s="16" t="s">
-        <v>94</v>
-      </c>
+      <c r="L32" s="16"/>
       <c r="M32" s="16"/>
       <c r="N32" s="16"/>
       <c r="O32" s="16"/>
       <c r="P32" s="18"/>
-      <c r="Q32" s="16"/>
+      <c r="Q32" s="18"/>
       <c r="R32" s="16"/>
-      <c r="T32" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="U32" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="V32" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="W32" s="21" t="s">
-        <v>94</v>
-      </c>
-      <c r="X32" s="21" t="s">
-        <v>94</v>
-      </c>
+      <c r="T32" s="16"/>
+      <c r="U32" s="16"/>
+      <c r="V32" s="16"/>
+      <c r="W32" s="16"/>
+      <c r="X32" s="21"/>
       <c r="Y32" s="21"/>
-      <c r="Z32" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="AA32" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="AB32" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="AC32" s="21" t="s">
-        <v>94</v>
-      </c>
-      <c r="AD32" s="21" t="s">
-        <v>94</v>
-      </c>
+      <c r="Z32" s="16"/>
+      <c r="AA32" s="16"/>
+      <c r="AB32" s="16"/>
+      <c r="AC32" s="16"/>
+      <c r="AD32" s="16"/>
       <c r="AE32" s="16"/>
       <c r="AF32" s="16"/>
       <c r="AG32" s="16"/>
       <c r="AH32" s="18"/>
-      <c r="AI32" s="16"/>
+      <c r="AI32" s="18"/>
       <c r="AJ32" s="16"/>
     </row>
-    <row r="33" spans="1:39" x14ac:dyDescent="0.2">
-      <c r="A33" s="20" t="s">
+    <row r="33" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A33" s="17" t="s">
+        <v>82</v>
+      </c>
+      <c r="B33" s="16"/>
+      <c r="C33" s="16"/>
+      <c r="D33" s="16"/>
+      <c r="E33" s="16"/>
+      <c r="F33" s="21"/>
+      <c r="G33" s="21"/>
+      <c r="H33" s="16"/>
+      <c r="I33" s="16"/>
+      <c r="J33" s="16"/>
+      <c r="K33" s="16"/>
+      <c r="L33" s="16"/>
+      <c r="M33" s="16"/>
+      <c r="N33" s="16"/>
+      <c r="O33" s="16"/>
+      <c r="P33" s="16"/>
+      <c r="Q33" s="16"/>
+      <c r="R33" s="16"/>
+      <c r="T33" s="16"/>
+      <c r="U33" s="16"/>
+      <c r="V33" s="16"/>
+      <c r="W33" s="16"/>
+      <c r="X33" s="21"/>
+      <c r="Y33" s="21"/>
+      <c r="Z33" s="16"/>
+      <c r="AA33" s="16"/>
+      <c r="AB33" s="16"/>
+      <c r="AC33" s="16"/>
+      <c r="AD33" s="16"/>
+      <c r="AE33" s="16"/>
+      <c r="AF33" s="16"/>
+      <c r="AG33" s="16"/>
+      <c r="AH33" s="16"/>
+      <c r="AI33" s="16"/>
+      <c r="AJ33" s="16"/>
+    </row>
+    <row r="34" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A34" s="16" t="s">
+        <v>84</v>
+      </c>
+      <c r="B34" s="16">
+        <v>10.965</v>
+      </c>
+      <c r="C34" s="16">
+        <v>0.158</v>
+      </c>
+      <c r="D34" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="E34" s="16">
+        <v>10.706</v>
+      </c>
+      <c r="F34" s="16">
+        <v>11.225</v>
+      </c>
+      <c r="G34" s="16"/>
+      <c r="H34" s="16"/>
+      <c r="I34" s="16"/>
+      <c r="J34" s="18"/>
+      <c r="K34" s="16"/>
+      <c r="L34" s="16"/>
+      <c r="M34" s="16"/>
+      <c r="N34" s="16"/>
+      <c r="O34" s="16"/>
+      <c r="P34" s="18"/>
+      <c r="Q34" s="16"/>
+      <c r="R34" s="16"/>
+      <c r="T34" s="16">
+        <v>13.827</v>
+      </c>
+      <c r="U34" s="16">
+        <v>0.20100000000000001</v>
+      </c>
+      <c r="V34" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="W34" s="16">
+        <v>13.496</v>
+      </c>
+      <c r="X34" s="16">
+        <v>14.157999999999999</v>
+      </c>
+      <c r="Y34" s="16"/>
+      <c r="Z34" s="16">
+        <v>13.829000000000001</v>
+      </c>
+      <c r="AA34" s="16">
+        <v>0.20200000000000001</v>
+      </c>
+      <c r="AB34" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="AC34" s="16">
+        <v>13.496</v>
+      </c>
+      <c r="AD34" s="16">
+        <v>14.161</v>
+      </c>
+      <c r="AE34" s="16"/>
+      <c r="AF34" s="16">
+        <v>13.829000000000001</v>
+      </c>
+      <c r="AG34" s="16">
+        <v>0.20200000000000001</v>
+      </c>
+      <c r="AH34" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="AI34" s="16">
+        <v>13.497</v>
+      </c>
+      <c r="AJ34" s="16">
+        <v>14.162000000000001</v>
+      </c>
+    </row>
+    <row r="35" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A35" s="16" t="s">
+        <v>89</v>
+      </c>
+      <c r="B35" s="16">
+        <v>3.7109999999999999</v>
+      </c>
+      <c r="C35" s="16">
+        <v>6.3E-2</v>
+      </c>
+      <c r="D35" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="E35" s="16">
+        <v>3.6070000000000002</v>
+      </c>
+      <c r="F35" s="16">
+        <v>3.8149999999999999</v>
+      </c>
+      <c r="G35" s="16"/>
+      <c r="H35" s="16"/>
+      <c r="I35" s="16"/>
+      <c r="J35" s="18"/>
+      <c r="K35" s="16"/>
+      <c r="L35" s="16"/>
+      <c r="M35" s="16"/>
+      <c r="N35" s="16"/>
+      <c r="O35" s="16"/>
+      <c r="P35" s="18"/>
+      <c r="Q35" s="16"/>
+      <c r="R35" s="16"/>
+      <c r="T35" s="16">
+        <v>3.8889999999999998</v>
+      </c>
+      <c r="U35" s="16">
+        <v>6.3E-2</v>
+      </c>
+      <c r="V35" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="W35" s="16">
+        <v>3.7839999999999998</v>
+      </c>
+      <c r="X35" s="16">
+        <v>3.9929999999999999</v>
+      </c>
+      <c r="Y35" s="16"/>
+      <c r="Z35" s="16">
+        <v>4.0620000000000003</v>
+      </c>
+      <c r="AA35" s="16">
+        <v>6.4000000000000001E-2</v>
+      </c>
+      <c r="AB35" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="AC35" s="16">
+        <v>3.9569999999999999</v>
+      </c>
+      <c r="AD35" s="16">
+        <v>4.1669999999999998</v>
+      </c>
+      <c r="AE35" s="16"/>
+      <c r="AF35" s="16">
+        <v>4.0609999999999999</v>
+      </c>
+      <c r="AG35" s="16">
+        <v>6.4000000000000001E-2</v>
+      </c>
+      <c r="AH35" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="AI35" s="16">
+        <v>3.956</v>
+      </c>
+      <c r="AJ35" s="16">
+        <v>4.1660000000000004</v>
+      </c>
+    </row>
+    <row r="36" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A36" s="16" t="s">
+        <v>93</v>
+      </c>
+      <c r="B36" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="C36" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="D36" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="E36" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="F36" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="G36" s="21"/>
+      <c r="H36" s="16"/>
+      <c r="I36" s="16"/>
+      <c r="J36" s="18"/>
+      <c r="K36" s="16"/>
+      <c r="L36" s="16"/>
+      <c r="M36" s="16"/>
+      <c r="N36" s="16"/>
+      <c r="O36" s="16"/>
+      <c r="P36" s="18"/>
+      <c r="Q36" s="16"/>
+      <c r="R36" s="16"/>
+      <c r="T36" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="U36" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="V36" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="W36" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="X36" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="Y36" s="21"/>
+      <c r="Z36" s="16">
+        <v>1.026</v>
+      </c>
+      <c r="AA36" s="16">
+        <v>1.7000000000000001E-2</v>
+      </c>
+      <c r="AB36" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="AC36" s="16">
+        <v>0.998</v>
+      </c>
+      <c r="AD36" s="16">
+        <v>1.054</v>
+      </c>
+      <c r="AE36" s="16"/>
+      <c r="AF36" s="16">
+        <v>1.0269999999999999</v>
+      </c>
+      <c r="AG36" s="16">
+        <v>1.7000000000000001E-2</v>
+      </c>
+      <c r="AH36" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="AI36" s="16">
+        <v>0.999</v>
+      </c>
+      <c r="AJ36" s="16">
+        <v>1.0549999999999999</v>
+      </c>
+    </row>
+    <row r="37" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A37" s="16" t="s">
+        <v>112</v>
+      </c>
+      <c r="B37" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="C37" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="D37" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="E37" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="F37" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="G37" s="21"/>
+      <c r="H37" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="I37" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="J37" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="K37" s="16"/>
+      <c r="L37" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="M37" s="16"/>
+      <c r="N37" s="16"/>
+      <c r="O37" s="16"/>
+      <c r="P37" s="18"/>
+      <c r="Q37" s="16"/>
+      <c r="R37" s="16"/>
+      <c r="T37" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="U37" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="V37" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="W37" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="X37" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="Y37" s="21"/>
+      <c r="Z37" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="AA37" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="AB37" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="AC37" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="AD37" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="AE37" s="16"/>
+      <c r="AF37" s="16">
+        <v>3.7440000000000002</v>
+      </c>
+      <c r="AG37" s="16">
+        <v>0.46500000000000002</v>
+      </c>
+      <c r="AH37" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="AI37" s="16">
+        <v>2.9790000000000001</v>
+      </c>
+      <c r="AJ37" s="16">
+        <v>4.5090000000000003</v>
+      </c>
+    </row>
+    <row r="38" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A38" s="20" t="s">
         <v>117</v>
       </c>
-      <c r="B33" s="14"/>
-      <c r="C33" s="14"/>
-      <c r="D33" s="14"/>
-      <c r="E33" s="14"/>
-      <c r="F33" s="14"/>
-      <c r="G33" s="16"/>
-      <c r="H33" s="14"/>
-      <c r="I33" s="14"/>
-      <c r="J33" s="14"/>
-      <c r="K33" s="14"/>
-      <c r="L33" s="14"/>
-      <c r="M33" s="16"/>
-      <c r="N33" s="14"/>
-      <c r="O33" s="14"/>
-      <c r="P33" s="14"/>
-      <c r="Q33" s="14"/>
-      <c r="R33" s="14"/>
-      <c r="S33" s="16"/>
-      <c r="T33" s="14"/>
-      <c r="U33" s="14"/>
-      <c r="V33" s="14"/>
-      <c r="W33" s="14"/>
-      <c r="X33" s="14"/>
-      <c r="Y33" s="16"/>
-      <c r="Z33" s="14"/>
-      <c r="AA33" s="14"/>
-      <c r="AB33" s="14"/>
-      <c r="AC33" s="14"/>
-      <c r="AD33" s="14"/>
-      <c r="AE33" s="16"/>
-      <c r="AF33" s="14"/>
-      <c r="AG33" s="14"/>
-      <c r="AH33" s="14"/>
-      <c r="AI33" s="14"/>
-      <c r="AJ33" s="14"/>
-      <c r="AK33" s="16"/>
-      <c r="AL33" s="16"/>
-      <c r="AM33" s="16"/>
-    </row>
-    <row r="34" spans="1:39" x14ac:dyDescent="0.2">
-      <c r="A34" s="15" t="s">
+      <c r="B38" s="14"/>
+      <c r="C38" s="14"/>
+      <c r="D38" s="14"/>
+      <c r="E38" s="14"/>
+      <c r="F38" s="14"/>
+      <c r="G38" s="16"/>
+      <c r="H38" s="14"/>
+      <c r="I38" s="14"/>
+      <c r="J38" s="14"/>
+      <c r="K38" s="14"/>
+      <c r="L38" s="14"/>
+      <c r="M38" s="16"/>
+      <c r="N38" s="14"/>
+      <c r="O38" s="14"/>
+      <c r="P38" s="14"/>
+      <c r="Q38" s="14"/>
+      <c r="R38" s="14"/>
+      <c r="S38" s="16"/>
+      <c r="T38" s="14"/>
+      <c r="U38" s="14"/>
+      <c r="V38" s="14"/>
+      <c r="W38" s="14"/>
+      <c r="X38" s="14"/>
+      <c r="Y38" s="16"/>
+      <c r="Z38" s="14"/>
+      <c r="AA38" s="14"/>
+      <c r="AB38" s="14"/>
+      <c r="AC38" s="14"/>
+      <c r="AD38" s="14"/>
+      <c r="AE38" s="16"/>
+      <c r="AF38" s="14"/>
+      <c r="AG38" s="14"/>
+      <c r="AH38" s="14"/>
+      <c r="AI38" s="14"/>
+      <c r="AJ38" s="14"/>
+      <c r="AK38" s="16"/>
+      <c r="AL38" s="16"/>
+      <c r="AM38" s="16"/>
+    </row>
+    <row r="39" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A39" s="15" t="s">
         <v>118</v>
       </c>
-      <c r="B34" s="31">
-        <v>74058.118000000002</v>
-      </c>
-      <c r="C34" s="31"/>
-      <c r="D34" s="31"/>
-      <c r="E34" s="31"/>
-      <c r="F34" s="31"/>
-      <c r="G34" s="27"/>
-      <c r="H34" s="31">
-        <v>83016.937999999995</v>
-      </c>
-      <c r="I34" s="31"/>
-      <c r="J34" s="31"/>
-      <c r="K34" s="31"/>
-      <c r="L34" s="31"/>
-      <c r="M34" s="27"/>
-      <c r="N34" s="31">
-        <v>94345.274999999994</v>
-      </c>
-      <c r="O34" s="31"/>
-      <c r="P34" s="31"/>
-      <c r="Q34" s="31"/>
-      <c r="R34" s="31"/>
-      <c r="S34" s="15"/>
-      <c r="T34" s="36">
+      <c r="B39" s="33">
+        <v>34697.703999999998</v>
+      </c>
+      <c r="C39" s="33"/>
+      <c r="D39" s="33"/>
+      <c r="E39" s="33"/>
+      <c r="F39" s="33"/>
+      <c r="G39" s="27"/>
+      <c r="H39" s="33"/>
+      <c r="I39" s="33"/>
+      <c r="J39" s="33"/>
+      <c r="K39" s="33"/>
+      <c r="L39" s="33"/>
+      <c r="M39" s="27"/>
+      <c r="N39" s="33"/>
+      <c r="O39" s="33"/>
+      <c r="P39" s="33"/>
+      <c r="Q39" s="33"/>
+      <c r="R39" s="33"/>
+      <c r="S39" s="15"/>
+      <c r="T39" s="33">
         <v>37782.404000000002</v>
       </c>
-      <c r="U34" s="36"/>
-      <c r="V34" s="36"/>
-      <c r="W34" s="36"/>
-      <c r="X34" s="36"/>
-      <c r="Y34" s="27"/>
-      <c r="Z34" s="31"/>
-      <c r="AA34" s="31"/>
-      <c r="AB34" s="31"/>
-      <c r="AC34" s="31"/>
-      <c r="AD34" s="31"/>
-      <c r="AE34" s="27"/>
-      <c r="AF34" s="31"/>
-      <c r="AG34" s="31"/>
-      <c r="AH34" s="31"/>
-      <c r="AI34" s="31"/>
-      <c r="AJ34" s="31"/>
-      <c r="AK34" s="16"/>
-      <c r="AL34" s="16"/>
-      <c r="AM34" s="16"/>
+      <c r="U39" s="33"/>
+      <c r="V39" s="33"/>
+      <c r="W39" s="33"/>
+      <c r="X39" s="33"/>
+      <c r="Y39" s="27"/>
+      <c r="Z39" s="33">
+        <v>47698.324999999997</v>
+      </c>
+      <c r="AA39" s="33"/>
+      <c r="AB39" s="33"/>
+      <c r="AC39" s="33"/>
+      <c r="AD39" s="33"/>
+      <c r="AE39" s="27"/>
+      <c r="AF39" s="33">
+        <v>60402.93</v>
+      </c>
+      <c r="AG39" s="33"/>
+      <c r="AH39" s="33"/>
+      <c r="AI39" s="33"/>
+      <c r="AJ39" s="33"/>
+      <c r="AK39" s="16"/>
+      <c r="AL39" s="16"/>
+      <c r="AM39" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="B34:F34"/>
-    <mergeCell ref="H34:L34"/>
-    <mergeCell ref="N34:R34"/>
-    <mergeCell ref="T34:X34"/>
-    <mergeCell ref="Z34:AD34"/>
-    <mergeCell ref="AF34:AJ34"/>
+    <mergeCell ref="AF39:AJ39"/>
     <mergeCell ref="B2:R2"/>
     <mergeCell ref="T2:AJ2"/>
     <mergeCell ref="B3:F3"/>
@@ -6572,6 +7480,11 @@
     <mergeCell ref="T3:X3"/>
     <mergeCell ref="Z3:AD3"/>
     <mergeCell ref="AF3:AJ3"/>
+    <mergeCell ref="B39:F39"/>
+    <mergeCell ref="H39:L39"/>
+    <mergeCell ref="N39:R39"/>
+    <mergeCell ref="T39:X39"/>
+    <mergeCell ref="Z39:AD39"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
@@ -6581,27 +7494,27 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57A86273-0E84-8246-B3ED-A023C6721217}">
   <dimension ref="A1:M38"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.1640625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="4.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="5.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="4.625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="5.875" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="7.5" style="1" customWidth="1"/>
     <col min="7" max="7" width="7" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="5.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="5.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="6.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="5.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="5.625" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="6.125" style="1" bestFit="1" customWidth="1"/>
     <col min="11" max="16384" width="11" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="14"/>
       <c r="B2" s="34"/>
       <c r="C2" s="34"/>
@@ -6612,7 +7525,7 @@
       <c r="I2" s="34"/>
       <c r="J2" s="34"/>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="15"/>
       <c r="B3" s="35" t="s">
         <v>81</v>
@@ -6627,7 +7540,7 @@
       <c r="I3" s="35"/>
       <c r="J3" s="35"/>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="16"/>
       <c r="B4" s="17" t="s">
         <v>90</v>
@@ -6654,7 +7567,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="17" t="s">
         <v>85</v>
       </c>
@@ -6667,7 +7580,7 @@
       <c r="I5" s="16"/>
       <c r="J5" s="16"/>
     </row>
-    <row r="6" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="16" t="s">
         <v>96</v>
       </c>
@@ -6680,7 +7593,7 @@
       <c r="I6" s="18"/>
       <c r="J6" s="16"/>
     </row>
-    <row r="7" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="16" t="s">
         <v>97</v>
       </c>
@@ -6693,7 +7606,7 @@
       <c r="I7" s="18"/>
       <c r="J7" s="16"/>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="17" t="s">
         <v>86</v>
       </c>
@@ -6706,7 +7619,7 @@
       <c r="I8" s="16"/>
       <c r="J8" s="16"/>
     </row>
-    <row r="9" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="16" t="s">
         <v>98</v>
       </c>
@@ -6719,7 +7632,7 @@
       <c r="I9" s="18"/>
       <c r="J9" s="16"/>
     </row>
-    <row r="10" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="16" t="s">
         <v>99</v>
       </c>
@@ -6736,7 +7649,7 @@
       <c r="I10" s="18"/>
       <c r="J10" s="16"/>
     </row>
-    <row r="11" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="16" t="s">
         <v>100</v>
       </c>
@@ -6753,7 +7666,7 @@
       <c r="I11" s="18"/>
       <c r="J11" s="16"/>
     </row>
-    <row r="12" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="25" t="s">
         <v>101</v>
       </c>
@@ -6770,7 +7683,7 @@
       <c r="I12" s="18"/>
       <c r="J12" s="16"/>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="16" t="s">
         <v>88</v>
       </c>
@@ -6787,7 +7700,7 @@
       <c r="I13" s="18"/>
       <c r="J13" s="16"/>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="17" t="s">
         <v>87</v>
       </c>
@@ -6800,7 +7713,7 @@
       <c r="I14" s="16"/>
       <c r="J14" s="16"/>
     </row>
-    <row r="15" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="16" t="s">
         <v>102</v>
       </c>
@@ -6817,7 +7730,7 @@
       <c r="I15" s="18"/>
       <c r="J15" s="16"/>
     </row>
-    <row r="16" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="16" t="s">
         <v>103</v>
       </c>
@@ -6830,7 +7743,7 @@
       <c r="I16" s="18"/>
       <c r="J16" s="16"/>
     </row>
-    <row r="17" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="16" t="s">
         <v>104</v>
       </c>
@@ -6843,7 +7756,7 @@
       <c r="I17" s="18"/>
       <c r="J17" s="16"/>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="16" t="s">
         <v>107</v>
       </c>
@@ -6860,7 +7773,7 @@
       <c r="I18" s="18"/>
       <c r="J18" s="16"/>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="16" t="s">
         <v>108</v>
       </c>
@@ -6877,7 +7790,7 @@
       <c r="I19" s="18"/>
       <c r="J19" s="16"/>
     </row>
-    <row r="20" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="16" t="s">
         <v>105</v>
       </c>
@@ -6890,7 +7803,7 @@
       <c r="I20" s="18"/>
       <c r="J20" s="16"/>
     </row>
-    <row r="21" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="16" t="s">
         <v>106</v>
       </c>
@@ -6903,7 +7816,7 @@
       <c r="I21" s="18"/>
       <c r="J21" s="16"/>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="16" t="s">
         <v>110</v>
       </c>
@@ -6920,7 +7833,7 @@
       <c r="I22" s="18"/>
       <c r="J22" s="16"/>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="16" t="s">
         <v>109</v>
       </c>
@@ -6937,7 +7850,7 @@
       <c r="I23" s="18"/>
       <c r="J23" s="16"/>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" s="16" t="s">
         <v>111</v>
       </c>
@@ -6950,7 +7863,7 @@
       <c r="I24" s="18"/>
       <c r="J24" s="16"/>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" s="17" t="s">
         <v>82</v>
       </c>
@@ -6963,7 +7876,7 @@
       <c r="I25" s="16"/>
       <c r="J25" s="16"/>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" s="16" t="s">
         <v>84</v>
       </c>
@@ -6980,7 +7893,7 @@
       <c r="I26" s="18"/>
       <c r="J26" s="16"/>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" s="16" t="s">
         <v>89</v>
       </c>
@@ -6997,7 +7910,7 @@
       <c r="I27" s="18"/>
       <c r="J27" s="16"/>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" s="16" t="s">
         <v>93</v>
       </c>
@@ -7016,7 +7929,7 @@
       <c r="I28" s="18"/>
       <c r="J28" s="16"/>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" s="16" t="s">
         <v>112</v>
       </c>
@@ -7029,7 +7942,7 @@
       <c r="I29" s="18"/>
       <c r="J29" s="16"/>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" s="17" t="s">
         <v>83</v>
       </c>
@@ -7042,7 +7955,7 @@
       <c r="I30" s="16"/>
       <c r="J30" s="16"/>
     </row>
-    <row r="31" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" s="16" t="s">
         <v>96</v>
       </c>
@@ -7061,7 +7974,7 @@
       <c r="I31" s="18"/>
       <c r="J31" s="16"/>
     </row>
-    <row r="32" spans="1:10" ht="17" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" s="16" t="s">
         <v>97</v>
       </c>
@@ -7080,7 +7993,7 @@
       <c r="I32" s="18"/>
       <c r="J32" s="16"/>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A33" s="16" t="s">
         <v>84</v>
       </c>
@@ -7097,7 +8010,7 @@
       <c r="I33" s="18"/>
       <c r="J33" s="16"/>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A34" s="16" t="s">
         <v>89</v>
       </c>
@@ -7114,7 +8027,7 @@
       <c r="I34" s="18"/>
       <c r="J34" s="16"/>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A35" s="16" t="s">
         <v>93</v>
       </c>
@@ -7127,7 +8040,7 @@
       <c r="I35" s="18"/>
       <c r="J35" s="16"/>
     </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A36" s="16" t="s">
         <v>112</v>
       </c>
@@ -7138,7 +8051,7 @@
       <c r="H36" s="16"/>
       <c r="I36" s="18"/>
     </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A37" s="20" t="s">
         <v>117</v>
       </c>
@@ -7155,7 +8068,7 @@
       <c r="L37" s="16"/>
       <c r="M37" s="16"/>
     </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A38" s="15" t="s">
         <v>118</v>
       </c>
@@ -7186,54 +8099,54 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{540507A6-720C-0B43-804E-087FEE710926}">
   <dimension ref="A1:E25"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.83203125" customWidth="1"/>
-    <col min="2" max="2" width="18.83203125" customWidth="1"/>
-    <col min="3" max="3" width="19.1640625" customWidth="1"/>
+    <col min="1" max="1" width="19.875" customWidth="1"/>
+    <col min="2" max="2" width="18.875" customWidth="1"/>
+    <col min="3" max="3" width="19.125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="23" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="2" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="24"/>
     </row>
-    <row r="3" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="24" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="4" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="24" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="5" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="24"/>
     </row>
-    <row r="6" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="24"/>
     </row>
-    <row r="7" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="8" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="8" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="23" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="24" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="24" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B11" s="23" t="s">
         <v>129</v>
       </c>
@@ -7241,7 +8154,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>126</v>
       </c>
@@ -7252,7 +8165,7 @@
         <v>-1.4E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>127</v>
       </c>
@@ -7263,7 +8176,7 @@
         <v>-8.0000000000000002E-3</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>128</v>
       </c>
@@ -7274,7 +8187,7 @@
         <v>-7.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>133</v>
       </c>
@@ -7285,17 +8198,17 @@
         <v>-8.0000000000000002E-3</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="23" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="24" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B19" s="23" t="s">
         <v>129</v>
       </c>
@@ -7303,7 +8216,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>126</v>
       </c>
@@ -7314,7 +8227,7 @@
         <v>-1.0999999999999999E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>127</v>
       </c>
@@ -7325,7 +8238,7 @@
         <v>-1.2999999999999999E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>128</v>
       </c>
@@ -7336,7 +8249,7 @@
         <v>9.7000000000000003E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>133</v>
       </c>
@@ -7347,7 +8260,7 @@
         <v>-1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="E25" s="23" t="s">
         <v>132</v>
       </c>

</xml_diff>

<commit_message>
added to sensitivity tables
</commit_message>
<xml_diff>
--- a/Tables.xlsx
+++ b/Tables.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10125"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nchaku\Documents\GitHub\pubertybrain\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uvmoffice-my.sharepoint.com/personal/abrieant_uvm_edu/Documents/OneDrive/Manuscripts/reg report DCN/pubertybrain/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF0C5C2D-21F6-4142-814F-EFC173B4BD72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="50" documentId="13_ncr:1_{DF0C5C2D-21F6-4142-814F-EFC173B4BD72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A66E4D3C-8232-9C46-9AFD-9E69F4CA7021}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="5" xr2:uid="{E0F15479-AA73-0644-8B08-3949D67CD8FE}"/>
+    <workbookView xWindow="-120" yWindow="500" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="6" xr2:uid="{E0F15479-AA73-0644-8B08-3949D67CD8FE}"/>
   </bookViews>
   <sheets>
     <sheet name="Descriptive table" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="805" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="810" uniqueCount="145">
   <si>
     <t>16.10 (2.98)</t>
   </si>
@@ -388,27 +388,6 @@
   </si>
   <si>
     <t>-</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>95%</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>CI</t>
-    </r>
   </si>
   <si>
     <r>
@@ -835,6 +814,15 @@
       </rPr>
       <t>with Tempo</t>
     </r>
+  </si>
+  <si>
+    <t>Model 3 - Boys</t>
+  </si>
+  <si>
+    <t>Model 3 - Girls</t>
+  </si>
+  <si>
+    <t>12.311      0.203</t>
   </si>
 </sst>
 </file>
@@ -957,7 +945,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -994,11 +982,114 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1046,20 +1137,34 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1641,20 +1746,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39987BE7-3659-524A-81AE-D479F97EF698}">
   <dimension ref="A1:F29"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="28.875" bestFit="1" customWidth="1"/>
-    <col min="2" max="4" width="20.125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28.83203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="4" width="20.1640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="9"/>
       <c r="B2" s="10" t="s">
         <v>63</v>
@@ -1672,7 +1777,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="6"/>
       <c r="B3" s="11" t="s">
         <v>69</v>
@@ -1686,7 +1791,7 @@
       <c r="E3" s="11"/>
       <c r="F3" s="6"/>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
         <v>60</v>
       </c>
@@ -1696,7 +1801,7 @@
       <c r="E4" s="2"/>
       <c r="F4" s="1"/>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
         <v>61</v>
       </c>
@@ -1716,7 +1821,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
         <v>62</v>
       </c>
@@ -1736,7 +1841,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
         <v>58</v>
       </c>
@@ -1756,7 +1861,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="8" t="s">
         <v>59</v>
       </c>
@@ -1766,7 +1871,7 @@
       <c r="E8" s="12"/>
       <c r="F8" s="1"/>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="3" t="s">
         <v>61</v>
       </c>
@@ -1786,7 +1891,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="3" t="s">
         <v>66</v>
       </c>
@@ -1806,7 +1911,7 @@
         <v>0.06</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="3" t="s">
         <v>67</v>
       </c>
@@ -1826,7 +1931,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="3" t="s">
         <v>62</v>
       </c>
@@ -1846,7 +1951,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" s="8" t="s">
         <v>68</v>
       </c>
@@ -1856,7 +1961,7 @@
       <c r="E13" s="12"/>
       <c r="F13" s="1"/>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" s="3" t="s">
         <v>73</v>
       </c>
@@ -1876,7 +1981,7 @@
         <v>1.74</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
         <v>74</v>
       </c>
@@ -1896,7 +2001,7 @@
         <v>1.93</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" s="3" t="s">
         <v>75</v>
       </c>
@@ -1916,7 +2021,7 @@
         <v>1.69</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" s="3" t="s">
         <v>76</v>
       </c>
@@ -1934,7 +2039,7 @@
       </c>
       <c r="F17" s="19"/>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" s="8" t="s">
         <v>71</v>
       </c>
@@ -1944,7 +2049,7 @@
       <c r="E18" s="12"/>
       <c r="F18" s="1"/>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" s="3" t="s">
         <v>61</v>
       </c>
@@ -1964,7 +2069,7 @@
         <v>0.87</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" s="3" t="s">
         <v>66</v>
       </c>
@@ -1984,7 +2089,7 @@
         <v>0.93</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" s="3" t="s">
         <v>67</v>
       </c>
@@ -2004,7 +2109,7 @@
         <v>1.18</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" s="3" t="s">
         <v>62</v>
       </c>
@@ -2024,7 +2129,7 @@
         <v>1.24</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23" s="8" t="s">
         <v>72</v>
       </c>
@@ -2034,7 +2139,7 @@
       <c r="E23" s="12"/>
       <c r="F23" s="1"/>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" s="3" t="s">
         <v>61</v>
       </c>
@@ -2054,7 +2159,7 @@
         <v>0.88</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" s="3" t="s">
         <v>66</v>
       </c>
@@ -2074,7 +2179,7 @@
         <v>0.88</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" s="3" t="s">
         <v>67</v>
       </c>
@@ -2094,7 +2199,7 @@
         <v>1.1299999999999999</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27" s="7" t="s">
         <v>62</v>
       </c>
@@ -2114,7 +2219,7 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="28" spans="1:6" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" ht="18" x14ac:dyDescent="0.2">
       <c r="A28" s="4"/>
       <c r="B28" s="1"/>
       <c r="C28" s="1"/>
@@ -2122,7 +2227,7 @@
       <c r="E28" s="1"/>
       <c r="F28" s="1"/>
     </row>
-    <row r="29" spans="1:6" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" ht="18" x14ac:dyDescent="0.2">
       <c r="A29" s="4"/>
       <c r="B29" s="1"/>
       <c r="C29" s="1"/>
@@ -2138,11 +2243,11 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A749072B-F938-0F49-BE23-243603B2B3D0}">
   <dimension ref="M2"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="2" spans="13:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="13:13" x14ac:dyDescent="0.2">
       <c r="M2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
   </sheetData>
@@ -2154,7 +2259,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45875D41-9C56-AA4E-A18A-2D3A4CE169B3}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2164,7 +2269,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A2A5153E-6E5C-054A-8ACA-5118463B96C5}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2174,142 +2279,142 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BBA86F85-A8D4-F648-84C3-730F1A42C846}">
   <dimension ref="A1:AM34"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.125" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="6.5" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="1.125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="1.1640625" style="1" customWidth="1"/>
     <col min="8" max="8" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="5.125" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="5.625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="5.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="5.6640625" style="1" customWidth="1"/>
     <col min="11" max="11" width="6.5" style="1" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="1.125" style="1" customWidth="1"/>
+    <col min="13" max="13" width="1.1640625" style="1" customWidth="1"/>
     <col min="14" max="14" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="5.125" style="1" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="5.625" style="1" customWidth="1"/>
+    <col min="15" max="15" width="5.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="5.6640625" style="1" customWidth="1"/>
     <col min="17" max="17" width="6.5" style="1" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="0.875" style="1" customWidth="1"/>
+    <col min="19" max="19" width="0.83203125" style="1" customWidth="1"/>
     <col min="20" max="20" width="8.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="5.125" style="1" bestFit="1" customWidth="1"/>
-    <col min="22" max="23" width="5.625" style="1" customWidth="1"/>
-    <col min="24" max="24" width="6.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="5.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="22" max="23" width="5.6640625" style="1" customWidth="1"/>
+    <col min="24" max="24" width="6.1640625" style="1" bestFit="1" customWidth="1"/>
     <col min="25" max="25" width="1" style="1" customWidth="1"/>
     <col min="26" max="26" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="5.125" style="1" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="5.625" style="1" customWidth="1"/>
+    <col min="27" max="27" width="5.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="5.6640625" style="1" customWidth="1"/>
     <col min="29" max="30" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="1.125" style="1" customWidth="1"/>
+    <col min="31" max="31" width="1.1640625" style="1" customWidth="1"/>
     <col min="32" max="32" width="7" style="1" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="5.125" style="1" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="5.625" style="1" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="5.625" style="1" customWidth="1"/>
-    <col min="36" max="36" width="6.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="5.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="5.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="5.6640625" style="1" customWidth="1"/>
+    <col min="36" max="36" width="6.1640625" style="1" bestFit="1" customWidth="1"/>
     <col min="37" max="16384" width="11" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="2" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A2" s="14"/>
-      <c r="B2" s="31" t="s">
+      <c r="B2" s="32" t="s">
+        <v>113</v>
+      </c>
+      <c r="C2" s="32"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
+      <c r="F2" s="32"/>
+      <c r="G2" s="32"/>
+      <c r="H2" s="32"/>
+      <c r="I2" s="32"/>
+      <c r="J2" s="32"/>
+      <c r="K2" s="32"/>
+      <c r="L2" s="32"/>
+      <c r="M2" s="32"/>
+      <c r="N2" s="32"/>
+      <c r="O2" s="32"/>
+      <c r="P2" s="32"/>
+      <c r="Q2" s="32"/>
+      <c r="R2" s="32"/>
+      <c r="S2" s="9"/>
+      <c r="T2" s="32" t="s">
         <v>114</v>
       </c>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
-      <c r="F2" s="31"/>
-      <c r="G2" s="31"/>
-      <c r="H2" s="31"/>
-      <c r="I2" s="31"/>
-      <c r="J2" s="31"/>
-      <c r="K2" s="31"/>
-      <c r="L2" s="31"/>
-      <c r="M2" s="31"/>
-      <c r="N2" s="31"/>
-      <c r="O2" s="31"/>
-      <c r="P2" s="31"/>
-      <c r="Q2" s="31"/>
-      <c r="R2" s="31"/>
-      <c r="S2" s="9"/>
-      <c r="T2" s="31" t="s">
-        <v>115</v>
-      </c>
-      <c r="U2" s="31"/>
-      <c r="V2" s="31"/>
-      <c r="W2" s="31"/>
-      <c r="X2" s="31"/>
-      <c r="Y2" s="31"/>
-      <c r="Z2" s="31"/>
-      <c r="AA2" s="31"/>
-      <c r="AB2" s="31"/>
-      <c r="AC2" s="31"/>
-      <c r="AD2" s="31"/>
-      <c r="AE2" s="31"/>
-      <c r="AF2" s="31"/>
-      <c r="AG2" s="31"/>
-      <c r="AH2" s="31"/>
-      <c r="AI2" s="31"/>
-      <c r="AJ2" s="31"/>
-    </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="U2" s="32"/>
+      <c r="V2" s="32"/>
+      <c r="W2" s="32"/>
+      <c r="X2" s="32"/>
+      <c r="Y2" s="32"/>
+      <c r="Z2" s="32"/>
+      <c r="AA2" s="32"/>
+      <c r="AB2" s="32"/>
+      <c r="AC2" s="32"/>
+      <c r="AD2" s="32"/>
+      <c r="AE2" s="32"/>
+      <c r="AF2" s="32"/>
+      <c r="AG2" s="32"/>
+      <c r="AH2" s="32"/>
+      <c r="AI2" s="32"/>
+      <c r="AJ2" s="32"/>
+    </row>
+    <row r="3" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A3" s="16"/>
-      <c r="B3" s="31" t="s">
+      <c r="B3" s="32" t="s">
         <v>79</v>
       </c>
-      <c r="C3" s="31"/>
-      <c r="D3" s="31"/>
-      <c r="E3" s="31"/>
-      <c r="F3" s="31"/>
+      <c r="C3" s="32"/>
+      <c r="D3" s="32"/>
+      <c r="E3" s="32"/>
+      <c r="F3" s="32"/>
       <c r="G3" s="28"/>
-      <c r="H3" s="31" t="s">
+      <c r="H3" s="32" t="s">
         <v>80</v>
       </c>
-      <c r="I3" s="31"/>
-      <c r="J3" s="31"/>
-      <c r="K3" s="31"/>
-      <c r="L3" s="31"/>
+      <c r="I3" s="32"/>
+      <c r="J3" s="32"/>
+      <c r="K3" s="32"/>
+      <c r="L3" s="32"/>
       <c r="M3" s="28"/>
-      <c r="N3" s="31" t="s">
+      <c r="N3" s="32" t="s">
         <v>81</v>
       </c>
-      <c r="O3" s="31"/>
-      <c r="P3" s="31"/>
-      <c r="Q3" s="31"/>
-      <c r="R3" s="31"/>
-      <c r="T3" s="32" t="s">
+      <c r="O3" s="32"/>
+      <c r="P3" s="32"/>
+      <c r="Q3" s="32"/>
+      <c r="R3" s="32"/>
+      <c r="T3" s="33" t="s">
         <v>79</v>
       </c>
-      <c r="U3" s="32"/>
-      <c r="V3" s="32"/>
-      <c r="W3" s="32"/>
-      <c r="X3" s="32"/>
+      <c r="U3" s="33"/>
+      <c r="V3" s="33"/>
+      <c r="W3" s="33"/>
+      <c r="X3" s="33"/>
       <c r="Y3" s="28"/>
-      <c r="Z3" s="31" t="s">
+      <c r="Z3" s="32" t="s">
         <v>80</v>
       </c>
-      <c r="AA3" s="31"/>
-      <c r="AB3" s="31"/>
-      <c r="AC3" s="31"/>
-      <c r="AD3" s="31"/>
+      <c r="AA3" s="32"/>
+      <c r="AB3" s="32"/>
+      <c r="AC3" s="32"/>
+      <c r="AD3" s="32"/>
       <c r="AE3" s="28"/>
-      <c r="AF3" s="31" t="s">
+      <c r="AF3" s="32" t="s">
         <v>81</v>
       </c>
-      <c r="AG3" s="31"/>
-      <c r="AH3" s="31"/>
-      <c r="AI3" s="31"/>
-      <c r="AJ3" s="31"/>
-    </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AG3" s="32"/>
+      <c r="AH3" s="32"/>
+      <c r="AI3" s="32"/>
+      <c r="AJ3" s="32"/>
+    </row>
+    <row r="4" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A4" s="15"/>
       <c r="B4" s="29" t="s">
         <v>90</v>
@@ -2321,10 +2426,10 @@
         <v>92</v>
       </c>
       <c r="E4" s="29" t="s">
+        <v>134</v>
+      </c>
+      <c r="F4" s="29" t="s">
         <v>135</v>
-      </c>
-      <c r="F4" s="29" t="s">
-        <v>136</v>
       </c>
       <c r="G4" s="29"/>
       <c r="H4" s="29" t="s">
@@ -2337,10 +2442,10 @@
         <v>92</v>
       </c>
       <c r="K4" s="29" t="s">
+        <v>134</v>
+      </c>
+      <c r="L4" s="29" t="s">
         <v>135</v>
-      </c>
-      <c r="L4" s="29" t="s">
-        <v>136</v>
       </c>
       <c r="M4" s="29"/>
       <c r="N4" s="29" t="s">
@@ -2353,10 +2458,10 @@
         <v>92</v>
       </c>
       <c r="Q4" s="29" t="s">
+        <v>134</v>
+      </c>
+      <c r="R4" s="29" t="s">
         <v>135</v>
-      </c>
-      <c r="R4" s="29" t="s">
-        <v>136</v>
       </c>
       <c r="S4" s="6"/>
       <c r="T4" s="29" t="s">
@@ -2369,10 +2474,10 @@
         <v>92</v>
       </c>
       <c r="W4" s="29" t="s">
+        <v>134</v>
+      </c>
+      <c r="X4" s="29" t="s">
         <v>135</v>
-      </c>
-      <c r="X4" s="29" t="s">
-        <v>136</v>
       </c>
       <c r="Y4" s="17"/>
       <c r="Z4" s="29" t="s">
@@ -2385,10 +2490,10 @@
         <v>92</v>
       </c>
       <c r="AC4" s="29" t="s">
+        <v>134</v>
+      </c>
+      <c r="AD4" s="29" t="s">
         <v>135</v>
-      </c>
-      <c r="AD4" s="29" t="s">
-        <v>136</v>
       </c>
       <c r="AE4" s="17"/>
       <c r="AF4" s="29" t="s">
@@ -2401,13 +2506,13 @@
         <v>92</v>
       </c>
       <c r="AI4" s="29" t="s">
+        <v>134</v>
+      </c>
+      <c r="AJ4" s="29" t="s">
         <v>135</v>
       </c>
-      <c r="AJ4" s="29" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A5" s="17" t="s">
         <v>85</v>
       </c>
@@ -2446,9 +2551,9 @@
       <c r="AI5" s="16"/>
       <c r="AJ5" s="16"/>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A6" s="16" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B6" s="16">
         <v>12.162000000000001</v>
@@ -2545,9 +2650,9 @@
         <v>12.236000000000001</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A7" s="16" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B7" s="16">
         <v>-9.1289999999999996</v>
@@ -2644,7 +2749,7 @@
         <v>-7.7560000000000002</v>
       </c>
     </row>
-    <row r="8" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A8" s="16"/>
       <c r="B8" s="16"/>
       <c r="C8" s="16"/>
@@ -2681,7 +2786,7 @@
       <c r="AI8" s="18"/>
       <c r="AJ8" s="16"/>
     </row>
-    <row r="9" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A9" s="17" t="s">
         <v>86</v>
       </c>
@@ -2720,9 +2825,9 @@
       <c r="AI9" s="16"/>
       <c r="AJ9" s="16"/>
     </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A10" s="16" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B10" s="16">
         <v>-0.312</v>
@@ -2819,9 +2924,9 @@
         <v>-0.24</v>
       </c>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A11" s="16" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B11" s="16">
         <v>0.13200000000000001</v>
@@ -2918,9 +3023,9 @@
         <v>0.09</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A12" s="16" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B12" s="16">
         <v>0.16300000000000001</v>
@@ -3017,9 +3122,9 @@
         <v>0.14899999999999999</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A13" s="16" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B13" s="16">
         <v>-5.5E-2</v>
@@ -3116,7 +3221,7 @@
         <v>3.5999999999999997E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A14" s="16" t="s">
         <v>88</v>
       </c>
@@ -3215,7 +3320,7 @@
         <v>0.28799999999999998</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A15" s="16"/>
       <c r="B15" s="16"/>
       <c r="C15" s="16"/>
@@ -3252,7 +3357,7 @@
       <c r="AI15" s="18"/>
       <c r="AJ15" s="16"/>
     </row>
-    <row r="16" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A16" s="17" t="s">
         <v>87</v>
       </c>
@@ -3291,9 +3396,9 @@
       <c r="AI16" s="16"/>
       <c r="AJ16" s="16"/>
     </row>
-    <row r="17" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A17" s="16" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B17" s="16">
         <v>0.34100000000000003</v>
@@ -3390,9 +3495,9 @@
         <v>0.443</v>
       </c>
     </row>
-    <row r="18" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A18" s="16" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B18" s="16" t="s">
         <v>94</v>
@@ -3489,9 +3594,9 @@
         <v>-0.10299999999999999</v>
       </c>
     </row>
-    <row r="19" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A19" s="16" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B19" s="16" t="s">
         <v>94</v>
@@ -3588,9 +3693,9 @@
         <v>9.0999999999999998E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A20" s="16" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B20" s="16" t="s">
         <v>94</v>
@@ -3687,9 +3792,9 @@
         <v>3.1E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A21" s="16" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B21" s="16" t="s">
         <v>94</v>
@@ -3786,9 +3891,9 @@
         <v>-0.13600000000000001</v>
       </c>
     </row>
-    <row r="22" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A22" s="16" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B22" s="16" t="s">
         <v>94</v>
@@ -3883,9 +3988,9 @@
         <v>0.156</v>
       </c>
     </row>
-    <row r="23" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A23" s="16" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B23" s="16" t="s">
         <v>94</v>
@@ -3980,9 +4085,9 @@
         <v>-1.6E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A24" s="16" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B24" s="16" t="s">
         <v>94</v>
@@ -4077,9 +4182,9 @@
         <v>0.112</v>
       </c>
     </row>
-    <row r="25" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A25" s="16" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B25" s="16" t="s">
         <v>94</v>
@@ -4174,9 +4279,9 @@
         <v>0.16</v>
       </c>
     </row>
-    <row r="26" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A26" s="16" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B26" s="16" t="s">
         <v>94</v>
@@ -4271,7 +4376,7 @@
         <v>-4.9000000000000002E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A27" s="16"/>
       <c r="B27" s="16"/>
       <c r="C27" s="16"/>
@@ -4308,7 +4413,7 @@
       <c r="AI27" s="18"/>
       <c r="AJ27" s="16"/>
     </row>
-    <row r="28" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A28" s="17" t="s">
         <v>82</v>
       </c>
@@ -4347,7 +4452,7 @@
       <c r="AI28" s="16"/>
       <c r="AJ28" s="16"/>
     </row>
-    <row r="29" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A29" s="16" t="s">
         <v>84</v>
       </c>
@@ -4446,7 +4551,7 @@
         <v>14.164999999999999</v>
       </c>
     </row>
-    <row r="30" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A30" s="16" t="s">
         <v>89</v>
       </c>
@@ -4545,7 +4650,7 @@
         <v>4.1660000000000004</v>
       </c>
     </row>
-    <row r="31" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A31" s="16" t="s">
         <v>93</v>
       </c>
@@ -4644,9 +4749,9 @@
         <v>1.0549999999999999</v>
       </c>
     </row>
-    <row r="32" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A32" s="16" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B32" s="16" t="s">
         <v>94</v>
@@ -4741,9 +4846,9 @@
         <v>4.202</v>
       </c>
     </row>
-    <row r="33" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:39" x14ac:dyDescent="0.2">
       <c r="A33" s="20" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B33" s="14"/>
       <c r="C33" s="14"/>
@@ -4784,69 +4889,63 @@
       <c r="AL33" s="16"/>
       <c r="AM33" s="16"/>
     </row>
-    <row r="34" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:39" x14ac:dyDescent="0.2">
       <c r="A34" s="15" t="s">
-        <v>118</v>
-      </c>
-      <c r="B34" s="33">
+        <v>117</v>
+      </c>
+      <c r="B34" s="31">
         <v>74058.118000000002</v>
       </c>
-      <c r="C34" s="33"/>
-      <c r="D34" s="33"/>
-      <c r="E34" s="33"/>
-      <c r="F34" s="33"/>
+      <c r="C34" s="31"/>
+      <c r="D34" s="31"/>
+      <c r="E34" s="31"/>
+      <c r="F34" s="31"/>
       <c r="G34" s="27"/>
-      <c r="H34" s="33">
+      <c r="H34" s="31">
         <v>83016.937999999995</v>
       </c>
-      <c r="I34" s="33"/>
-      <c r="J34" s="33"/>
-      <c r="K34" s="33"/>
-      <c r="L34" s="33"/>
+      <c r="I34" s="31"/>
+      <c r="J34" s="31"/>
+      <c r="K34" s="31"/>
+      <c r="L34" s="31"/>
       <c r="M34" s="27"/>
-      <c r="N34" s="33">
+      <c r="N34" s="31">
         <v>94345.274999999994</v>
       </c>
-      <c r="O34" s="33"/>
-      <c r="P34" s="33"/>
-      <c r="Q34" s="33"/>
-      <c r="R34" s="33"/>
+      <c r="O34" s="31"/>
+      <c r="P34" s="31"/>
+      <c r="Q34" s="31"/>
+      <c r="R34" s="31"/>
       <c r="S34" s="15"/>
-      <c r="T34" s="33">
+      <c r="T34" s="31">
         <v>83167.763000000006</v>
       </c>
-      <c r="U34" s="33"/>
-      <c r="V34" s="33"/>
-      <c r="W34" s="33"/>
-      <c r="X34" s="33"/>
+      <c r="U34" s="31"/>
+      <c r="V34" s="31"/>
+      <c r="W34" s="31"/>
+      <c r="X34" s="31"/>
       <c r="Y34" s="27"/>
-      <c r="Z34" s="33">
+      <c r="Z34" s="31">
         <v>93083.505999999994</v>
       </c>
-      <c r="AA34" s="33"/>
-      <c r="AB34" s="33"/>
-      <c r="AC34" s="33"/>
-      <c r="AD34" s="33"/>
+      <c r="AA34" s="31"/>
+      <c r="AB34" s="31"/>
+      <c r="AC34" s="31"/>
+      <c r="AD34" s="31"/>
       <c r="AE34" s="27"/>
-      <c r="AF34" s="33">
+      <c r="AF34" s="31">
         <v>105770.462</v>
       </c>
-      <c r="AG34" s="33"/>
-      <c r="AH34" s="33"/>
-      <c r="AI34" s="33"/>
-      <c r="AJ34" s="33"/>
+      <c r="AG34" s="31"/>
+      <c r="AH34" s="31"/>
+      <c r="AI34" s="31"/>
+      <c r="AJ34" s="31"/>
       <c r="AK34" s="16"/>
       <c r="AL34" s="16"/>
       <c r="AM34" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="AF34:AJ34"/>
-    <mergeCell ref="B34:F34"/>
-    <mergeCell ref="H34:L34"/>
-    <mergeCell ref="T34:X34"/>
-    <mergeCell ref="N34:R34"/>
-    <mergeCell ref="Z34:AD34"/>
     <mergeCell ref="B3:F3"/>
     <mergeCell ref="B2:R2"/>
     <mergeCell ref="H3:L3"/>
@@ -4855,6 +4954,12 @@
     <mergeCell ref="T3:X3"/>
     <mergeCell ref="Z3:AD3"/>
     <mergeCell ref="AF3:AJ3"/>
+    <mergeCell ref="AF34:AJ34"/>
+    <mergeCell ref="B34:F34"/>
+    <mergeCell ref="H34:L34"/>
+    <mergeCell ref="T34:X34"/>
+    <mergeCell ref="N34:R34"/>
+    <mergeCell ref="Z34:AD34"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
@@ -4864,141 +4969,141 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CD5CF7F-81D6-D24D-8228-B4C578C35D65}">
   <dimension ref="A1:AM39"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="24" style="1" customWidth="1"/>
     <col min="2" max="2" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.125" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="5.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.6640625" style="1" customWidth="1"/>
     <col min="5" max="6" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="1.125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="1.1640625" style="1" customWidth="1"/>
     <col min="8" max="8" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="5.125" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="5.625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="5.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="5.6640625" style="1" customWidth="1"/>
     <col min="11" max="11" width="6.5" style="1" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="1.125" style="1" customWidth="1"/>
+    <col min="13" max="13" width="1.1640625" style="1" customWidth="1"/>
     <col min="14" max="14" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="5.125" style="1" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="5.625" style="1" customWidth="1"/>
+    <col min="15" max="15" width="5.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="5.6640625" style="1" customWidth="1"/>
     <col min="17" max="17" width="6.5" style="1" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="0.875" style="1" customWidth="1"/>
+    <col min="19" max="19" width="0.83203125" style="1" customWidth="1"/>
     <col min="20" max="20" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="5.875" style="1" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="6.375" style="1" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="5.625" style="1" customWidth="1"/>
+    <col min="21" max="21" width="5.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="6.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="5.6640625" style="1" customWidth="1"/>
     <col min="24" max="24" width="6" style="1" bestFit="1" customWidth="1"/>
     <col min="25" max="25" width="1" style="1" customWidth="1"/>
     <col min="26" max="26" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="5.125" style="1" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="5.625" style="1" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="5.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="5.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="29" max="30" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="1.125" style="1" customWidth="1"/>
+    <col min="31" max="31" width="1.1640625" style="1" customWidth="1"/>
     <col min="32" max="32" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="5.125" style="1" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="5.625" style="1" customWidth="1"/>
+    <col min="33" max="33" width="5.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="5.6640625" style="1" customWidth="1"/>
     <col min="35" max="36" width="6" style="1" bestFit="1" customWidth="1"/>
     <col min="37" max="16384" width="11" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="2" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A2" s="14"/>
-      <c r="B2" s="31" t="s">
+      <c r="B2" s="32" t="s">
+        <v>113</v>
+      </c>
+      <c r="C2" s="32"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
+      <c r="F2" s="32"/>
+      <c r="G2" s="32"/>
+      <c r="H2" s="32"/>
+      <c r="I2" s="32"/>
+      <c r="J2" s="32"/>
+      <c r="K2" s="32"/>
+      <c r="L2" s="32"/>
+      <c r="M2" s="32"/>
+      <c r="N2" s="32"/>
+      <c r="O2" s="32"/>
+      <c r="P2" s="32"/>
+      <c r="Q2" s="32"/>
+      <c r="R2" s="32"/>
+      <c r="S2" s="9"/>
+      <c r="T2" s="32" t="s">
         <v>114</v>
       </c>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
-      <c r="F2" s="31"/>
-      <c r="G2" s="31"/>
-      <c r="H2" s="31"/>
-      <c r="I2" s="31"/>
-      <c r="J2" s="31"/>
-      <c r="K2" s="31"/>
-      <c r="L2" s="31"/>
-      <c r="M2" s="31"/>
-      <c r="N2" s="31"/>
-      <c r="O2" s="31"/>
-      <c r="P2" s="31"/>
-      <c r="Q2" s="31"/>
-      <c r="R2" s="31"/>
-      <c r="S2" s="9"/>
-      <c r="T2" s="31" t="s">
-        <v>115</v>
-      </c>
-      <c r="U2" s="31"/>
-      <c r="V2" s="31"/>
-      <c r="W2" s="31"/>
-      <c r="X2" s="31"/>
-      <c r="Y2" s="31"/>
-      <c r="Z2" s="31"/>
-      <c r="AA2" s="31"/>
-      <c r="AB2" s="31"/>
-      <c r="AC2" s="31"/>
-      <c r="AD2" s="31"/>
-      <c r="AE2" s="31"/>
-      <c r="AF2" s="31"/>
-      <c r="AG2" s="31"/>
-      <c r="AH2" s="31"/>
-      <c r="AI2" s="31"/>
-      <c r="AJ2" s="31"/>
-    </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="U2" s="32"/>
+      <c r="V2" s="32"/>
+      <c r="W2" s="32"/>
+      <c r="X2" s="32"/>
+      <c r="Y2" s="32"/>
+      <c r="Z2" s="32"/>
+      <c r="AA2" s="32"/>
+      <c r="AB2" s="32"/>
+      <c r="AC2" s="32"/>
+      <c r="AD2" s="32"/>
+      <c r="AE2" s="32"/>
+      <c r="AF2" s="32"/>
+      <c r="AG2" s="32"/>
+      <c r="AH2" s="32"/>
+      <c r="AI2" s="32"/>
+      <c r="AJ2" s="32"/>
+    </row>
+    <row r="3" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A3" s="16"/>
-      <c r="B3" s="31" t="s">
+      <c r="B3" s="32" t="s">
         <v>79</v>
       </c>
-      <c r="C3" s="31"/>
-      <c r="D3" s="31"/>
-      <c r="E3" s="31"/>
-      <c r="F3" s="31"/>
+      <c r="C3" s="32"/>
+      <c r="D3" s="32"/>
+      <c r="E3" s="32"/>
+      <c r="F3" s="32"/>
       <c r="G3" s="28"/>
-      <c r="H3" s="31" t="s">
+      <c r="H3" s="32" t="s">
         <v>80</v>
       </c>
-      <c r="I3" s="31"/>
-      <c r="J3" s="31"/>
-      <c r="K3" s="31"/>
-      <c r="L3" s="31"/>
+      <c r="I3" s="32"/>
+      <c r="J3" s="32"/>
+      <c r="K3" s="32"/>
+      <c r="L3" s="32"/>
       <c r="M3" s="28"/>
-      <c r="N3" s="31" t="s">
+      <c r="N3" s="32" t="s">
         <v>81</v>
       </c>
-      <c r="O3" s="31"/>
-      <c r="P3" s="31"/>
-      <c r="Q3" s="31"/>
-      <c r="R3" s="31"/>
-      <c r="T3" s="32" t="s">
+      <c r="O3" s="32"/>
+      <c r="P3" s="32"/>
+      <c r="Q3" s="32"/>
+      <c r="R3" s="32"/>
+      <c r="T3" s="33" t="s">
         <v>79</v>
       </c>
-      <c r="U3" s="32"/>
-      <c r="V3" s="32"/>
-      <c r="W3" s="32"/>
-      <c r="X3" s="32"/>
+      <c r="U3" s="33"/>
+      <c r="V3" s="33"/>
+      <c r="W3" s="33"/>
+      <c r="X3" s="33"/>
       <c r="Y3" s="28"/>
-      <c r="Z3" s="31" t="s">
+      <c r="Z3" s="32" t="s">
         <v>80</v>
       </c>
-      <c r="AA3" s="31"/>
-      <c r="AB3" s="31"/>
-      <c r="AC3" s="31"/>
-      <c r="AD3" s="31"/>
+      <c r="AA3" s="32"/>
+      <c r="AB3" s="32"/>
+      <c r="AC3" s="32"/>
+      <c r="AD3" s="32"/>
       <c r="AE3" s="28"/>
-      <c r="AF3" s="31" t="s">
+      <c r="AF3" s="32" t="s">
         <v>81</v>
       </c>
-      <c r="AG3" s="31"/>
-      <c r="AH3" s="31"/>
-      <c r="AI3" s="31"/>
-      <c r="AJ3" s="31"/>
-    </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AG3" s="32"/>
+      <c r="AH3" s="32"/>
+      <c r="AI3" s="32"/>
+      <c r="AJ3" s="32"/>
+    </row>
+    <row r="4" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A4" s="15"/>
       <c r="B4" s="29" t="s">
         <v>90</v>
@@ -5010,10 +5115,10 @@
         <v>92</v>
       </c>
       <c r="E4" s="29" t="s">
+        <v>134</v>
+      </c>
+      <c r="F4" s="29" t="s">
         <v>135</v>
-      </c>
-      <c r="F4" s="29" t="s">
-        <v>136</v>
       </c>
       <c r="G4" s="29"/>
       <c r="H4" s="29" t="s">
@@ -5026,10 +5131,10 @@
         <v>92</v>
       </c>
       <c r="K4" s="29" t="s">
+        <v>134</v>
+      </c>
+      <c r="L4" s="29" t="s">
         <v>135</v>
-      </c>
-      <c r="L4" s="29" t="s">
-        <v>136</v>
       </c>
       <c r="M4" s="29"/>
       <c r="N4" s="29" t="s">
@@ -5042,10 +5147,10 @@
         <v>92</v>
       </c>
       <c r="Q4" s="29" t="s">
+        <v>134</v>
+      </c>
+      <c r="R4" s="29" t="s">
         <v>135</v>
-      </c>
-      <c r="R4" s="29" t="s">
-        <v>136</v>
       </c>
       <c r="S4" s="6"/>
       <c r="T4" s="29" t="s">
@@ -5058,10 +5163,10 @@
         <v>92</v>
       </c>
       <c r="W4" s="29" t="s">
+        <v>134</v>
+      </c>
+      <c r="X4" s="29" t="s">
         <v>135</v>
-      </c>
-      <c r="X4" s="29" t="s">
-        <v>136</v>
       </c>
       <c r="Y4" s="17"/>
       <c r="Z4" s="29" t="s">
@@ -5074,10 +5179,10 @@
         <v>92</v>
       </c>
       <c r="AC4" s="29" t="s">
+        <v>134</v>
+      </c>
+      <c r="AD4" s="29" t="s">
         <v>135</v>
-      </c>
-      <c r="AD4" s="29" t="s">
-        <v>136</v>
       </c>
       <c r="AE4" s="17"/>
       <c r="AF4" s="29" t="s">
@@ -5090,13 +5195,13 @@
         <v>92</v>
       </c>
       <c r="AI4" s="29" t="s">
+        <v>134</v>
+      </c>
+      <c r="AJ4" s="29" t="s">
         <v>135</v>
       </c>
-      <c r="AJ4" s="29" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A5" s="17" t="s">
         <v>85</v>
       </c>
@@ -5135,9 +5240,9 @@
       <c r="AI5" s="16"/>
       <c r="AJ5" s="16"/>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A6" s="16" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B6" s="16">
         <v>13.944000000000001</v>
@@ -5214,9 +5319,9 @@
         <v>13.875999999999999</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A7" s="16" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B7" s="16">
         <v>-7.5229999999999997</v>
@@ -5293,9 +5398,9 @@
         <v>2.1219999999999999</v>
       </c>
     </row>
-    <row r="8" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A8" s="16" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B8" s="16">
         <v>-0.253</v>
@@ -5342,7 +5447,7 @@
       <c r="AI8" s="16"/>
       <c r="AJ8" s="16"/>
     </row>
-    <row r="9" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A9" s="16"/>
       <c r="B9" s="16"/>
       <c r="C9" s="16"/>
@@ -5379,7 +5484,7 @@
       <c r="AI9" s="18"/>
       <c r="AJ9" s="16"/>
     </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A10" s="17" t="s">
         <v>86</v>
       </c>
@@ -5418,9 +5523,9 @@
       <c r="AI10" s="16"/>
       <c r="AJ10" s="16"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A11" s="16" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B11" s="16" t="s">
         <v>94</v>
@@ -5517,9 +5622,9 @@
         <v>0.40300000000000002</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A12" s="16" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B12" s="16">
         <v>0.11700000000000001</v>
@@ -5566,9 +5671,9 @@
       <c r="AI12" s="16"/>
       <c r="AJ12" s="16"/>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A13" s="16" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B13" s="16">
         <v>0.02</v>
@@ -5645,9 +5750,9 @@
         <v>2.4E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A14" s="16" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B14" s="16">
         <v>6.9000000000000006E-2</v>
@@ -5724,9 +5829,9 @@
         <v>8.5999999999999993E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A15" s="16" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B15" s="16" t="s">
         <v>94</v>
@@ -5793,9 +5898,9 @@
       <c r="AI15" s="16"/>
       <c r="AJ15" s="16"/>
     </row>
-    <row r="16" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A16" s="16" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B16" s="16" t="s">
         <v>94</v>
@@ -5872,9 +5977,9 @@
         <v>0.22900000000000001</v>
       </c>
     </row>
-    <row r="17" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A17" s="16" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B17" s="16">
         <v>-0.45300000000000001</v>
@@ -5921,7 +6026,7 @@
       <c r="AI17" s="16"/>
       <c r="AJ17" s="16"/>
     </row>
-    <row r="18" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A18" s="16" t="s">
         <v>88</v>
       </c>
@@ -6000,7 +6105,7 @@
         <v>0.28799999999999998</v>
       </c>
     </row>
-    <row r="19" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A19" s="16"/>
       <c r="B19" s="16"/>
       <c r="C19" s="16"/>
@@ -6037,7 +6142,7 @@
       <c r="AI19" s="18"/>
       <c r="AJ19" s="16"/>
     </row>
-    <row r="20" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A20" s="17" t="s">
         <v>87</v>
       </c>
@@ -6076,9 +6181,9 @@
       <c r="AI20" s="16"/>
       <c r="AJ20" s="16"/>
     </row>
-    <row r="21" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A21" s="16" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B21" s="16">
         <v>-0.29099999999999998</v>
@@ -6125,9 +6230,9 @@
       <c r="AI21" s="16"/>
       <c r="AJ21" s="16"/>
     </row>
-    <row r="22" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A22" s="16" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B22" s="16" t="s">
         <v>94</v>
@@ -6224,9 +6329,9 @@
         <v>0.14499999999999999</v>
       </c>
     </row>
-    <row r="23" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A23" s="16" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B23" s="16" t="s">
         <v>94</v>
@@ -6303,9 +6408,9 @@
         <v>-9.5000000000000001E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A24" s="16" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B24" s="16" t="s">
         <v>94</v>
@@ -6382,9 +6487,9 @@
         <v>5.0999999999999997E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A25" s="16" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B25" s="16" t="s">
         <v>94</v>
@@ -6461,9 +6566,9 @@
         <v>3.2000000000000001E-2</v>
       </c>
     </row>
-    <row r="26" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A26" s="16" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B26" s="16" t="s">
         <v>94</v>
@@ -6540,9 +6645,9 @@
         <v>-0.13600000000000001</v>
       </c>
     </row>
-    <row r="27" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A27" s="16" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B27" s="16" t="s">
         <v>94</v>
@@ -6627,9 +6732,9 @@
         <v>0.17199999999999999</v>
       </c>
     </row>
-    <row r="28" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A28" s="16" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B28" s="16" t="s">
         <v>94</v>
@@ -6714,9 +6819,9 @@
         <v>3.5999999999999997E-2</v>
       </c>
     </row>
-    <row r="29" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A29" s="16" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B29" s="16" t="s">
         <v>94</v>
@@ -6801,9 +6906,9 @@
         <v>7.4999999999999997E-2</v>
       </c>
     </row>
-    <row r="30" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A30" s="16" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B30" s="16" t="s">
         <v>94</v>
@@ -6888,9 +6993,9 @@
         <v>0.17499999999999999</v>
       </c>
     </row>
-    <row r="31" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A31" s="16" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B31" s="16" t="s">
         <v>94</v>
@@ -6975,7 +7080,7 @@
         <v>-0.05</v>
       </c>
     </row>
-    <row r="32" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A32" s="16"/>
       <c r="B32" s="16"/>
       <c r="C32" s="16"/>
@@ -7012,7 +7117,7 @@
       <c r="AI32" s="18"/>
       <c r="AJ32" s="16"/>
     </row>
-    <row r="33" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:39" x14ac:dyDescent="0.2">
       <c r="A33" s="17" t="s">
         <v>82</v>
       </c>
@@ -7051,7 +7156,7 @@
       <c r="AI33" s="16"/>
       <c r="AJ33" s="16"/>
     </row>
-    <row r="34" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:39" x14ac:dyDescent="0.2">
       <c r="A34" s="16" t="s">
         <v>84</v>
       </c>
@@ -7130,7 +7235,7 @@
         <v>14.162000000000001</v>
       </c>
     </row>
-    <row r="35" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:39" x14ac:dyDescent="0.2">
       <c r="A35" s="16" t="s">
         <v>89</v>
       </c>
@@ -7209,7 +7314,7 @@
         <v>4.1660000000000004</v>
       </c>
     </row>
-    <row r="36" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:39" x14ac:dyDescent="0.2">
       <c r="A36" s="16" t="s">
         <v>93</v>
       </c>
@@ -7288,9 +7393,9 @@
         <v>1.0549999999999999</v>
       </c>
     </row>
-    <row r="37" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:39" x14ac:dyDescent="0.2">
       <c r="A37" s="16" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B37" s="16" t="s">
         <v>94</v>
@@ -7375,9 +7480,9 @@
         <v>4.5090000000000003</v>
       </c>
     </row>
-    <row r="38" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:39" x14ac:dyDescent="0.2">
       <c r="A38" s="20" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B38" s="14"/>
       <c r="C38" s="14"/>
@@ -7418,53 +7523,53 @@
       <c r="AL38" s="16"/>
       <c r="AM38" s="16"/>
     </row>
-    <row r="39" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:39" x14ac:dyDescent="0.2">
       <c r="A39" s="15" t="s">
-        <v>118</v>
-      </c>
-      <c r="B39" s="33">
+        <v>117</v>
+      </c>
+      <c r="B39" s="31">
         <v>34697.703999999998</v>
       </c>
-      <c r="C39" s="33"/>
-      <c r="D39" s="33"/>
-      <c r="E39" s="33"/>
-      <c r="F39" s="33"/>
+      <c r="C39" s="31"/>
+      <c r="D39" s="31"/>
+      <c r="E39" s="31"/>
+      <c r="F39" s="31"/>
       <c r="G39" s="27"/>
-      <c r="H39" s="33"/>
-      <c r="I39" s="33"/>
-      <c r="J39" s="33"/>
-      <c r="K39" s="33"/>
-      <c r="L39" s="33"/>
+      <c r="H39" s="31"/>
+      <c r="I39" s="31"/>
+      <c r="J39" s="31"/>
+      <c r="K39" s="31"/>
+      <c r="L39" s="31"/>
       <c r="M39" s="27"/>
-      <c r="N39" s="33"/>
-      <c r="O39" s="33"/>
-      <c r="P39" s="33"/>
-      <c r="Q39" s="33"/>
-      <c r="R39" s="33"/>
+      <c r="N39" s="31"/>
+      <c r="O39" s="31"/>
+      <c r="P39" s="31"/>
+      <c r="Q39" s="31"/>
+      <c r="R39" s="31"/>
       <c r="S39" s="15"/>
-      <c r="T39" s="33">
+      <c r="T39" s="31">
         <v>37782.404000000002</v>
       </c>
-      <c r="U39" s="33"/>
-      <c r="V39" s="33"/>
-      <c r="W39" s="33"/>
-      <c r="X39" s="33"/>
+      <c r="U39" s="31"/>
+      <c r="V39" s="31"/>
+      <c r="W39" s="31"/>
+      <c r="X39" s="31"/>
       <c r="Y39" s="27"/>
-      <c r="Z39" s="33">
+      <c r="Z39" s="31">
         <v>47698.324999999997</v>
       </c>
-      <c r="AA39" s="33"/>
-      <c r="AB39" s="33"/>
-      <c r="AC39" s="33"/>
-      <c r="AD39" s="33"/>
+      <c r="AA39" s="31"/>
+      <c r="AB39" s="31"/>
+      <c r="AC39" s="31"/>
+      <c r="AD39" s="31"/>
       <c r="AE39" s="27"/>
-      <c r="AF39" s="33">
+      <c r="AF39" s="31">
         <v>60402.93</v>
       </c>
-      <c r="AG39" s="33"/>
-      <c r="AH39" s="33"/>
-      <c r="AI39" s="33"/>
-      <c r="AJ39" s="33"/>
+      <c r="AG39" s="31"/>
+      <c r="AH39" s="31"/>
+      <c r="AI39" s="31"/>
+      <c r="AJ39" s="31"/>
       <c r="AK39" s="16"/>
       <c r="AL39" s="16"/>
       <c r="AM39" s="16"/>
@@ -7493,604 +7598,601 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57A86273-0E84-8246-B3ED-A023C6721217}">
-  <dimension ref="A1:M38"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:L38"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="4.625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="5.875" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.5" style="1" customWidth="1"/>
-    <col min="7" max="7" width="7" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="5.125" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="5.625" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="6.125" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="16384" width="11" style="1"/>
+    <col min="1" max="1" width="19.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.1640625" style="38" customWidth="1"/>
+    <col min="3" max="3" width="4.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="5.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.5" style="35" customWidth="1"/>
+    <col min="7" max="7" width="11" style="1"/>
+    <col min="8" max="8" width="6.1640625" style="38" customWidth="1"/>
+    <col min="9" max="9" width="4.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="5.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="5.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="7.5" style="35" customWidth="1"/>
+    <col min="13" max="16384" width="11" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A2" s="14"/>
+      <c r="B2" s="43"/>
+      <c r="C2" s="32"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
+      <c r="F2" s="44"/>
+      <c r="H2" s="43"/>
+      <c r="I2" s="32"/>
+      <c r="J2" s="32"/>
+      <c r="K2" s="32"/>
+      <c r="L2" s="44"/>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A3" s="15"/>
+      <c r="B3" s="43" t="s">
+        <v>143</v>
+      </c>
+      <c r="C3" s="32"/>
+      <c r="D3" s="32"/>
+      <c r="E3" s="32"/>
+      <c r="F3" s="44"/>
+      <c r="H3" s="43" t="s">
+        <v>142</v>
+      </c>
+      <c r="I3" s="32"/>
+      <c r="J3" s="32"/>
+      <c r="K3" s="32"/>
+      <c r="L3" s="44"/>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A4" s="16"/>
+      <c r="B4" s="34" t="s">
+        <v>90</v>
+      </c>
+      <c r="C4" s="34" t="s">
+        <v>91</v>
+      </c>
+      <c r="D4" s="34" t="s">
+        <v>92</v>
+      </c>
+      <c r="E4" s="34" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="14"/>
-      <c r="B2" s="34"/>
-      <c r="C2" s="34"/>
-      <c r="D2" s="34"/>
-      <c r="E2" s="34"/>
-      <c r="G2" s="34"/>
-      <c r="H2" s="34"/>
-      <c r="I2" s="34"/>
-      <c r="J2" s="34"/>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A3" s="15"/>
-      <c r="B3" s="35" t="s">
-        <v>81</v>
-      </c>
-      <c r="C3" s="35"/>
-      <c r="D3" s="35"/>
-      <c r="E3" s="35"/>
-      <c r="G3" s="35" t="s">
-        <v>81</v>
-      </c>
-      <c r="H3" s="35"/>
-      <c r="I3" s="35"/>
-      <c r="J3" s="35"/>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" s="16"/>
-      <c r="B4" s="17" t="s">
+      <c r="F4" s="34" t="s">
+        <v>135</v>
+      </c>
+      <c r="H4" s="34" t="s">
         <v>90</v>
       </c>
-      <c r="C4" s="17" t="s">
+      <c r="I4" s="34" t="s">
         <v>91</v>
       </c>
-      <c r="D4" s="17" t="s">
+      <c r="J4" s="34" t="s">
         <v>92</v>
       </c>
-      <c r="E4" s="17" t="s">
-        <v>95</v>
-      </c>
-      <c r="G4" s="17" t="s">
-        <v>90</v>
-      </c>
-      <c r="H4" s="17" t="s">
-        <v>91</v>
-      </c>
-      <c r="I4" s="17" t="s">
-        <v>92</v>
-      </c>
-      <c r="J4" s="17" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K4" s="34" t="s">
+        <v>134</v>
+      </c>
+      <c r="L4" s="34" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" s="17" t="s">
         <v>85</v>
       </c>
-      <c r="B5" s="16"/>
-      <c r="C5" s="16"/>
-      <c r="D5" s="16"/>
       <c r="E5" s="16"/>
-      <c r="G5" s="16"/>
-      <c r="H5" s="16"/>
+      <c r="H5" s="39"/>
       <c r="I5" s="16"/>
       <c r="J5" s="16"/>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K5" s="16"/>
+    </row>
+    <row r="6" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A6" s="16" t="s">
+        <v>95</v>
+      </c>
+      <c r="B6" s="39" t="s">
+        <v>144</v>
+      </c>
+      <c r="C6" s="16">
+        <v>0.17599999999999999</v>
+      </c>
+      <c r="D6" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="E6" s="16"/>
+      <c r="H6" s="39"/>
+      <c r="I6" s="16"/>
+      <c r="J6" s="18"/>
+      <c r="K6" s="16"/>
+    </row>
+    <row r="7" spans="1:12" ht="17" x14ac:dyDescent="0.25">
+      <c r="A7" s="16" t="s">
         <v>96</v>
       </c>
-      <c r="B6" s="16"/>
-      <c r="C6" s="16"/>
-      <c r="D6" s="18"/>
-      <c r="E6" s="16"/>
-      <c r="G6" s="16"/>
-      <c r="H6" s="16"/>
-      <c r="I6" s="18"/>
-      <c r="J6" s="16"/>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A7" s="16" t="s">
-        <v>97</v>
-      </c>
-      <c r="B7" s="16"/>
-      <c r="C7" s="16"/>
-      <c r="D7" s="18"/>
+      <c r="B7" s="39">
+        <v>-9.1010000000000009</v>
+      </c>
+      <c r="C7" s="16">
+        <v>0.74299999999999999</v>
+      </c>
+      <c r="D7" s="16" t="s">
+        <v>24</v>
+      </c>
       <c r="E7" s="16"/>
-      <c r="G7" s="16"/>
-      <c r="H7" s="16"/>
-      <c r="I7" s="18"/>
-      <c r="J7" s="16"/>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="H7" s="39"/>
+      <c r="I7" s="16"/>
+      <c r="J7" s="18"/>
+      <c r="K7" s="16"/>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A8" s="17" t="s">
         <v>86</v>
       </c>
-      <c r="B8" s="16"/>
+      <c r="B8" s="39"/>
       <c r="C8" s="16"/>
       <c r="D8" s="16"/>
       <c r="E8" s="16"/>
-      <c r="G8" s="16"/>
-      <c r="H8" s="16"/>
+      <c r="H8" s="39"/>
       <c r="I8" s="16"/>
       <c r="J8" s="16"/>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K8" s="16"/>
+    </row>
+    <row r="9" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A9" s="16" t="s">
+        <v>97</v>
+      </c>
+      <c r="B9" s="39">
+        <v>-0.28799999999999998</v>
+      </c>
+      <c r="C9" s="16">
+        <v>3.9E-2</v>
+      </c>
+      <c r="D9" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="E9" s="16"/>
+      <c r="H9" s="39"/>
+      <c r="I9" s="16"/>
+      <c r="J9" s="18"/>
+      <c r="K9" s="16"/>
+    </row>
+    <row r="10" spans="1:12" ht="17" x14ac:dyDescent="0.25">
+      <c r="A10" s="16" t="s">
         <v>98</v>
       </c>
-      <c r="B9" s="16"/>
-      <c r="C9" s="16"/>
-      <c r="D9" s="18"/>
-      <c r="E9" s="16"/>
-      <c r="G9" s="16"/>
-      <c r="H9" s="16"/>
-      <c r="I9" s="18"/>
-      <c r="J9" s="16"/>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A10" s="16" t="s">
-        <v>99</v>
-      </c>
-      <c r="B10" s="16">
-        <v>2.3919999999999999</v>
-      </c>
-      <c r="C10" s="16"/>
+      <c r="B10" s="39">
+        <v>5.2999999999999999E-2</v>
+      </c>
+      <c r="C10" s="16">
+        <v>2.1000000000000001E-2</v>
+      </c>
       <c r="D10" s="18">
         <v>1.0999999999999999E-2</v>
       </c>
       <c r="E10" s="16"/>
-      <c r="G10" s="16"/>
-      <c r="H10" s="16"/>
-      <c r="I10" s="18"/>
-      <c r="J10" s="16"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="H10" s="39"/>
+      <c r="I10" s="16"/>
+      <c r="J10" s="18"/>
+      <c r="K10" s="16"/>
+    </row>
+    <row r="11" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A11" s="16" t="s">
+        <v>99</v>
+      </c>
+      <c r="B11" s="39">
+        <v>0.124</v>
+      </c>
+      <c r="C11" s="16">
+        <v>2.1000000000000001E-2</v>
+      </c>
+      <c r="D11" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="E11" s="16"/>
+      <c r="H11" s="39"/>
+      <c r="I11" s="16"/>
+      <c r="J11" s="18"/>
+      <c r="K11" s="16"/>
+    </row>
+    <row r="12" spans="1:12" ht="17" x14ac:dyDescent="0.25">
+      <c r="A12" s="46" t="s">
         <v>100</v>
       </c>
-      <c r="B11" s="16">
-        <v>0.76400000000000001</v>
-      </c>
-      <c r="C11" s="16"/>
-      <c r="D11" s="18" t="s">
-        <v>24</v>
-      </c>
-      <c r="E11" s="16"/>
-      <c r="G11" s="16"/>
-      <c r="H11" s="16"/>
-      <c r="I11" s="18"/>
-      <c r="J11" s="16"/>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A12" s="25" t="s">
-        <v>101</v>
-      </c>
-      <c r="B12" s="25">
-        <v>-4.1000000000000002E-2</v>
-      </c>
-      <c r="C12" s="25"/>
+      <c r="B12" s="40">
+        <v>-3.2000000000000001E-2</v>
+      </c>
+      <c r="C12" s="25">
+        <v>3.9E-2</v>
+      </c>
       <c r="D12" s="26">
-        <v>0.40300000000000002</v>
+        <v>0.40699999999999997</v>
       </c>
       <c r="E12" s="16"/>
-      <c r="G12" s="16"/>
-      <c r="H12" s="16"/>
-      <c r="I12" s="18"/>
-      <c r="J12" s="16"/>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="H12" s="45"/>
+      <c r="I12" s="46"/>
+      <c r="J12" s="47"/>
+      <c r="K12" s="16"/>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A13" s="16" t="s">
         <v>88</v>
       </c>
-      <c r="B13" s="16">
-        <v>0.03</v>
-      </c>
+      <c r="B13" s="39"/>
       <c r="C13" s="16"/>
-      <c r="D13" s="18" t="s">
-        <v>24</v>
-      </c>
+      <c r="D13" s="18"/>
       <c r="E13" s="16"/>
-      <c r="G13" s="16"/>
-      <c r="H13" s="16"/>
-      <c r="I13" s="18"/>
-      <c r="J13" s="16"/>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="H13" s="39"/>
+      <c r="I13" s="16"/>
+      <c r="J13" s="18"/>
+      <c r="K13" s="16"/>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A14" s="17" t="s">
         <v>87</v>
       </c>
-      <c r="B14" s="16"/>
+      <c r="B14" s="39"/>
       <c r="C14" s="16"/>
       <c r="D14" s="16"/>
       <c r="E14" s="16"/>
-      <c r="G14" s="16"/>
-      <c r="H14" s="16"/>
+      <c r="H14" s="39"/>
       <c r="I14" s="16"/>
       <c r="J14" s="16"/>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K14" s="16"/>
+    </row>
+    <row r="15" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A15" s="16" t="s">
-        <v>102</v>
-      </c>
-      <c r="B15" s="16">
-        <v>3.1</v>
-      </c>
+        <v>101</v>
+      </c>
+      <c r="B15" s="39"/>
       <c r="C15" s="16"/>
       <c r="D15" s="18" t="s">
         <v>24</v>
       </c>
       <c r="E15" s="16"/>
-      <c r="G15" s="16"/>
-      <c r="H15" s="16"/>
-      <c r="I15" s="18"/>
-      <c r="J15" s="16"/>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="H15" s="39"/>
+      <c r="I15" s="16"/>
+      <c r="J15" s="18"/>
+      <c r="K15" s="16"/>
+    </row>
+    <row r="16" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A16" s="16" t="s">
-        <v>103</v>
-      </c>
-      <c r="B16" s="16"/>
+        <v>102</v>
+      </c>
+      <c r="B16" s="39"/>
       <c r="C16" s="16"/>
       <c r="D16" s="18"/>
       <c r="E16" s="16"/>
-      <c r="G16" s="16"/>
-      <c r="H16" s="16"/>
-      <c r="I16" s="18"/>
-      <c r="J16" s="16"/>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="H16" s="39"/>
+      <c r="I16" s="16"/>
+      <c r="J16" s="18"/>
+      <c r="K16" s="16"/>
+    </row>
+    <row r="17" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A17" s="16" t="s">
-        <v>104</v>
-      </c>
-      <c r="B17" s="16"/>
+        <v>103</v>
+      </c>
+      <c r="B17" s="39"/>
       <c r="C17" s="16"/>
       <c r="D17" s="18"/>
       <c r="E17" s="16"/>
-      <c r="G17" s="16"/>
-      <c r="H17" s="16"/>
-      <c r="I17" s="18"/>
-      <c r="J17" s="16"/>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="H17" s="39"/>
+      <c r="I17" s="16"/>
+      <c r="J17" s="18"/>
+      <c r="K17" s="16"/>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A18" s="16" t="s">
-        <v>107</v>
-      </c>
-      <c r="B18" s="16">
-        <v>-7.8E-2</v>
-      </c>
+        <v>106</v>
+      </c>
+      <c r="B18" s="39"/>
       <c r="C18" s="16"/>
       <c r="D18" s="18" t="s">
         <v>24</v>
       </c>
       <c r="E18" s="16"/>
-      <c r="G18" s="16"/>
-      <c r="H18" s="16"/>
-      <c r="I18" s="18"/>
-      <c r="J18" s="16"/>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="H18" s="39"/>
+      <c r="I18" s="16"/>
+      <c r="J18" s="18"/>
+      <c r="K18" s="16"/>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19" s="16" t="s">
-        <v>108</v>
-      </c>
-      <c r="B19" s="16">
-        <v>-1.2E-2</v>
-      </c>
+        <v>107</v>
+      </c>
+      <c r="B19" s="39"/>
       <c r="C19" s="16"/>
       <c r="D19" s="18" t="s">
         <v>24</v>
       </c>
       <c r="E19" s="16"/>
-      <c r="G19" s="16"/>
-      <c r="H19" s="16"/>
-      <c r="I19" s="18"/>
-      <c r="J19" s="16"/>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="H19" s="39"/>
+      <c r="I19" s="16"/>
+      <c r="J19" s="18"/>
+      <c r="K19" s="16"/>
+    </row>
+    <row r="20" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A20" s="16" t="s">
-        <v>105</v>
-      </c>
-      <c r="B20" s="16"/>
+        <v>104</v>
+      </c>
+      <c r="B20" s="39"/>
       <c r="C20" s="16"/>
       <c r="D20" s="18"/>
       <c r="E20" s="16"/>
-      <c r="G20" s="16"/>
-      <c r="H20" s="16"/>
-      <c r="I20" s="18"/>
-      <c r="J20" s="16"/>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="H20" s="39"/>
+      <c r="I20" s="16"/>
+      <c r="J20" s="18"/>
+      <c r="K20" s="16"/>
+    </row>
+    <row r="21" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A21" s="16" t="s">
-        <v>106</v>
-      </c>
-      <c r="B21" s="16"/>
+        <v>105</v>
+      </c>
+      <c r="B21" s="39"/>
       <c r="C21" s="16"/>
       <c r="D21" s="18"/>
       <c r="E21" s="16"/>
-      <c r="G21" s="16"/>
-      <c r="H21" s="16"/>
-      <c r="I21" s="18"/>
-      <c r="J21" s="16"/>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="H21" s="39"/>
+      <c r="I21" s="16"/>
+      <c r="J21" s="18"/>
+      <c r="K21" s="16"/>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22" s="16" t="s">
-        <v>110</v>
-      </c>
-      <c r="B22" s="16">
-        <v>4.7E-2</v>
-      </c>
+        <v>109</v>
+      </c>
+      <c r="B22" s="39"/>
       <c r="C22" s="16"/>
       <c r="D22" s="18">
         <v>0.51400000000000001</v>
       </c>
       <c r="E22" s="16"/>
-      <c r="G22" s="16"/>
-      <c r="H22" s="16"/>
-      <c r="I22" s="18"/>
-      <c r="J22" s="16"/>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="H22" s="39"/>
+      <c r="I22" s="16"/>
+      <c r="J22" s="18"/>
+      <c r="K22" s="16"/>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A23" s="16" t="s">
-        <v>109</v>
-      </c>
-      <c r="B23" s="16">
-        <v>1.41</v>
-      </c>
+        <v>108</v>
+      </c>
+      <c r="B23" s="39"/>
       <c r="C23" s="16"/>
       <c r="D23" s="18">
         <v>4.0000000000000001E-3</v>
       </c>
       <c r="E23" s="16"/>
-      <c r="G23" s="16"/>
-      <c r="H23" s="16"/>
-      <c r="I23" s="18"/>
-      <c r="J23" s="16"/>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="H23" s="39"/>
+      <c r="I23" s="16"/>
+      <c r="J23" s="18"/>
+      <c r="K23" s="16"/>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A24" s="16" t="s">
-        <v>111</v>
-      </c>
-      <c r="B24" s="16"/>
+        <v>110</v>
+      </c>
+      <c r="B24" s="39"/>
       <c r="C24" s="16"/>
       <c r="D24" s="18"/>
       <c r="E24" s="16"/>
-      <c r="G24" s="16"/>
-      <c r="H24" s="16"/>
-      <c r="I24" s="18"/>
-      <c r="J24" s="16"/>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="H24" s="39"/>
+      <c r="I24" s="16"/>
+      <c r="J24" s="18"/>
+      <c r="K24" s="16"/>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A25" s="17" t="s">
         <v>82</v>
       </c>
-      <c r="B25" s="16"/>
+      <c r="B25" s="39"/>
       <c r="C25" s="16"/>
       <c r="D25" s="16"/>
       <c r="E25" s="16"/>
-      <c r="G25" s="16"/>
-      <c r="H25" s="16"/>
+      <c r="H25" s="39"/>
       <c r="I25" s="16"/>
       <c r="J25" s="16"/>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K25" s="16"/>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A26" s="16" t="s">
         <v>84</v>
       </c>
-      <c r="B26" s="16">
-        <v>12.433</v>
-      </c>
+      <c r="B26" s="39"/>
       <c r="C26" s="16"/>
       <c r="D26" s="18" t="s">
         <v>24</v>
       </c>
       <c r="E26" s="16"/>
-      <c r="G26" s="16"/>
-      <c r="H26" s="16"/>
-      <c r="I26" s="18"/>
-      <c r="J26" s="16"/>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="H26" s="39"/>
+      <c r="I26" s="16"/>
+      <c r="J26" s="18"/>
+      <c r="K26" s="16"/>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A27" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="B27" s="16">
-        <v>0.60799999999999998</v>
-      </c>
+      <c r="B27" s="39"/>
       <c r="C27" s="16"/>
       <c r="D27" s="18" t="s">
         <v>24</v>
       </c>
       <c r="E27" s="16"/>
-      <c r="G27" s="16"/>
-      <c r="H27" s="16"/>
-      <c r="I27" s="18"/>
-      <c r="J27" s="16"/>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="H27" s="39"/>
+      <c r="I27" s="16"/>
+      <c r="J27" s="18"/>
+      <c r="K27" s="16"/>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A28" s="16" t="s">
         <v>93</v>
       </c>
-      <c r="B28" s="16">
-        <v>1.83</v>
-      </c>
-      <c r="C28" s="16">
-        <v>0.04</v>
-      </c>
+      <c r="B28" s="39"/>
+      <c r="C28" s="16"/>
       <c r="D28" s="18" t="s">
         <v>24</v>
       </c>
       <c r="E28" s="16"/>
-      <c r="G28" s="16"/>
-      <c r="H28" s="16"/>
-      <c r="I28" s="18"/>
-      <c r="J28" s="16"/>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="H28" s="39"/>
+      <c r="I28" s="16"/>
+      <c r="J28" s="18"/>
+      <c r="K28" s="16"/>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A29" s="16" t="s">
-        <v>112</v>
-      </c>
-      <c r="B29" s="16"/>
+        <v>111</v>
+      </c>
+      <c r="B29" s="39"/>
       <c r="C29" s="16"/>
       <c r="D29" s="18"/>
       <c r="E29" s="16"/>
-      <c r="G29" s="16"/>
-      <c r="H29" s="16"/>
-      <c r="I29" s="18"/>
-      <c r="J29" s="16"/>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="H29" s="39"/>
+      <c r="I29" s="16"/>
+      <c r="J29" s="18"/>
+      <c r="K29" s="16"/>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A30" s="17" t="s">
         <v>83</v>
       </c>
-      <c r="B30" s="16"/>
+      <c r="B30" s="39"/>
       <c r="C30" s="16"/>
       <c r="D30" s="16"/>
       <c r="E30" s="16"/>
-      <c r="G30" s="16"/>
-      <c r="H30" s="16"/>
+      <c r="H30" s="39"/>
       <c r="I30" s="16"/>
       <c r="J30" s="16"/>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K30" s="16"/>
+    </row>
+    <row r="31" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A31" s="16" t="s">
+        <v>95</v>
+      </c>
+      <c r="B31" s="39"/>
+      <c r="C31" s="16"/>
+      <c r="D31" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="E31" s="16"/>
+      <c r="H31" s="39"/>
+      <c r="I31" s="16"/>
+      <c r="J31" s="18"/>
+      <c r="K31" s="16"/>
+    </row>
+    <row r="32" spans="1:11" ht="17" x14ac:dyDescent="0.25">
+      <c r="A32" s="16" t="s">
         <v>96</v>
       </c>
-      <c r="B31" s="16">
-        <v>2199.7800000000002</v>
-      </c>
-      <c r="C31" s="16">
-        <v>74.569999999999993</v>
-      </c>
-      <c r="D31" s="18" t="s">
-        <v>24</v>
-      </c>
-      <c r="E31" s="16"/>
-      <c r="G31" s="16"/>
-      <c r="H31" s="16"/>
-      <c r="I31" s="18"/>
-      <c r="J31" s="16"/>
-    </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A32" s="16" t="s">
-        <v>97</v>
-      </c>
-      <c r="B32" s="16">
-        <v>93.71</v>
-      </c>
-      <c r="C32" s="16">
-        <v>14.08</v>
-      </c>
+      <c r="B32" s="39"/>
+      <c r="C32" s="16"/>
       <c r="D32" s="18" t="s">
         <v>24</v>
       </c>
       <c r="E32" s="16"/>
-      <c r="G32" s="16"/>
-      <c r="H32" s="16"/>
-      <c r="I32" s="18"/>
-      <c r="J32" s="16"/>
-    </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="H32" s="39"/>
+      <c r="I32" s="16"/>
+      <c r="J32" s="18"/>
+      <c r="K32" s="16"/>
+    </row>
+    <row r="33" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A33" s="16" t="s">
         <v>84</v>
       </c>
-      <c r="B33" s="16">
-        <v>0.93400000000000005</v>
-      </c>
+      <c r="B33" s="39"/>
       <c r="C33" s="16"/>
       <c r="D33" s="18" t="s">
         <v>24</v>
       </c>
       <c r="E33" s="16"/>
-      <c r="G33" s="16"/>
-      <c r="H33" s="16"/>
-      <c r="I33" s="18"/>
-      <c r="J33" s="16"/>
-    </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="H33" s="39"/>
+      <c r="I33" s="16"/>
+      <c r="J33" s="18"/>
+      <c r="K33" s="16"/>
+    </row>
+    <row r="34" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A34" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="B34" s="16">
-        <v>1.7000000000000001E-2</v>
-      </c>
+      <c r="B34" s="39"/>
       <c r="C34" s="16"/>
       <c r="D34" s="18" t="s">
         <v>24</v>
       </c>
       <c r="E34" s="16"/>
-      <c r="G34" s="16"/>
-      <c r="H34" s="16"/>
-      <c r="I34" s="18"/>
-      <c r="J34" s="16"/>
-    </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="H34" s="39"/>
+      <c r="I34" s="16"/>
+      <c r="J34" s="18"/>
+      <c r="K34" s="16"/>
+    </row>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A35" s="16" t="s">
         <v>93</v>
       </c>
-      <c r="B35" s="16"/>
+      <c r="B35" s="39"/>
       <c r="C35" s="16"/>
       <c r="D35" s="18"/>
       <c r="E35" s="16"/>
-      <c r="G35" s="16"/>
-      <c r="H35" s="16"/>
-      <c r="I35" s="18"/>
-      <c r="J35" s="16"/>
-    </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="H35" s="39"/>
+      <c r="I35" s="16"/>
+      <c r="J35" s="18"/>
+      <c r="K35" s="16"/>
+    </row>
+    <row r="36" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A36" s="16" t="s">
-        <v>112</v>
-      </c>
-      <c r="B36" s="16"/>
+        <v>111</v>
+      </c>
+      <c r="B36" s="39"/>
       <c r="C36" s="16"/>
       <c r="D36" s="18"/>
-      <c r="G36" s="16"/>
-      <c r="H36" s="16"/>
-      <c r="I36" s="18"/>
-    </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="H36" s="39"/>
+      <c r="I36" s="16"/>
+      <c r="J36" s="18"/>
+    </row>
+    <row r="37" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A37" s="20" t="s">
-        <v>117</v>
-      </c>
-      <c r="B37" s="14"/>
+        <v>116</v>
+      </c>
+      <c r="B37" s="41"/>
       <c r="C37" s="14"/>
       <c r="D37" s="14"/>
       <c r="E37" s="14"/>
-      <c r="F37" s="14"/>
+      <c r="F37" s="36"/>
       <c r="G37" s="14"/>
-      <c r="H37" s="14"/>
+      <c r="H37" s="41"/>
       <c r="I37" s="14"/>
       <c r="J37" s="14"/>
       <c r="K37" s="14"/>
-      <c r="L37" s="16"/>
-      <c r="M37" s="16"/>
-    </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="L37" s="36"/>
+    </row>
+    <row r="38" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A38" s="15" t="s">
-        <v>118</v>
-      </c>
-      <c r="B38" s="15"/>
+        <v>117</v>
+      </c>
+      <c r="B38" s="42"/>
       <c r="C38" s="15"/>
       <c r="D38" s="15"/>
       <c r="E38" s="15"/>
-      <c r="F38" s="15"/>
+      <c r="F38" s="37"/>
       <c r="G38" s="15"/>
-      <c r="H38" s="15"/>
+      <c r="H38" s="42"/>
       <c r="I38" s="15"/>
       <c r="J38" s="15"/>
       <c r="K38" s="15"/>
-      <c r="L38" s="16"/>
-      <c r="M38" s="16"/>
+      <c r="L38" s="37"/>
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="B2:E2"/>
-    <mergeCell ref="G2:J2"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="G3:J3"/>
+    <mergeCell ref="H2:L2"/>
+    <mergeCell ref="H3:L3"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B2:F2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -8099,64 +8201,64 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{540507A6-720C-0B43-804E-087FEE710926}">
   <dimension ref="A1:E25"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.875" customWidth="1"/>
-    <col min="2" max="2" width="18.875" customWidth="1"/>
-    <col min="3" max="3" width="19.125" customWidth="1"/>
+    <col min="1" max="1" width="19.83203125" customWidth="1"/>
+    <col min="2" max="2" width="18.83203125" customWidth="1"/>
+    <col min="3" max="3" width="19.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="23" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="24"/>
+    </row>
+    <row r="3" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="24" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="24" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="24"/>
+    </row>
+    <row r="6" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="24"/>
+    </row>
+    <row r="7" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="8" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="23" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="2" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="24"/>
-    </row>
-    <row r="3" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="24" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="24" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="24"/>
-    </row>
-    <row r="6" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="24"/>
-    </row>
-    <row r="7" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="8" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="23" t="s">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A9" s="24" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A10" s="24" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B11" s="23" t="s">
+        <v>128</v>
+      </c>
+      <c r="C11" s="23" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
         <v>125</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="24" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="24" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B11" s="23" t="s">
-        <v>129</v>
-      </c>
-      <c r="C11" s="23" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>126</v>
       </c>
       <c r="B12">
         <v>-3.4000000000000002E-2</v>
@@ -8165,9 +8267,9 @@
         <v>-1.4E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B13">
         <v>-2.4E-2</v>
@@ -8176,9 +8278,9 @@
         <v>-8.0000000000000002E-3</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B14">
         <v>-2.3E-2</v>
@@ -8187,9 +8289,9 @@
         <v>-7.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B15">
         <v>-2.5999999999999999E-2</v>
@@ -8198,27 +8300,27 @@
         <v>-8.0000000000000002E-3</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" s="23" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" s="24" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B19" s="23" t="s">
+        <v>128</v>
+      </c>
+      <c r="C19" s="23" t="s">
         <v>129</v>
       </c>
-      <c r="C19" s="23" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B20">
         <v>-3.1E-2</v>
@@ -8227,9 +8329,9 @@
         <v>-1.0999999999999999E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B21">
         <v>-0.03</v>
@@ -8238,9 +8340,9 @@
         <v>-1.2999999999999999E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B22">
         <v>-0.113</v>
@@ -8249,9 +8351,9 @@
         <v>9.7000000000000003E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B23">
         <v>-3.3000000000000002E-2</v>
@@ -8260,9 +8362,9 @@
         <v>-1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="E25" s="23" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Just really looked at tables!
</commit_message>
<xml_diff>
--- a/Tables.xlsx
+++ b/Tables.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nchaku\Documents\GitHub\pubertybrain\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nchaku/Documents/GitHub/pubertybrain/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69659088-394A-467C-AD8B-B0810D623CC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DBDCA32-700C-9942-8973-B738A2BA3D07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="4" xr2:uid="{E0F15479-AA73-0644-8B08-3949D67CD8FE}"/>
+    <workbookView xWindow="1440" yWindow="500" windowWidth="27360" windowHeight="16400" activeTab="7" xr2:uid="{E0F15479-AA73-0644-8B08-3949D67CD8FE}"/>
   </bookViews>
   <sheets>
     <sheet name="Descriptive table" sheetId="1" r:id="rId1"/>
@@ -19,8 +19,9 @@
     <sheet name="Fig2 (Brain)" sheetId="4" r:id="rId4"/>
     <sheet name="CortModels" sheetId="6" r:id="rId5"/>
     <sheet name="SubCortModel" sheetId="10" r:id="rId6"/>
-    <sheet name="Youth report PDS" sheetId="9" r:id="rId7"/>
-    <sheet name="Indirect effects" sheetId="7" r:id="rId8"/>
+    <sheet name="Indirect effects" sheetId="7" r:id="rId7"/>
+    <sheet name="Sex Differences" sheetId="11" r:id="rId8"/>
+    <sheet name="Youth report PDS" sheetId="9" r:id="rId9"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -1177,14 +1178,14 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1772,20 +1773,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39987BE7-3659-524A-81AE-D479F97EF698}">
   <dimension ref="A1:F29"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="28.875" bestFit="1" customWidth="1"/>
-    <col min="2" max="4" width="20.125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28.83203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="4" width="20.1640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="9"/>
       <c r="B2" s="10" t="s">
         <v>63</v>
@@ -1803,7 +1804,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="6"/>
       <c r="B3" s="11" t="s">
         <v>69</v>
@@ -1817,7 +1818,7 @@
       <c r="E3" s="11"/>
       <c r="F3" s="6"/>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
         <v>60</v>
       </c>
@@ -1827,7 +1828,7 @@
       <c r="E4" s="2"/>
       <c r="F4" s="1"/>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
         <v>61</v>
       </c>
@@ -1847,7 +1848,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
         <v>62</v>
       </c>
@@ -1867,7 +1868,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
         <v>58</v>
       </c>
@@ -1887,7 +1888,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="8" t="s">
         <v>59</v>
       </c>
@@ -1897,7 +1898,7 @@
       <c r="E8" s="12"/>
       <c r="F8" s="1"/>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="3" t="s">
         <v>61</v>
       </c>
@@ -1917,7 +1918,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="3" t="s">
         <v>66</v>
       </c>
@@ -1937,7 +1938,7 @@
         <v>0.06</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="3" t="s">
         <v>67</v>
       </c>
@@ -1957,7 +1958,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="3" t="s">
         <v>62</v>
       </c>
@@ -1977,7 +1978,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" s="8" t="s">
         <v>68</v>
       </c>
@@ -1987,7 +1988,7 @@
       <c r="E13" s="12"/>
       <c r="F13" s="1"/>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" s="3" t="s">
         <v>73</v>
       </c>
@@ -2007,7 +2008,7 @@
         <v>1.74</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
         <v>74</v>
       </c>
@@ -2027,7 +2028,7 @@
         <v>1.93</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" s="3" t="s">
         <v>75</v>
       </c>
@@ -2047,7 +2048,7 @@
         <v>1.69</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" s="3" t="s">
         <v>76</v>
       </c>
@@ -2065,7 +2066,7 @@
       </c>
       <c r="F17" s="19"/>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" s="8" t="s">
         <v>71</v>
       </c>
@@ -2075,7 +2076,7 @@
       <c r="E18" s="12"/>
       <c r="F18" s="1"/>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" s="3" t="s">
         <v>61</v>
       </c>
@@ -2095,7 +2096,7 @@
         <v>0.87</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" s="3" t="s">
         <v>66</v>
       </c>
@@ -2115,7 +2116,7 @@
         <v>0.93</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" s="3" t="s">
         <v>67</v>
       </c>
@@ -2135,7 +2136,7 @@
         <v>1.18</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" s="3" t="s">
         <v>62</v>
       </c>
@@ -2155,7 +2156,7 @@
         <v>1.24</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23" s="8" t="s">
         <v>72</v>
       </c>
@@ -2165,7 +2166,7 @@
       <c r="E23" s="12"/>
       <c r="F23" s="1"/>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" s="3" t="s">
         <v>61</v>
       </c>
@@ -2185,7 +2186,7 @@
         <v>0.88</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" s="3" t="s">
         <v>66</v>
       </c>
@@ -2205,7 +2206,7 @@
         <v>0.88</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" s="3" t="s">
         <v>67</v>
       </c>
@@ -2225,7 +2226,7 @@
         <v>1.1299999999999999</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27" s="7" t="s">
         <v>62</v>
       </c>
@@ -2245,7 +2246,7 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="28" spans="1:6" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" ht="18" x14ac:dyDescent="0.2">
       <c r="A28" s="4"/>
       <c r="B28" s="1"/>
       <c r="C28" s="1"/>
@@ -2253,7 +2254,7 @@
       <c r="E28" s="1"/>
       <c r="F28" s="1"/>
     </row>
-    <row r="29" spans="1:6" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" ht="18" x14ac:dyDescent="0.2">
       <c r="A29" s="4"/>
       <c r="B29" s="1"/>
       <c r="C29" s="1"/>
@@ -2269,9 +2270,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A749072B-F938-0F49-BE23-243603B2B3D0}">
   <dimension ref="M2"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="2" spans="13:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="13:13" x14ac:dyDescent="0.2">
       <c r="M2" t="s">
         <v>111</v>
       </c>
@@ -2285,7 +2286,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45875D41-9C56-AA4E-A18A-2D3A4CE169B3}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2295,7 +2296,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A2A5153E-6E5C-054A-8ACA-5118463B96C5}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2305,142 +2306,142 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BBA86F85-A8D4-F648-84C3-730F1A42C846}">
   <dimension ref="A1:AM34"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.125" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="6.5" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="1.125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="1.1640625" style="1" customWidth="1"/>
     <col min="8" max="8" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="5.125" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="5.625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="5.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="5.6640625" style="1" customWidth="1"/>
     <col min="11" max="11" width="6.5" style="1" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="1.125" style="1" customWidth="1"/>
+    <col min="13" max="13" width="1.1640625" style="1" customWidth="1"/>
     <col min="14" max="14" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="5.125" style="1" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="5.625" style="1" customWidth="1"/>
+    <col min="15" max="15" width="5.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="5.6640625" style="1" customWidth="1"/>
     <col min="17" max="17" width="6.5" style="1" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="0.875" style="1" customWidth="1"/>
+    <col min="19" max="19" width="0.83203125" style="1" customWidth="1"/>
     <col min="20" max="20" width="8.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="5.125" style="1" bestFit="1" customWidth="1"/>
-    <col min="22" max="23" width="5.625" style="1" customWidth="1"/>
-    <col min="24" max="24" width="6.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="5.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="22" max="23" width="5.6640625" style="1" customWidth="1"/>
+    <col min="24" max="24" width="6.1640625" style="1" bestFit="1" customWidth="1"/>
     <col min="25" max="25" width="1" style="1" customWidth="1"/>
     <col min="26" max="26" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="5.125" style="1" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="5.625" style="1" customWidth="1"/>
+    <col min="27" max="27" width="5.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="5.6640625" style="1" customWidth="1"/>
     <col min="29" max="30" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="1.125" style="1" customWidth="1"/>
+    <col min="31" max="31" width="1.1640625" style="1" customWidth="1"/>
     <col min="32" max="32" width="7" style="1" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="5.125" style="1" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="5.625" style="1" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="5.625" style="1" customWidth="1"/>
-    <col min="36" max="36" width="6.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="5.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="5.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="5.6640625" style="1" customWidth="1"/>
+    <col min="36" max="36" width="6.1640625" style="1" bestFit="1" customWidth="1"/>
     <col min="37" max="16384" width="11" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A2" s="14"/>
-      <c r="B2" s="41" t="s">
+      <c r="B2" s="42" t="s">
         <v>112</v>
       </c>
-      <c r="C2" s="41"/>
-      <c r="D2" s="41"/>
-      <c r="E2" s="41"/>
-      <c r="F2" s="41"/>
-      <c r="G2" s="41"/>
-      <c r="H2" s="41"/>
-      <c r="I2" s="41"/>
-      <c r="J2" s="41"/>
-      <c r="K2" s="41"/>
-      <c r="L2" s="41"/>
-      <c r="M2" s="41"/>
-      <c r="N2" s="41"/>
-      <c r="O2" s="41"/>
-      <c r="P2" s="41"/>
-      <c r="Q2" s="41"/>
-      <c r="R2" s="41"/>
+      <c r="C2" s="42"/>
+      <c r="D2" s="42"/>
+      <c r="E2" s="42"/>
+      <c r="F2" s="42"/>
+      <c r="G2" s="42"/>
+      <c r="H2" s="42"/>
+      <c r="I2" s="42"/>
+      <c r="J2" s="42"/>
+      <c r="K2" s="42"/>
+      <c r="L2" s="42"/>
+      <c r="M2" s="42"/>
+      <c r="N2" s="42"/>
+      <c r="O2" s="42"/>
+      <c r="P2" s="42"/>
+      <c r="Q2" s="42"/>
+      <c r="R2" s="42"/>
       <c r="S2" s="9"/>
-      <c r="T2" s="41" t="s">
+      <c r="T2" s="42" t="s">
         <v>113</v>
       </c>
-      <c r="U2" s="41"/>
-      <c r="V2" s="41"/>
-      <c r="W2" s="41"/>
-      <c r="X2" s="41"/>
-      <c r="Y2" s="41"/>
-      <c r="Z2" s="41"/>
-      <c r="AA2" s="41"/>
-      <c r="AB2" s="41"/>
-      <c r="AC2" s="41"/>
-      <c r="AD2" s="41"/>
-      <c r="AE2" s="41"/>
-      <c r="AF2" s="41"/>
-      <c r="AG2" s="41"/>
-      <c r="AH2" s="41"/>
-      <c r="AI2" s="41"/>
-      <c r="AJ2" s="41"/>
-    </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="U2" s="42"/>
+      <c r="V2" s="42"/>
+      <c r="W2" s="42"/>
+      <c r="X2" s="42"/>
+      <c r="Y2" s="42"/>
+      <c r="Z2" s="42"/>
+      <c r="AA2" s="42"/>
+      <c r="AB2" s="42"/>
+      <c r="AC2" s="42"/>
+      <c r="AD2" s="42"/>
+      <c r="AE2" s="42"/>
+      <c r="AF2" s="42"/>
+      <c r="AG2" s="42"/>
+      <c r="AH2" s="42"/>
+      <c r="AI2" s="42"/>
+      <c r="AJ2" s="42"/>
+    </row>
+    <row r="3" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A3" s="16"/>
-      <c r="B3" s="41" t="s">
+      <c r="B3" s="42" t="s">
         <v>79</v>
       </c>
-      <c r="C3" s="41"/>
-      <c r="D3" s="41"/>
-      <c r="E3" s="41"/>
-      <c r="F3" s="41"/>
+      <c r="C3" s="42"/>
+      <c r="D3" s="42"/>
+      <c r="E3" s="42"/>
+      <c r="F3" s="42"/>
       <c r="G3" s="28"/>
-      <c r="H3" s="41" t="s">
+      <c r="H3" s="42" t="s">
         <v>80</v>
       </c>
-      <c r="I3" s="41"/>
-      <c r="J3" s="41"/>
-      <c r="K3" s="41"/>
-      <c r="L3" s="41"/>
+      <c r="I3" s="42"/>
+      <c r="J3" s="42"/>
+      <c r="K3" s="42"/>
+      <c r="L3" s="42"/>
       <c r="M3" s="28"/>
-      <c r="N3" s="41" t="s">
+      <c r="N3" s="42" t="s">
         <v>81</v>
       </c>
-      <c r="O3" s="41"/>
-      <c r="P3" s="41"/>
-      <c r="Q3" s="41"/>
-      <c r="R3" s="41"/>
-      <c r="T3" s="42" t="s">
+      <c r="O3" s="42"/>
+      <c r="P3" s="42"/>
+      <c r="Q3" s="42"/>
+      <c r="R3" s="42"/>
+      <c r="T3" s="43" t="s">
         <v>79</v>
       </c>
-      <c r="U3" s="42"/>
-      <c r="V3" s="42"/>
-      <c r="W3" s="42"/>
-      <c r="X3" s="42"/>
+      <c r="U3" s="43"/>
+      <c r="V3" s="43"/>
+      <c r="W3" s="43"/>
+      <c r="X3" s="43"/>
       <c r="Y3" s="28"/>
-      <c r="Z3" s="41" t="s">
+      <c r="Z3" s="42" t="s">
         <v>80</v>
       </c>
-      <c r="AA3" s="41"/>
-      <c r="AB3" s="41"/>
-      <c r="AC3" s="41"/>
-      <c r="AD3" s="41"/>
+      <c r="AA3" s="42"/>
+      <c r="AB3" s="42"/>
+      <c r="AC3" s="42"/>
+      <c r="AD3" s="42"/>
       <c r="AE3" s="28"/>
-      <c r="AF3" s="41" t="s">
+      <c r="AF3" s="42" t="s">
         <v>81</v>
       </c>
-      <c r="AG3" s="41"/>
-      <c r="AH3" s="41"/>
-      <c r="AI3" s="41"/>
-      <c r="AJ3" s="41"/>
-    </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AG3" s="42"/>
+      <c r="AH3" s="42"/>
+      <c r="AI3" s="42"/>
+      <c r="AJ3" s="42"/>
+    </row>
+    <row r="4" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A4" s="15"/>
       <c r="B4" s="29" t="s">
         <v>89</v>
@@ -2538,7 +2539,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A5" s="17" t="s">
         <v>84</v>
       </c>
@@ -2577,7 +2578,7 @@
       <c r="AI5" s="16"/>
       <c r="AJ5" s="16"/>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A6" s="16" t="s">
         <v>94</v>
       </c>
@@ -2676,7 +2677,7 @@
         <v>12.236000000000001</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A7" s="16" t="s">
         <v>95</v>
       </c>
@@ -2775,7 +2776,7 @@
         <v>-7.7560000000000002</v>
       </c>
     </row>
-    <row r="8" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A8" s="16"/>
       <c r="B8" s="16"/>
       <c r="C8" s="16"/>
@@ -2812,7 +2813,7 @@
       <c r="AI8" s="18"/>
       <c r="AJ8" s="16"/>
     </row>
-    <row r="9" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A9" s="17" t="s">
         <v>85</v>
       </c>
@@ -2851,7 +2852,7 @@
       <c r="AI9" s="16"/>
       <c r="AJ9" s="16"/>
     </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A10" s="16" t="s">
         <v>96</v>
       </c>
@@ -2950,7 +2951,7 @@
         <v>-0.24</v>
       </c>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A11" s="16" t="s">
         <v>97</v>
       </c>
@@ -3049,7 +3050,7 @@
         <v>0.09</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A12" s="16" t="s">
         <v>98</v>
       </c>
@@ -3148,7 +3149,7 @@
         <v>0.14899999999999999</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A13" s="16" t="s">
         <v>99</v>
       </c>
@@ -3247,7 +3248,7 @@
         <v>3.5999999999999997E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A14" s="16" t="s">
         <v>87</v>
       </c>
@@ -3346,7 +3347,7 @@
         <v>0.28799999999999998</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A15" s="16"/>
       <c r="B15" s="16"/>
       <c r="C15" s="16"/>
@@ -3383,7 +3384,7 @@
       <c r="AI15" s="18"/>
       <c r="AJ15" s="16"/>
     </row>
-    <row r="16" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A16" s="17" t="s">
         <v>86</v>
       </c>
@@ -3422,7 +3423,7 @@
       <c r="AI16" s="16"/>
       <c r="AJ16" s="16"/>
     </row>
-    <row r="17" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A17" s="16" t="s">
         <v>100</v>
       </c>
@@ -3521,7 +3522,7 @@
         <v>0.443</v>
       </c>
     </row>
-    <row r="18" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A18" s="16" t="s">
         <v>101</v>
       </c>
@@ -3620,7 +3621,7 @@
         <v>-0.10299999999999999</v>
       </c>
     </row>
-    <row r="19" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A19" s="16" t="s">
         <v>102</v>
       </c>
@@ -3719,7 +3720,7 @@
         <v>9.0999999999999998E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A20" s="16" t="s">
         <v>105</v>
       </c>
@@ -3818,7 +3819,7 @@
         <v>3.1E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A21" s="16" t="s">
         <v>106</v>
       </c>
@@ -3917,7 +3918,7 @@
         <v>-0.13600000000000001</v>
       </c>
     </row>
-    <row r="22" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A22" s="16" t="s">
         <v>103</v>
       </c>
@@ -4014,7 +4015,7 @@
         <v>0.156</v>
       </c>
     </row>
-    <row r="23" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A23" s="16" t="s">
         <v>104</v>
       </c>
@@ -4111,7 +4112,7 @@
         <v>-1.6E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A24" s="16" t="s">
         <v>108</v>
       </c>
@@ -4208,7 +4209,7 @@
         <v>0.112</v>
       </c>
     </row>
-    <row r="25" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A25" s="16" t="s">
         <v>107</v>
       </c>
@@ -4305,7 +4306,7 @@
         <v>0.16</v>
       </c>
     </row>
-    <row r="26" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A26" s="16" t="s">
         <v>109</v>
       </c>
@@ -4402,7 +4403,7 @@
         <v>-4.9000000000000002E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A27" s="16"/>
       <c r="B27" s="16"/>
       <c r="C27" s="16"/>
@@ -4439,7 +4440,7 @@
       <c r="AI27" s="18"/>
       <c r="AJ27" s="16"/>
     </row>
-    <row r="28" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A28" s="17" t="s">
         <v>82</v>
       </c>
@@ -4478,7 +4479,7 @@
       <c r="AI28" s="16"/>
       <c r="AJ28" s="16"/>
     </row>
-    <row r="29" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A29" s="16" t="s">
         <v>83</v>
       </c>
@@ -4577,7 +4578,7 @@
         <v>14.164999999999999</v>
       </c>
     </row>
-    <row r="30" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A30" s="16" t="s">
         <v>88</v>
       </c>
@@ -4676,7 +4677,7 @@
         <v>4.1660000000000004</v>
       </c>
     </row>
-    <row r="31" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A31" s="16" t="s">
         <v>92</v>
       </c>
@@ -4775,7 +4776,7 @@
         <v>1.0549999999999999</v>
       </c>
     </row>
-    <row r="32" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A32" s="16" t="s">
         <v>110</v>
       </c>
@@ -4872,7 +4873,7 @@
         <v>4.202</v>
       </c>
     </row>
-    <row r="33" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:39" x14ac:dyDescent="0.2">
       <c r="A33" s="20" t="s">
         <v>115</v>
       </c>
@@ -4915,69 +4916,63 @@
       <c r="AL33" s="16"/>
       <c r="AM33" s="16"/>
     </row>
-    <row r="34" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:39" x14ac:dyDescent="0.2">
       <c r="A34" s="15" t="s">
         <v>116</v>
       </c>
-      <c r="B34" s="43">
+      <c r="B34" s="41">
         <v>74058.118000000002</v>
       </c>
-      <c r="C34" s="43"/>
-      <c r="D34" s="43"/>
-      <c r="E34" s="43"/>
-      <c r="F34" s="43"/>
+      <c r="C34" s="41"/>
+      <c r="D34" s="41"/>
+      <c r="E34" s="41"/>
+      <c r="F34" s="41"/>
       <c r="G34" s="27"/>
-      <c r="H34" s="43">
+      <c r="H34" s="41">
         <v>83016.937999999995</v>
       </c>
-      <c r="I34" s="43"/>
-      <c r="J34" s="43"/>
-      <c r="K34" s="43"/>
-      <c r="L34" s="43"/>
+      <c r="I34" s="41"/>
+      <c r="J34" s="41"/>
+      <c r="K34" s="41"/>
+      <c r="L34" s="41"/>
       <c r="M34" s="27"/>
-      <c r="N34" s="43">
+      <c r="N34" s="41">
         <v>94345.274999999994</v>
       </c>
-      <c r="O34" s="43"/>
-      <c r="P34" s="43"/>
-      <c r="Q34" s="43"/>
-      <c r="R34" s="43"/>
+      <c r="O34" s="41"/>
+      <c r="P34" s="41"/>
+      <c r="Q34" s="41"/>
+      <c r="R34" s="41"/>
       <c r="S34" s="15"/>
-      <c r="T34" s="43">
+      <c r="T34" s="41">
         <v>83167.763000000006</v>
       </c>
-      <c r="U34" s="43"/>
-      <c r="V34" s="43"/>
-      <c r="W34" s="43"/>
-      <c r="X34" s="43"/>
+      <c r="U34" s="41"/>
+      <c r="V34" s="41"/>
+      <c r="W34" s="41"/>
+      <c r="X34" s="41"/>
       <c r="Y34" s="27"/>
-      <c r="Z34" s="43">
+      <c r="Z34" s="41">
         <v>93083.505999999994</v>
       </c>
-      <c r="AA34" s="43"/>
-      <c r="AB34" s="43"/>
-      <c r="AC34" s="43"/>
-      <c r="AD34" s="43"/>
+      <c r="AA34" s="41"/>
+      <c r="AB34" s="41"/>
+      <c r="AC34" s="41"/>
+      <c r="AD34" s="41"/>
       <c r="AE34" s="27"/>
-      <c r="AF34" s="43">
+      <c r="AF34" s="41">
         <v>105770.462</v>
       </c>
-      <c r="AG34" s="43"/>
-      <c r="AH34" s="43"/>
-      <c r="AI34" s="43"/>
-      <c r="AJ34" s="43"/>
+      <c r="AG34" s="41"/>
+      <c r="AH34" s="41"/>
+      <c r="AI34" s="41"/>
+      <c r="AJ34" s="41"/>
       <c r="AK34" s="16"/>
       <c r="AL34" s="16"/>
       <c r="AM34" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="AF34:AJ34"/>
-    <mergeCell ref="B34:F34"/>
-    <mergeCell ref="H34:L34"/>
-    <mergeCell ref="T34:X34"/>
-    <mergeCell ref="N34:R34"/>
-    <mergeCell ref="Z34:AD34"/>
     <mergeCell ref="B3:F3"/>
     <mergeCell ref="B2:R2"/>
     <mergeCell ref="H3:L3"/>
@@ -4986,6 +4981,12 @@
     <mergeCell ref="T3:X3"/>
     <mergeCell ref="Z3:AD3"/>
     <mergeCell ref="AF3:AJ3"/>
+    <mergeCell ref="AF34:AJ34"/>
+    <mergeCell ref="B34:F34"/>
+    <mergeCell ref="H34:L34"/>
+    <mergeCell ref="T34:X34"/>
+    <mergeCell ref="N34:R34"/>
+    <mergeCell ref="Z34:AD34"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
@@ -4995,140 +4996,140 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CD5CF7F-81D6-D24D-8228-B4C578C35D65}">
   <dimension ref="A1:AM41"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="24" style="1" customWidth="1"/>
     <col min="2" max="2" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.125" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="5.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.6640625" style="1" customWidth="1"/>
     <col min="5" max="6" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="1.125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="1.1640625" style="1" customWidth="1"/>
     <col min="8" max="8" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="5.125" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="5.625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="5.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="5.6640625" style="1" customWidth="1"/>
     <col min="11" max="12" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="1.125" style="1" customWidth="1"/>
+    <col min="13" max="13" width="1.1640625" style="1" customWidth="1"/>
     <col min="14" max="14" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="5.125" style="1" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="5.625" style="1" customWidth="1"/>
+    <col min="15" max="15" width="5.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="5.6640625" style="1" customWidth="1"/>
     <col min="17" max="17" width="6.5" style="1" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="0.875" style="1" customWidth="1"/>
+    <col min="19" max="19" width="0.83203125" style="1" customWidth="1"/>
     <col min="20" max="20" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="5.875" style="1" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="6.375" style="1" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="5.625" style="1" customWidth="1"/>
+    <col min="21" max="21" width="5.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="6.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="5.6640625" style="1" customWidth="1"/>
     <col min="24" max="24" width="6" style="1" bestFit="1" customWidth="1"/>
     <col min="25" max="25" width="1" style="1" customWidth="1"/>
     <col min="26" max="26" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="5.125" style="1" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="5.625" style="1" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="5.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="5.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="29" max="30" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="1.125" style="1" customWidth="1"/>
+    <col min="31" max="31" width="1.1640625" style="1" customWidth="1"/>
     <col min="32" max="32" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="5.125" style="1" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="5.625" style="1" customWidth="1"/>
+    <col min="33" max="33" width="5.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="5.6640625" style="1" customWidth="1"/>
     <col min="35" max="36" width="6" style="1" bestFit="1" customWidth="1"/>
     <col min="37" max="16384" width="11" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A2" s="14"/>
-      <c r="B2" s="41" t="s">
+      <c r="B2" s="42" t="s">
         <v>112</v>
       </c>
-      <c r="C2" s="41"/>
-      <c r="D2" s="41"/>
-      <c r="E2" s="41"/>
-      <c r="F2" s="41"/>
-      <c r="G2" s="41"/>
-      <c r="H2" s="41"/>
-      <c r="I2" s="41"/>
-      <c r="J2" s="41"/>
-      <c r="K2" s="41"/>
-      <c r="L2" s="41"/>
-      <c r="M2" s="41"/>
-      <c r="N2" s="41"/>
-      <c r="O2" s="41"/>
-      <c r="P2" s="41"/>
-      <c r="Q2" s="41"/>
-      <c r="R2" s="41"/>
+      <c r="C2" s="42"/>
+      <c r="D2" s="42"/>
+      <c r="E2" s="42"/>
+      <c r="F2" s="42"/>
+      <c r="G2" s="42"/>
+      <c r="H2" s="42"/>
+      <c r="I2" s="42"/>
+      <c r="J2" s="42"/>
+      <c r="K2" s="42"/>
+      <c r="L2" s="42"/>
+      <c r="M2" s="42"/>
+      <c r="N2" s="42"/>
+      <c r="O2" s="42"/>
+      <c r="P2" s="42"/>
+      <c r="Q2" s="42"/>
+      <c r="R2" s="42"/>
       <c r="S2" s="9"/>
-      <c r="T2" s="41" t="s">
+      <c r="T2" s="42" t="s">
         <v>113</v>
       </c>
-      <c r="U2" s="41"/>
-      <c r="V2" s="41"/>
-      <c r="W2" s="41"/>
-      <c r="X2" s="41"/>
-      <c r="Y2" s="41"/>
-      <c r="Z2" s="41"/>
-      <c r="AA2" s="41"/>
-      <c r="AB2" s="41"/>
-      <c r="AC2" s="41"/>
-      <c r="AD2" s="41"/>
-      <c r="AE2" s="41"/>
-      <c r="AF2" s="41"/>
-      <c r="AG2" s="41"/>
-      <c r="AH2" s="41"/>
-      <c r="AI2" s="41"/>
-      <c r="AJ2" s="41"/>
-    </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="U2" s="42"/>
+      <c r="V2" s="42"/>
+      <c r="W2" s="42"/>
+      <c r="X2" s="42"/>
+      <c r="Y2" s="42"/>
+      <c r="Z2" s="42"/>
+      <c r="AA2" s="42"/>
+      <c r="AB2" s="42"/>
+      <c r="AC2" s="42"/>
+      <c r="AD2" s="42"/>
+      <c r="AE2" s="42"/>
+      <c r="AF2" s="42"/>
+      <c r="AG2" s="42"/>
+      <c r="AH2" s="42"/>
+      <c r="AI2" s="42"/>
+      <c r="AJ2" s="42"/>
+    </row>
+    <row r="3" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A3" s="16"/>
-      <c r="B3" s="41" t="s">
+      <c r="B3" s="42" t="s">
         <v>79</v>
       </c>
-      <c r="C3" s="41"/>
-      <c r="D3" s="41"/>
-      <c r="E3" s="41"/>
-      <c r="F3" s="41"/>
+      <c r="C3" s="42"/>
+      <c r="D3" s="42"/>
+      <c r="E3" s="42"/>
+      <c r="F3" s="42"/>
       <c r="G3" s="28"/>
-      <c r="H3" s="41" t="s">
+      <c r="H3" s="42" t="s">
         <v>80</v>
       </c>
-      <c r="I3" s="41"/>
-      <c r="J3" s="41"/>
-      <c r="K3" s="41"/>
-      <c r="L3" s="41"/>
+      <c r="I3" s="42"/>
+      <c r="J3" s="42"/>
+      <c r="K3" s="42"/>
+      <c r="L3" s="42"/>
       <c r="M3" s="28"/>
-      <c r="N3" s="41" t="s">
+      <c r="N3" s="42" t="s">
         <v>81</v>
       </c>
-      <c r="O3" s="41"/>
-      <c r="P3" s="41"/>
-      <c r="Q3" s="41"/>
-      <c r="R3" s="41"/>
-      <c r="T3" s="42" t="s">
+      <c r="O3" s="42"/>
+      <c r="P3" s="42"/>
+      <c r="Q3" s="42"/>
+      <c r="R3" s="42"/>
+      <c r="T3" s="43" t="s">
         <v>79</v>
       </c>
-      <c r="U3" s="42"/>
-      <c r="V3" s="42"/>
-      <c r="W3" s="42"/>
-      <c r="X3" s="42"/>
+      <c r="U3" s="43"/>
+      <c r="V3" s="43"/>
+      <c r="W3" s="43"/>
+      <c r="X3" s="43"/>
       <c r="Y3" s="28"/>
-      <c r="Z3" s="41" t="s">
+      <c r="Z3" s="42" t="s">
         <v>80</v>
       </c>
-      <c r="AA3" s="41"/>
-      <c r="AB3" s="41"/>
-      <c r="AC3" s="41"/>
-      <c r="AD3" s="41"/>
+      <c r="AA3" s="42"/>
+      <c r="AB3" s="42"/>
+      <c r="AC3" s="42"/>
+      <c r="AD3" s="42"/>
       <c r="AE3" s="28"/>
-      <c r="AF3" s="41" t="s">
+      <c r="AF3" s="42" t="s">
         <v>81</v>
       </c>
-      <c r="AG3" s="41"/>
-      <c r="AH3" s="41"/>
-      <c r="AI3" s="41"/>
-      <c r="AJ3" s="41"/>
-    </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AG3" s="42"/>
+      <c r="AH3" s="42"/>
+      <c r="AI3" s="42"/>
+      <c r="AJ3" s="42"/>
+    </row>
+    <row r="4" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A4" s="15"/>
       <c r="B4" s="29" t="s">
         <v>89</v>
@@ -5226,7 +5227,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A5" s="17" t="s">
         <v>84</v>
       </c>
@@ -5265,7 +5266,7 @@
       <c r="AI5" s="16"/>
       <c r="AJ5" s="16"/>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A6" s="16" t="s">
         <v>94</v>
       </c>
@@ -5364,7 +5365,7 @@
         <v>13.875999999999999</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A7" s="16" t="s">
         <v>95</v>
       </c>
@@ -5463,7 +5464,7 @@
         <v>2.1219999999999999</v>
       </c>
     </row>
-    <row r="8" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A8" s="16" t="s">
         <v>138</v>
       </c>
@@ -5562,7 +5563,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="9" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A9" s="16"/>
       <c r="B9" s="16"/>
       <c r="C9" s="16"/>
@@ -5599,7 +5600,7 @@
       <c r="AI9" s="18"/>
       <c r="AJ9" s="16"/>
     </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A10" s="17" t="s">
         <v>85</v>
       </c>
@@ -5638,7 +5639,7 @@
       <c r="AI10" s="16"/>
       <c r="AJ10" s="16"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A11" s="16" t="s">
         <v>96</v>
       </c>
@@ -5737,7 +5738,7 @@
         <v>0.40300000000000002</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A12" s="16" t="s">
         <v>137</v>
       </c>
@@ -5836,7 +5837,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A13" s="16" t="s">
         <v>97</v>
       </c>
@@ -5935,7 +5936,7 @@
         <v>2.4E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A14" s="16" t="s">
         <v>98</v>
       </c>
@@ -6034,7 +6035,7 @@
         <v>8.5999999999999993E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A15" s="16" t="s">
         <v>139</v>
       </c>
@@ -6133,7 +6134,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="16" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A16" s="16" t="s">
         <v>99</v>
       </c>
@@ -6232,7 +6233,7 @@
         <v>0.22900000000000001</v>
       </c>
     </row>
-    <row r="17" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A17" s="16" t="s">
         <v>140</v>
       </c>
@@ -6331,7 +6332,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="18" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A18" s="16" t="s">
         <v>87</v>
       </c>
@@ -6430,7 +6431,7 @@
         <v>0.28799999999999998</v>
       </c>
     </row>
-    <row r="19" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A19" s="16"/>
       <c r="B19" s="16"/>
       <c r="C19" s="16"/>
@@ -6467,7 +6468,7 @@
       <c r="AI19" s="18"/>
       <c r="AJ19" s="16"/>
     </row>
-    <row r="20" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A20" s="17" t="s">
         <v>86</v>
       </c>
@@ -6506,7 +6507,7 @@
       <c r="AI20" s="16"/>
       <c r="AJ20" s="16"/>
     </row>
-    <row r="21" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A21" s="16" t="s">
         <v>100</v>
       </c>
@@ -6605,7 +6606,7 @@
         <v>0.14499999999999999</v>
       </c>
     </row>
-    <row r="22" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A22" s="16" t="s">
         <v>136</v>
       </c>
@@ -6704,7 +6705,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="23" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A23" s="16" t="s">
         <v>101</v>
       </c>
@@ -6803,7 +6804,7 @@
         <v>-9.5000000000000001E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A24" s="16" t="s">
         <v>102</v>
       </c>
@@ -6902,7 +6903,7 @@
         <v>5.0999999999999997E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:36" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:36" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A25" s="16" t="s">
         <v>144</v>
       </c>
@@ -6982,7 +6983,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="26" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A26" s="16" t="s">
         <v>105</v>
       </c>
@@ -7081,7 +7082,7 @@
         <v>3.2000000000000001E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A27" s="16" t="s">
         <v>106</v>
       </c>
@@ -7180,7 +7181,7 @@
         <v>-0.13600000000000001</v>
       </c>
     </row>
-    <row r="28" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A28" s="16" t="s">
         <v>103</v>
       </c>
@@ -7277,7 +7278,7 @@
         <v>0.17199999999999999</v>
       </c>
     </row>
-    <row r="29" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:36" ht="17" x14ac:dyDescent="0.25">
       <c r="A29" s="16" t="s">
         <v>104</v>
       </c>
@@ -7374,7 +7375,7 @@
         <v>3.5999999999999997E-2</v>
       </c>
     </row>
-    <row r="30" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A30" s="16" t="s">
         <v>145</v>
       </c>
@@ -7453,7 +7454,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="31" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A31" s="16" t="s">
         <v>108</v>
       </c>
@@ -7550,7 +7551,7 @@
         <v>7.4999999999999997E-2</v>
       </c>
     </row>
-    <row r="32" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A32" s="16" t="s">
         <v>107</v>
       </c>
@@ -7647,7 +7648,7 @@
         <v>0.17499999999999999</v>
       </c>
     </row>
-    <row r="33" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:39" x14ac:dyDescent="0.2">
       <c r="A33" s="16" t="s">
         <v>109</v>
       </c>
@@ -7744,7 +7745,7 @@
         <v>-0.05</v>
       </c>
     </row>
-    <row r="34" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:39" x14ac:dyDescent="0.2">
       <c r="A34" s="16"/>
       <c r="B34" s="16"/>
       <c r="C34" s="16"/>
@@ -7781,7 +7782,7 @@
       <c r="AI34" s="18"/>
       <c r="AJ34" s="16"/>
     </row>
-    <row r="35" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:39" x14ac:dyDescent="0.2">
       <c r="A35" s="17" t="s">
         <v>82</v>
       </c>
@@ -7820,7 +7821,7 @@
       <c r="AI35" s="16"/>
       <c r="AJ35" s="16"/>
     </row>
-    <row r="36" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:39" x14ac:dyDescent="0.2">
       <c r="A36" s="16" t="s">
         <v>83</v>
       </c>
@@ -7919,7 +7920,7 @@
         <v>14.162000000000001</v>
       </c>
     </row>
-    <row r="37" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:39" x14ac:dyDescent="0.2">
       <c r="A37" s="16" t="s">
         <v>88</v>
       </c>
@@ -8018,7 +8019,7 @@
         <v>4.1660000000000004</v>
       </c>
     </row>
-    <row r="38" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:39" x14ac:dyDescent="0.2">
       <c r="A38" s="16" t="s">
         <v>92</v>
       </c>
@@ -8117,7 +8118,7 @@
         <v>1.0549999999999999</v>
       </c>
     </row>
-    <row r="39" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:39" x14ac:dyDescent="0.2">
       <c r="A39" s="16" t="s">
         <v>110</v>
       </c>
@@ -8214,7 +8215,7 @@
         <v>4.5090000000000003</v>
       </c>
     </row>
-    <row r="40" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:39" x14ac:dyDescent="0.2">
       <c r="A40" s="20" t="s">
         <v>115</v>
       </c>
@@ -8257,57 +8258,57 @@
       <c r="AL40" s="16"/>
       <c r="AM40" s="16"/>
     </row>
-    <row r="41" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:39" x14ac:dyDescent="0.2">
       <c r="A41" s="15" t="s">
         <v>116</v>
       </c>
-      <c r="B41" s="43">
+      <c r="B41" s="41">
         <v>34697.703999999998</v>
       </c>
-      <c r="C41" s="43"/>
-      <c r="D41" s="43"/>
-      <c r="E41" s="43"/>
-      <c r="F41" s="43"/>
+      <c r="C41" s="41"/>
+      <c r="D41" s="41"/>
+      <c r="E41" s="41"/>
+      <c r="F41" s="41"/>
       <c r="G41" s="27"/>
-      <c r="H41" s="43">
+      <c r="H41" s="41">
         <v>43730.449000000001</v>
       </c>
-      <c r="I41" s="43"/>
-      <c r="J41" s="43"/>
-      <c r="K41" s="43"/>
-      <c r="L41" s="43"/>
+      <c r="I41" s="41"/>
+      <c r="J41" s="41"/>
+      <c r="K41" s="41"/>
+      <c r="L41" s="41"/>
       <c r="M41" s="27"/>
-      <c r="N41" s="43">
+      <c r="N41" s="41">
         <v>55075.362999999998</v>
       </c>
-      <c r="O41" s="43"/>
-      <c r="P41" s="43"/>
-      <c r="Q41" s="43"/>
-      <c r="R41" s="43"/>
+      <c r="O41" s="41"/>
+      <c r="P41" s="41"/>
+      <c r="Q41" s="41"/>
+      <c r="R41" s="41"/>
       <c r="S41" s="15"/>
-      <c r="T41" s="43">
+      <c r="T41" s="41">
         <v>37782.404000000002</v>
       </c>
-      <c r="U41" s="43"/>
-      <c r="V41" s="43"/>
-      <c r="W41" s="43"/>
-      <c r="X41" s="43"/>
+      <c r="U41" s="41"/>
+      <c r="V41" s="41"/>
+      <c r="W41" s="41"/>
+      <c r="X41" s="41"/>
       <c r="Y41" s="27"/>
-      <c r="Z41" s="43">
+      <c r="Z41" s="41">
         <v>47698.324999999997</v>
       </c>
-      <c r="AA41" s="43"/>
-      <c r="AB41" s="43"/>
-      <c r="AC41" s="43"/>
-      <c r="AD41" s="43"/>
+      <c r="AA41" s="41"/>
+      <c r="AB41" s="41"/>
+      <c r="AC41" s="41"/>
+      <c r="AD41" s="41"/>
       <c r="AE41" s="27"/>
-      <c r="AF41" s="43">
+      <c r="AF41" s="41">
         <v>60402.93</v>
       </c>
-      <c r="AG41" s="43"/>
-      <c r="AH41" s="43"/>
-      <c r="AI41" s="43"/>
-      <c r="AJ41" s="43"/>
+      <c r="AG41" s="41"/>
+      <c r="AH41" s="41"/>
+      <c r="AI41" s="41"/>
+      <c r="AJ41" s="41"/>
       <c r="AK41" s="16"/>
       <c r="AL41" s="16"/>
       <c r="AM41" s="16"/>
@@ -8335,61 +8336,244 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{540507A6-720C-0B43-804E-087FEE710926}">
+  <dimension ref="A1:E25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="19.83203125" customWidth="1"/>
+    <col min="2" max="2" width="18.83203125" customWidth="1"/>
+    <col min="3" max="3" width="19.1640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="23" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="24"/>
+    </row>
+    <row r="3" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="24" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="24" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="24"/>
+    </row>
+    <row r="6" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="24"/>
+    </row>
+    <row r="7" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="8" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="23" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A9" s="24" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A10" s="24" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B11" s="23" t="s">
+        <v>127</v>
+      </c>
+      <c r="C11" s="23" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>124</v>
+      </c>
+      <c r="B12">
+        <v>-3.4000000000000002E-2</v>
+      </c>
+      <c r="C12">
+        <v>-1.4E-2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>125</v>
+      </c>
+      <c r="B13">
+        <v>-2.4E-2</v>
+      </c>
+      <c r="C13">
+        <v>-8.0000000000000002E-3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>126</v>
+      </c>
+      <c r="B14">
+        <v>-2.3E-2</v>
+      </c>
+      <c r="C14">
+        <v>-7.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>131</v>
+      </c>
+      <c r="B15">
+        <v>-2.5999999999999999E-2</v>
+      </c>
+      <c r="C15">
+        <v>-8.0000000000000002E-3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A17" s="23" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A18" s="24" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B19" s="23" t="s">
+        <v>127</v>
+      </c>
+      <c r="C19" s="23" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>124</v>
+      </c>
+      <c r="B20">
+        <v>-3.1E-2</v>
+      </c>
+      <c r="C20">
+        <v>-1.0999999999999999E-2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>125</v>
+      </c>
+      <c r="B21">
+        <v>-0.03</v>
+      </c>
+      <c r="C21">
+        <v>-1.2999999999999999E-2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>126</v>
+      </c>
+      <c r="B22">
+        <v>-0.113</v>
+      </c>
+      <c r="C22">
+        <v>9.7000000000000003E-2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>131</v>
+      </c>
+      <c r="B23">
+        <v>-3.3000000000000002E-2</v>
+      </c>
+      <c r="C23">
+        <v>-1.4999999999999999E-2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="E25" s="23" t="s">
+        <v>130</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A439B20-C024-854E-8504-DA6820AADA52}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57A86273-0E84-8246-B3ED-A023C6721217}">
   <dimension ref="A1:L31"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.125" style="35" customWidth="1"/>
-    <col min="3" max="3" width="4.625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="5.875" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.1640625" style="35" customWidth="1"/>
+    <col min="3" max="3" width="4.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="5.83203125" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="7.5" style="40" customWidth="1"/>
     <col min="7" max="7" width="11" style="1"/>
-    <col min="8" max="8" width="6.125" style="35" customWidth="1"/>
-    <col min="9" max="9" width="4.625" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="5.625" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="5.875" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="6.1640625" style="35" customWidth="1"/>
+    <col min="9" max="9" width="4.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="5.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="5.83203125" style="1" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="7.5" style="32" customWidth="1"/>
     <col min="13" max="16384" width="11" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" s="14"/>
       <c r="B2" s="44"/>
-      <c r="C2" s="41"/>
-      <c r="D2" s="41"/>
-      <c r="E2" s="41"/>
+      <c r="C2" s="42"/>
+      <c r="D2" s="42"/>
+      <c r="E2" s="42"/>
       <c r="F2" s="45"/>
       <c r="H2" s="44"/>
-      <c r="I2" s="41"/>
-      <c r="J2" s="41"/>
-      <c r="K2" s="41"/>
+      <c r="I2" s="42"/>
+      <c r="J2" s="42"/>
+      <c r="K2" s="42"/>
       <c r="L2" s="45"/>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3" s="15"/>
       <c r="B3" s="44" t="s">
         <v>142</v>
       </c>
-      <c r="C3" s="41"/>
-      <c r="D3" s="41"/>
-      <c r="E3" s="41"/>
+      <c r="C3" s="42"/>
+      <c r="D3" s="42"/>
+      <c r="E3" s="42"/>
       <c r="F3" s="45"/>
       <c r="H3" s="44" t="s">
         <v>141</v>
       </c>
-      <c r="I3" s="41"/>
-      <c r="J3" s="41"/>
-      <c r="K3" s="41"/>
+      <c r="I3" s="42"/>
+      <c r="J3" s="42"/>
+      <c r="K3" s="42"/>
       <c r="L3" s="45"/>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4" s="16"/>
       <c r="B4" s="31" t="s">
         <v>89</v>
@@ -8422,7 +8606,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" s="17" t="s">
         <v>84</v>
       </c>
@@ -8432,7 +8616,7 @@
       <c r="J5" s="16"/>
       <c r="K5" s="16"/>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A6" s="16" t="s">
         <v>94</v>
       </c>
@@ -8456,7 +8640,7 @@
       <c r="J6" s="18"/>
       <c r="K6" s="16"/>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A7" s="16" t="s">
         <v>95</v>
       </c>
@@ -8480,7 +8664,7 @@
       <c r="J7" s="18"/>
       <c r="K7" s="16"/>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A8" s="17" t="s">
         <v>85</v>
       </c>
@@ -8493,7 +8677,7 @@
       <c r="J8" s="16"/>
       <c r="K8" s="16"/>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A9" s="16" t="s">
         <v>96</v>
       </c>
@@ -8512,7 +8696,7 @@
       <c r="J9" s="18"/>
       <c r="K9" s="16"/>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A10" s="16" t="s">
         <v>97</v>
       </c>
@@ -8531,7 +8715,7 @@
       <c r="J10" s="18"/>
       <c r="K10" s="16"/>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A11" s="16" t="s">
         <v>98</v>
       </c>
@@ -8550,7 +8734,7 @@
       <c r="J11" s="18"/>
       <c r="K11" s="16"/>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A12" s="16" t="s">
         <v>146</v>
       </c>
@@ -8569,7 +8753,7 @@
       <c r="J12" s="18"/>
       <c r="K12" s="16"/>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A13" s="16" t="s">
         <v>147</v>
       </c>
@@ -8588,7 +8772,7 @@
       <c r="J13" s="18"/>
       <c r="K13" s="16"/>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A14" s="17" t="s">
         <v>86</v>
       </c>
@@ -8601,7 +8785,7 @@
       <c r="J14" s="16"/>
       <c r="K14" s="16"/>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A15" s="16" t="s">
         <v>100</v>
       </c>
@@ -8620,7 +8804,7 @@
       <c r="J15" s="18"/>
       <c r="K15" s="16"/>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A16" s="16" t="s">
         <v>101</v>
       </c>
@@ -8639,7 +8823,7 @@
       <c r="J16" s="18"/>
       <c r="K16" s="16"/>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A17" s="16" t="s">
         <v>102</v>
       </c>
@@ -8658,7 +8842,7 @@
       <c r="J17" s="18"/>
       <c r="K17" s="16"/>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A18" s="16" t="s">
         <v>105</v>
       </c>
@@ -8677,7 +8861,7 @@
       <c r="J18" s="18"/>
       <c r="K18" s="16"/>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A19" s="16" t="s">
         <v>106</v>
       </c>
@@ -8696,7 +8880,7 @@
       <c r="J19" s="18"/>
       <c r="K19" s="16"/>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A20" s="16" t="s">
         <v>103</v>
       </c>
@@ -8715,7 +8899,7 @@
       <c r="J20" s="18"/>
       <c r="K20" s="16"/>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A21" s="16" t="s">
         <v>104</v>
       </c>
@@ -8734,7 +8918,7 @@
       <c r="J21" s="18"/>
       <c r="K21" s="16"/>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A22" s="16" t="s">
         <v>108</v>
       </c>
@@ -8753,7 +8937,7 @@
       <c r="J22" s="18"/>
       <c r="K22" s="16"/>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A23" s="16" t="s">
         <v>107</v>
       </c>
@@ -8772,7 +8956,7 @@
       <c r="J23" s="18"/>
       <c r="K23" s="16"/>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A24" s="16" t="s">
         <v>109</v>
       </c>
@@ -8791,7 +8975,7 @@
       <c r="J24" s="18"/>
       <c r="K24" s="16"/>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A25" s="17" t="s">
         <v>82</v>
       </c>
@@ -8804,7 +8988,7 @@
       <c r="J25" s="16"/>
       <c r="K25" s="16"/>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A26" s="16" t="s">
         <v>83</v>
       </c>
@@ -8823,7 +9007,7 @@
       <c r="J26" s="18"/>
       <c r="K26" s="16"/>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A27" s="16" t="s">
         <v>88</v>
       </c>
@@ -8842,7 +9026,7 @@
       <c r="J27" s="18"/>
       <c r="K27" s="16"/>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A28" s="16" t="s">
         <v>92</v>
       </c>
@@ -8861,7 +9045,7 @@
       <c r="J28" s="18"/>
       <c r="K28" s="16"/>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A29" s="16" t="s">
         <v>110</v>
       </c>
@@ -8880,7 +9064,7 @@
       <c r="J29" s="18"/>
       <c r="K29" s="16"/>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A30" s="20" t="s">
         <v>115</v>
       </c>
@@ -8896,7 +9080,7 @@
       <c r="K30" s="14"/>
       <c r="L30" s="33"/>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A31" s="15" t="s">
         <v>116</v>
       </c>
@@ -8921,178 +9105,4 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{540507A6-720C-0B43-804E-087FEE710926}">
-  <dimension ref="A1:E25"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="19.875" customWidth="1"/>
-    <col min="2" max="2" width="18.875" customWidth="1"/>
-    <col min="3" max="3" width="19.125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="23" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="24"/>
-    </row>
-    <row r="3" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="24" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="24" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="24"/>
-    </row>
-    <row r="6" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="24"/>
-    </row>
-    <row r="7" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="8" spans="1:3" s="23" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="23" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="24" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="24" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B11" s="23" t="s">
-        <v>127</v>
-      </c>
-      <c r="C11" s="23" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>124</v>
-      </c>
-      <c r="B12">
-        <v>-3.4000000000000002E-2</v>
-      </c>
-      <c r="C12">
-        <v>-1.4E-2</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>125</v>
-      </c>
-      <c r="B13">
-        <v>-2.4E-2</v>
-      </c>
-      <c r="C13">
-        <v>-8.0000000000000002E-3</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>126</v>
-      </c>
-      <c r="B14">
-        <v>-2.3E-2</v>
-      </c>
-      <c r="C14">
-        <v>-7.0000000000000001E-3</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>131</v>
-      </c>
-      <c r="B15">
-        <v>-2.5999999999999999E-2</v>
-      </c>
-      <c r="C15">
-        <v>-8.0000000000000002E-3</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="23" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" s="24" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B19" s="23" t="s">
-        <v>127</v>
-      </c>
-      <c r="C19" s="23" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>124</v>
-      </c>
-      <c r="B20">
-        <v>-3.1E-2</v>
-      </c>
-      <c r="C20">
-        <v>-1.0999999999999999E-2</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>125</v>
-      </c>
-      <c r="B21">
-        <v>-0.03</v>
-      </c>
-      <c r="C21">
-        <v>-1.2999999999999999E-2</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>126</v>
-      </c>
-      <c r="B22">
-        <v>-0.113</v>
-      </c>
-      <c r="C22">
-        <v>9.7000000000000003E-2</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>131</v>
-      </c>
-      <c r="B23">
-        <v>-3.3000000000000002E-2</v>
-      </c>
-      <c r="C23">
-        <v>-1.4999999999999999E-2</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E25" s="23" t="s">
-        <v>130</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>